<commit_message>
Dimensional de fabricação vem de "Rastreabilidade - dimensional"
- Data DF Fab do Mapa de Spools passa a ser consolidada a partir da
  data do grupo "Rastreabilidade - dimensional" do Mapa de Juntas.
- Ignora a linha de numeração das colunas (1, 2, 3...) abaixo do
  cabeçalho do Mapa de Juntas.
- Atualiza o Mapa de Juntas v2 com a versão nova e regenera o Mapa de
  Spools atualizado e o relatório.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jhm2rrJCBVkJYZMmi4pDeT
</commit_message>
<xml_diff>
--- a/saida/Situacao_Geral_de_Spools_ATUALIZADO.xlsx
+++ b/saida/Situacao_Geral_de_Spools_ATUALIZADO.xlsx
@@ -4748,13 +4748,13 @@
       <c r="AG17" s="7"/>
       <c r="AH17" s="34"/>
       <c r="AI17" s="34">
-        <v>47363</v>
+        <v>46267</v>
       </c>
       <c r="AJ17" s="34">
-        <v>47363</v>
+        <v>46267</v>
       </c>
       <c r="AK17" s="34">
-        <v>47363</v>
+        <v>46267</v>
       </c>
       <c r="AL17" s="34">
         <v>47363</v>
@@ -5006,13 +5006,13 @@
       <c r="AG19" s="7"/>
       <c r="AH19" s="34"/>
       <c r="AI19" s="34">
-        <v>47363</v>
+        <v>46267</v>
       </c>
       <c r="AJ19" s="34">
-        <v>47363</v>
+        <v>46267</v>
       </c>
       <c r="AK19" s="34">
-        <v>47363</v>
+        <v>46267</v>
       </c>
       <c r="AL19" s="34">
         <v>47363</v>
@@ -5253,14 +5253,24 @@
       <c r="AF21" s="34"/>
       <c r="AG21" s="7"/>
       <c r="AH21" s="34"/>
-      <c r="AI21" s="34"/>
-      <c r="AJ21" s="34"/>
-      <c r="AK21" s="34"/>
-      <c r="AL21" s="34"/>
+      <c r="AI21" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AJ21" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AK21" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AL21" s="34">
+        <v>46288</v>
+      </c>
       <c r="AM21" s="34"/>
       <c r="AN21" s="7"/>
       <c r="AO21" s="7"/>
-      <c r="AP21" s="34"/>
+      <c r="AP21" s="34">
+        <v>46288</v>
+      </c>
       <c r="AQ21" s="7"/>
       <c r="AR21" s="34"/>
       <c r="AS21" s="34"/>
@@ -5387,7 +5397,9 @@
       <c r="AM22" s="34"/>
       <c r="AN22" s="7"/>
       <c r="AO22" s="7"/>
-      <c r="AP22" s="34"/>
+      <c r="AP22" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ22" s="7"/>
       <c r="AR22" s="34"/>
       <c r="AS22" s="34"/>
@@ -5514,7 +5526,9 @@
       <c r="AM23" s="34"/>
       <c r="AN23" s="7"/>
       <c r="AO23" s="7"/>
-      <c r="AP23" s="34"/>
+      <c r="AP23" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ23" s="7"/>
       <c r="AR23" s="34"/>
       <c r="AS23" s="34"/>
@@ -6385,7 +6399,9 @@
       <c r="AM30" s="34"/>
       <c r="AN30" s="7"/>
       <c r="AO30" s="7"/>
-      <c r="AP30" s="34"/>
+      <c r="AP30" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ30" s="7"/>
       <c r="AR30" s="34"/>
       <c r="AS30" s="34"/>
@@ -6631,7 +6647,9 @@
       <c r="AM32" s="34"/>
       <c r="AN32" s="7"/>
       <c r="AO32" s="7"/>
-      <c r="AP32" s="34"/>
+      <c r="AP32" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ32" s="7"/>
       <c r="AR32" s="34"/>
       <c r="AS32" s="34"/>
@@ -6758,7 +6776,9 @@
       <c r="AM33" s="34"/>
       <c r="AN33" s="7"/>
       <c r="AO33" s="7"/>
-      <c r="AP33" s="34"/>
+      <c r="AP33" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ33" s="7"/>
       <c r="AR33" s="34"/>
       <c r="AS33" s="34"/>
@@ -6885,7 +6905,9 @@
       <c r="AM34" s="34"/>
       <c r="AN34" s="7"/>
       <c r="AO34" s="7"/>
-      <c r="AP34" s="34"/>
+      <c r="AP34" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ34" s="7"/>
       <c r="AR34" s="34"/>
       <c r="AS34" s="34"/>
@@ -7012,7 +7034,9 @@
       <c r="AM35" s="34"/>
       <c r="AN35" s="7"/>
       <c r="AO35" s="7"/>
-      <c r="AP35" s="34"/>
+      <c r="AP35" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ35" s="7"/>
       <c r="AR35" s="34"/>
       <c r="AS35" s="34"/>
@@ -7139,7 +7163,9 @@
       <c r="AM36" s="34"/>
       <c r="AN36" s="7"/>
       <c r="AO36" s="7"/>
-      <c r="AP36" s="34"/>
+      <c r="AP36" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ36" s="7"/>
       <c r="AR36" s="34"/>
       <c r="AS36" s="34"/>
@@ -10213,7 +10239,9 @@
       <c r="AM60" s="34"/>
       <c r="AN60" s="7"/>
       <c r="AO60" s="7"/>
-      <c r="AP60" s="34"/>
+      <c r="AP60" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ60" s="7"/>
       <c r="AR60" s="34"/>
       <c r="AS60" s="34"/>
@@ -10340,7 +10368,9 @@
       <c r="AM61" s="34"/>
       <c r="AN61" s="7"/>
       <c r="AO61" s="7"/>
-      <c r="AP61" s="34"/>
+      <c r="AP61" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ61" s="7"/>
       <c r="AR61" s="34"/>
       <c r="AS61" s="34"/>
@@ -10467,7 +10497,9 @@
       <c r="AM62" s="34"/>
       <c r="AN62" s="7"/>
       <c r="AO62" s="7"/>
-      <c r="AP62" s="34"/>
+      <c r="AP62" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ62" s="7"/>
       <c r="AR62" s="34"/>
       <c r="AS62" s="34"/>
@@ -10594,7 +10626,9 @@
       <c r="AM63" s="34"/>
       <c r="AN63" s="7"/>
       <c r="AO63" s="7"/>
-      <c r="AP63" s="34"/>
+      <c r="AP63" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ63" s="7"/>
       <c r="AR63" s="34"/>
       <c r="AS63" s="34"/>
@@ -10721,7 +10755,9 @@
       <c r="AM64" s="34"/>
       <c r="AN64" s="7"/>
       <c r="AO64" s="7"/>
-      <c r="AP64" s="34"/>
+      <c r="AP64" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ64" s="7"/>
       <c r="AR64" s="34"/>
       <c r="AS64" s="34"/>
@@ -10848,7 +10884,9 @@
       <c r="AM65" s="34"/>
       <c r="AN65" s="7"/>
       <c r="AO65" s="7"/>
-      <c r="AP65" s="34"/>
+      <c r="AP65" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ65" s="7"/>
       <c r="AR65" s="34"/>
       <c r="AS65" s="34"/>
@@ -10975,7 +11013,9 @@
       <c r="AM66" s="34"/>
       <c r="AN66" s="7"/>
       <c r="AO66" s="7"/>
-      <c r="AP66" s="34"/>
+      <c r="AP66" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ66" s="7"/>
       <c r="AR66" s="34"/>
       <c r="AS66" s="34"/>
@@ -11102,7 +11142,9 @@
       <c r="AM67" s="34"/>
       <c r="AN67" s="7"/>
       <c r="AO67" s="7"/>
-      <c r="AP67" s="34"/>
+      <c r="AP67" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ67" s="7"/>
       <c r="AR67" s="34"/>
       <c r="AS67" s="34"/>
@@ -11229,7 +11271,9 @@
       <c r="AM68" s="34"/>
       <c r="AN68" s="7"/>
       <c r="AO68" s="7"/>
-      <c r="AP68" s="34"/>
+      <c r="AP68" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ68" s="7"/>
       <c r="AR68" s="34"/>
       <c r="AS68" s="34"/>
@@ -11356,7 +11400,9 @@
       <c r="AM69" s="34"/>
       <c r="AN69" s="7"/>
       <c r="AO69" s="7"/>
-      <c r="AP69" s="34"/>
+      <c r="AP69" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ69" s="7"/>
       <c r="AR69" s="34"/>
       <c r="AS69" s="34"/>
@@ -11610,7 +11656,9 @@
       <c r="AM71" s="34"/>
       <c r="AN71" s="7"/>
       <c r="AO71" s="7"/>
-      <c r="AP71" s="34"/>
+      <c r="AP71" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ71" s="7"/>
       <c r="AR71" s="34"/>
       <c r="AS71" s="34"/>
@@ -13602,9 +13650,7 @@
       <c r="AM87" s="34"/>
       <c r="AN87" s="7"/>
       <c r="AO87" s="7"/>
-      <c r="AP87" s="34">
-        <v>46263</v>
-      </c>
+      <c r="AP87" s="34"/>
       <c r="AQ87" s="7"/>
       <c r="AR87" s="34"/>
       <c r="AS87" s="34"/>
@@ -13731,9 +13777,7 @@
       <c r="AM88" s="34"/>
       <c r="AN88" s="7"/>
       <c r="AO88" s="7"/>
-      <c r="AP88" s="34">
-        <v>46263</v>
-      </c>
+      <c r="AP88" s="34"/>
       <c r="AQ88" s="7"/>
       <c r="AR88" s="34"/>
       <c r="AS88" s="34"/>
@@ -13858,7 +13902,9 @@
       <c r="AM89" s="34"/>
       <c r="AN89" s="7"/>
       <c r="AO89" s="7"/>
-      <c r="AP89" s="34"/>
+      <c r="AP89" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ89" s="7"/>
       <c r="AR89" s="34"/>
       <c r="AS89" s="34"/>
@@ -13968,10 +14014,18 @@
       <c r="AF90" s="34"/>
       <c r="AG90" s="7"/>
       <c r="AH90" s="34"/>
-      <c r="AI90" s="34"/>
-      <c r="AJ90" s="34"/>
-      <c r="AK90" s="34"/>
-      <c r="AL90" s="34"/>
+      <c r="AI90" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AJ90" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AK90" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AL90" s="34">
+        <v>46288</v>
+      </c>
       <c r="AM90" s="34"/>
       <c r="AN90" s="7"/>
       <c r="AO90" s="7"/>
@@ -14085,10 +14139,18 @@
       <c r="AF91" s="34"/>
       <c r="AG91" s="7"/>
       <c r="AH91" s="34"/>
-      <c r="AI91" s="34"/>
-      <c r="AJ91" s="34"/>
-      <c r="AK91" s="34"/>
-      <c r="AL91" s="34"/>
+      <c r="AI91" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AJ91" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AK91" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AL91" s="34">
+        <v>46288</v>
+      </c>
       <c r="AM91" s="34"/>
       <c r="AN91" s="7"/>
       <c r="AO91" s="7"/>
@@ -14202,10 +14264,18 @@
       <c r="AF92" s="34"/>
       <c r="AG92" s="7"/>
       <c r="AH92" s="34"/>
-      <c r="AI92" s="34"/>
-      <c r="AJ92" s="34"/>
-      <c r="AK92" s="34"/>
-      <c r="AL92" s="34"/>
+      <c r="AI92" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AJ92" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AK92" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AL92" s="34">
+        <v>46288</v>
+      </c>
       <c r="AM92" s="34"/>
       <c r="AN92" s="7"/>
       <c r="AO92" s="7"/>
@@ -14319,10 +14389,18 @@
       <c r="AF93" s="34"/>
       <c r="AG93" s="7"/>
       <c r="AH93" s="34"/>
-      <c r="AI93" s="34"/>
-      <c r="AJ93" s="34"/>
-      <c r="AK93" s="34"/>
-      <c r="AL93" s="34"/>
+      <c r="AI93" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AJ93" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AK93" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AL93" s="34">
+        <v>46288</v>
+      </c>
       <c r="AM93" s="34"/>
       <c r="AN93" s="7"/>
       <c r="AO93" s="7"/>
@@ -14436,10 +14514,18 @@
       <c r="AF94" s="34"/>
       <c r="AG94" s="7"/>
       <c r="AH94" s="34"/>
-      <c r="AI94" s="34"/>
-      <c r="AJ94" s="34"/>
-      <c r="AK94" s="34"/>
-      <c r="AL94" s="34"/>
+      <c r="AI94" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AJ94" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AK94" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AL94" s="34">
+        <v>46288</v>
+      </c>
       <c r="AM94" s="34"/>
       <c r="AN94" s="7"/>
       <c r="AO94" s="7"/>
@@ -14553,10 +14639,18 @@
       <c r="AF95" s="34"/>
       <c r="AG95" s="7"/>
       <c r="AH95" s="34"/>
-      <c r="AI95" s="34"/>
-      <c r="AJ95" s="34"/>
-      <c r="AK95" s="34"/>
-      <c r="AL95" s="34"/>
+      <c r="AI95" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AJ95" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AK95" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AL95" s="34">
+        <v>46288</v>
+      </c>
       <c r="AM95" s="34"/>
       <c r="AN95" s="7"/>
       <c r="AO95" s="7"/>
@@ -14670,10 +14764,18 @@
       <c r="AF96" s="34"/>
       <c r="AG96" s="7"/>
       <c r="AH96" s="34"/>
-      <c r="AI96" s="34"/>
-      <c r="AJ96" s="34"/>
-      <c r="AK96" s="34"/>
-      <c r="AL96" s="34"/>
+      <c r="AI96" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AJ96" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AK96" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AL96" s="34">
+        <v>46288</v>
+      </c>
       <c r="AM96" s="34"/>
       <c r="AN96" s="7"/>
       <c r="AO96" s="7"/>
@@ -14787,10 +14889,18 @@
       <c r="AF97" s="34"/>
       <c r="AG97" s="7"/>
       <c r="AH97" s="34"/>
-      <c r="AI97" s="34"/>
-      <c r="AJ97" s="34"/>
-      <c r="AK97" s="34"/>
-      <c r="AL97" s="34"/>
+      <c r="AI97" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AJ97" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AK97" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AL97" s="34">
+        <v>46288</v>
+      </c>
       <c r="AM97" s="34"/>
       <c r="AN97" s="7"/>
       <c r="AO97" s="7"/>
@@ -14904,10 +15014,18 @@
       <c r="AF98" s="34"/>
       <c r="AG98" s="7"/>
       <c r="AH98" s="34"/>
-      <c r="AI98" s="34"/>
-      <c r="AJ98" s="34"/>
-      <c r="AK98" s="34"/>
-      <c r="AL98" s="34"/>
+      <c r="AI98" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AJ98" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AK98" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AL98" s="34">
+        <v>46288</v>
+      </c>
       <c r="AM98" s="34"/>
       <c r="AN98" s="7"/>
       <c r="AO98" s="7"/>
@@ -15021,10 +15139,18 @@
       <c r="AF99" s="34"/>
       <c r="AG99" s="7"/>
       <c r="AH99" s="34"/>
-      <c r="AI99" s="34"/>
-      <c r="AJ99" s="34"/>
-      <c r="AK99" s="34"/>
-      <c r="AL99" s="34"/>
+      <c r="AI99" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AJ99" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AK99" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AL99" s="34">
+        <v>46288</v>
+      </c>
       <c r="AM99" s="34"/>
       <c r="AN99" s="7"/>
       <c r="AO99" s="7"/>
@@ -15138,10 +15264,18 @@
       <c r="AF100" s="34"/>
       <c r="AG100" s="7"/>
       <c r="AH100" s="34"/>
-      <c r="AI100" s="34"/>
-      <c r="AJ100" s="34"/>
-      <c r="AK100" s="34"/>
-      <c r="AL100" s="34"/>
+      <c r="AI100" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AJ100" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AK100" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AL100" s="34">
+        <v>46286</v>
+      </c>
       <c r="AM100" s="34"/>
       <c r="AN100" s="7"/>
       <c r="AO100" s="7"/>
@@ -15255,10 +15389,18 @@
       <c r="AF101" s="34"/>
       <c r="AG101" s="7"/>
       <c r="AH101" s="34"/>
-      <c r="AI101" s="34"/>
-      <c r="AJ101" s="34"/>
-      <c r="AK101" s="34"/>
-      <c r="AL101" s="34"/>
+      <c r="AI101" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AJ101" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AK101" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AL101" s="34">
+        <v>46286</v>
+      </c>
       <c r="AM101" s="34"/>
       <c r="AN101" s="7"/>
       <c r="AO101" s="7"/>
@@ -15372,10 +15514,18 @@
       <c r="AF102" s="34"/>
       <c r="AG102" s="7"/>
       <c r="AH102" s="34"/>
-      <c r="AI102" s="34"/>
-      <c r="AJ102" s="34"/>
-      <c r="AK102" s="34"/>
-      <c r="AL102" s="34"/>
+      <c r="AI102" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AJ102" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AK102" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AL102" s="34">
+        <v>46286</v>
+      </c>
       <c r="AM102" s="34"/>
       <c r="AN102" s="7"/>
       <c r="AO102" s="7"/>
@@ -15489,10 +15639,18 @@
       <c r="AF103" s="34"/>
       <c r="AG103" s="7"/>
       <c r="AH103" s="34"/>
-      <c r="AI103" s="34"/>
-      <c r="AJ103" s="34"/>
-      <c r="AK103" s="34"/>
-      <c r="AL103" s="34"/>
+      <c r="AI103" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AJ103" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AK103" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AL103" s="34">
+        <v>46286</v>
+      </c>
       <c r="AM103" s="34"/>
       <c r="AN103" s="7"/>
       <c r="AO103" s="7"/>
@@ -15723,10 +15881,18 @@
       <c r="AF105" s="34"/>
       <c r="AG105" s="7"/>
       <c r="AH105" s="34"/>
-      <c r="AI105" s="34"/>
-      <c r="AJ105" s="34"/>
-      <c r="AK105" s="34"/>
-      <c r="AL105" s="34"/>
+      <c r="AI105" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AJ105" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AK105" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AL105" s="34">
+        <v>46286</v>
+      </c>
       <c r="AM105" s="34"/>
       <c r="AN105" s="7"/>
       <c r="AO105" s="7"/>
@@ -15840,10 +16006,18 @@
       <c r="AF106" s="34"/>
       <c r="AG106" s="7"/>
       <c r="AH106" s="34"/>
-      <c r="AI106" s="34"/>
-      <c r="AJ106" s="34"/>
-      <c r="AK106" s="34"/>
-      <c r="AL106" s="34"/>
+      <c r="AI106" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AJ106" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AK106" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AL106" s="34">
+        <v>46286</v>
+      </c>
       <c r="AM106" s="34"/>
       <c r="AN106" s="7"/>
       <c r="AO106" s="7"/>
@@ -15957,10 +16131,18 @@
       <c r="AF107" s="34"/>
       <c r="AG107" s="7"/>
       <c r="AH107" s="34"/>
-      <c r="AI107" s="34"/>
-      <c r="AJ107" s="34"/>
-      <c r="AK107" s="34"/>
-      <c r="AL107" s="34"/>
+      <c r="AI107" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AJ107" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AK107" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AL107" s="34">
+        <v>46286</v>
+      </c>
       <c r="AM107" s="34"/>
       <c r="AN107" s="7"/>
       <c r="AO107" s="7"/>
@@ -16191,10 +16373,18 @@
       <c r="AF109" s="34"/>
       <c r="AG109" s="7"/>
       <c r="AH109" s="34"/>
-      <c r="AI109" s="34"/>
-      <c r="AJ109" s="34"/>
-      <c r="AK109" s="34"/>
-      <c r="AL109" s="34"/>
+      <c r="AI109" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AJ109" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AK109" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AL109" s="34">
+        <v>46285</v>
+      </c>
       <c r="AM109" s="34"/>
       <c r="AN109" s="7"/>
       <c r="AO109" s="7"/>
@@ -16308,10 +16498,18 @@
       <c r="AF110" s="34"/>
       <c r="AG110" s="7"/>
       <c r="AH110" s="34"/>
-      <c r="AI110" s="34"/>
-      <c r="AJ110" s="34"/>
-      <c r="AK110" s="34"/>
-      <c r="AL110" s="34"/>
+      <c r="AI110" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AJ110" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AK110" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AL110" s="34">
+        <v>46285</v>
+      </c>
       <c r="AM110" s="34"/>
       <c r="AN110" s="7"/>
       <c r="AO110" s="7"/>
@@ -16425,10 +16623,18 @@
       <c r="AF111" s="34"/>
       <c r="AG111" s="7"/>
       <c r="AH111" s="34"/>
-      <c r="AI111" s="34"/>
-      <c r="AJ111" s="34"/>
-      <c r="AK111" s="34"/>
-      <c r="AL111" s="34"/>
+      <c r="AI111" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AJ111" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AK111" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AL111" s="34">
+        <v>46285</v>
+      </c>
       <c r="AM111" s="34"/>
       <c r="AN111" s="7"/>
       <c r="AO111" s="7"/>
@@ -16659,10 +16865,18 @@
       <c r="AF113" s="34"/>
       <c r="AG113" s="7"/>
       <c r="AH113" s="34"/>
-      <c r="AI113" s="34"/>
-      <c r="AJ113" s="34"/>
-      <c r="AK113" s="34"/>
-      <c r="AL113" s="34"/>
+      <c r="AI113" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AJ113" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AK113" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AL113" s="34">
+        <v>46285</v>
+      </c>
       <c r="AM113" s="34"/>
       <c r="AN113" s="7"/>
       <c r="AO113" s="7"/>
@@ -16893,10 +17107,18 @@
       <c r="AF115" s="34"/>
       <c r="AG115" s="7"/>
       <c r="AH115" s="34"/>
-      <c r="AI115" s="34"/>
-      <c r="AJ115" s="34"/>
-      <c r="AK115" s="34"/>
-      <c r="AL115" s="34"/>
+      <c r="AI115" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AJ115" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AK115" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AL115" s="34">
+        <v>46286</v>
+      </c>
       <c r="AM115" s="34"/>
       <c r="AN115" s="7"/>
       <c r="AO115" s="7"/>
@@ -17244,10 +17466,18 @@
       <c r="AF118" s="34"/>
       <c r="AG118" s="7"/>
       <c r="AH118" s="34"/>
-      <c r="AI118" s="34"/>
-      <c r="AJ118" s="34"/>
-      <c r="AK118" s="34"/>
-      <c r="AL118" s="34"/>
+      <c r="AI118" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AJ118" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AK118" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AL118" s="34">
+        <v>46287</v>
+      </c>
       <c r="AM118" s="34"/>
       <c r="AN118" s="7"/>
       <c r="AO118" s="7"/>
@@ -17486,14 +17716,24 @@
       <c r="AF120" s="34"/>
       <c r="AG120" s="7"/>
       <c r="AH120" s="34"/>
-      <c r="AI120" s="34"/>
-      <c r="AJ120" s="34"/>
-      <c r="AK120" s="34"/>
-      <c r="AL120" s="34"/>
+      <c r="AI120" s="34">
+        <v>46254</v>
+      </c>
+      <c r="AJ120" s="34">
+        <v>46254</v>
+      </c>
+      <c r="AK120" s="34">
+        <v>46254</v>
+      </c>
+      <c r="AL120" s="34">
+        <v>46254</v>
+      </c>
       <c r="AM120" s="34"/>
       <c r="AN120" s="7"/>
       <c r="AO120" s="7"/>
-      <c r="AP120" s="34"/>
+      <c r="AP120" s="34">
+        <v>46255</v>
+      </c>
       <c r="AQ120" s="7"/>
       <c r="AR120" s="34"/>
       <c r="AS120" s="34"/>
@@ -17837,14 +18077,24 @@
       <c r="AF123" s="34"/>
       <c r="AG123" s="7"/>
       <c r="AH123" s="34"/>
-      <c r="AI123" s="34"/>
-      <c r="AJ123" s="34"/>
-      <c r="AK123" s="34"/>
-      <c r="AL123" s="34"/>
+      <c r="AI123" s="34">
+        <v>46258</v>
+      </c>
+      <c r="AJ123" s="34">
+        <v>46258</v>
+      </c>
+      <c r="AK123" s="34">
+        <v>46258</v>
+      </c>
+      <c r="AL123" s="34">
+        <v>46258</v>
+      </c>
       <c r="AM123" s="34"/>
       <c r="AN123" s="7"/>
       <c r="AO123" s="7"/>
-      <c r="AP123" s="34"/>
+      <c r="AP123" s="34">
+        <v>46258</v>
+      </c>
       <c r="AQ123" s="7"/>
       <c r="AR123" s="34"/>
       <c r="AS123" s="34"/>
@@ -17954,14 +18204,24 @@
       <c r="AF124" s="34"/>
       <c r="AG124" s="7"/>
       <c r="AH124" s="34"/>
-      <c r="AI124" s="34"/>
-      <c r="AJ124" s="34"/>
-      <c r="AK124" s="34"/>
-      <c r="AL124" s="34"/>
+      <c r="AI124" s="34">
+        <v>46258</v>
+      </c>
+      <c r="AJ124" s="34">
+        <v>46258</v>
+      </c>
+      <c r="AK124" s="34">
+        <v>46258</v>
+      </c>
+      <c r="AL124" s="34">
+        <v>46258</v>
+      </c>
       <c r="AM124" s="34"/>
       <c r="AN124" s="7"/>
       <c r="AO124" s="7"/>
-      <c r="AP124" s="34"/>
+      <c r="AP124" s="34">
+        <v>46258</v>
+      </c>
       <c r="AQ124" s="7"/>
       <c r="AR124" s="34"/>
       <c r="AS124" s="34"/>
@@ -18071,10 +18331,18 @@
       <c r="AF125" s="34"/>
       <c r="AG125" s="7"/>
       <c r="AH125" s="34"/>
-      <c r="AI125" s="34"/>
-      <c r="AJ125" s="34"/>
-      <c r="AK125" s="34"/>
-      <c r="AL125" s="34"/>
+      <c r="AI125" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AJ125" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AK125" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AL125" s="34">
+        <v>46287</v>
+      </c>
       <c r="AM125" s="34"/>
       <c r="AN125" s="7"/>
       <c r="AO125" s="7"/>
@@ -18188,10 +18456,18 @@
       <c r="AF126" s="34"/>
       <c r="AG126" s="7"/>
       <c r="AH126" s="34"/>
-      <c r="AI126" s="34"/>
-      <c r="AJ126" s="34"/>
-      <c r="AK126" s="34"/>
-      <c r="AL126" s="34"/>
+      <c r="AI126" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AJ126" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AK126" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AL126" s="34">
+        <v>46287</v>
+      </c>
       <c r="AM126" s="34"/>
       <c r="AN126" s="7"/>
       <c r="AO126" s="7"/>
@@ -18305,10 +18581,18 @@
       <c r="AF127" s="34"/>
       <c r="AG127" s="7"/>
       <c r="AH127" s="34"/>
-      <c r="AI127" s="34"/>
-      <c r="AJ127" s="34"/>
-      <c r="AK127" s="34"/>
-      <c r="AL127" s="34"/>
+      <c r="AI127" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AJ127" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AK127" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AL127" s="34">
+        <v>46287</v>
+      </c>
       <c r="AM127" s="34"/>
       <c r="AN127" s="7"/>
       <c r="AO127" s="7"/>
@@ -18422,14 +18706,24 @@
       <c r="AF128" s="34"/>
       <c r="AG128" s="7"/>
       <c r="AH128" s="34"/>
-      <c r="AI128" s="34"/>
-      <c r="AJ128" s="34"/>
-      <c r="AK128" s="34"/>
-      <c r="AL128" s="34"/>
+      <c r="AI128" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AJ128" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AK128" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AL128" s="34">
+        <v>46287</v>
+      </c>
       <c r="AM128" s="34"/>
       <c r="AN128" s="7"/>
       <c r="AO128" s="7"/>
-      <c r="AP128" s="34"/>
+      <c r="AP128" s="34">
+        <v>46288</v>
+      </c>
       <c r="AQ128" s="7"/>
       <c r="AR128" s="34"/>
       <c r="AS128" s="34"/>
@@ -18539,14 +18833,24 @@
       <c r="AF129" s="34"/>
       <c r="AG129" s="7"/>
       <c r="AH129" s="34"/>
-      <c r="AI129" s="34"/>
-      <c r="AJ129" s="34"/>
-      <c r="AK129" s="34"/>
-      <c r="AL129" s="34"/>
+      <c r="AI129" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AJ129" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AK129" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AL129" s="34">
+        <v>46287</v>
+      </c>
       <c r="AM129" s="34"/>
       <c r="AN129" s="7"/>
       <c r="AO129" s="7"/>
-      <c r="AP129" s="34"/>
+      <c r="AP129" s="34">
+        <v>46288</v>
+      </c>
       <c r="AQ129" s="7"/>
       <c r="AR129" s="34"/>
       <c r="AS129" s="34"/>
@@ -18656,14 +18960,24 @@
       <c r="AF130" s="34"/>
       <c r="AG130" s="7"/>
       <c r="AH130" s="34"/>
-      <c r="AI130" s="34"/>
-      <c r="AJ130" s="34"/>
-      <c r="AK130" s="34"/>
-      <c r="AL130" s="34"/>
+      <c r="AI130" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AJ130" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AK130" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AL130" s="34">
+        <v>46287</v>
+      </c>
       <c r="AM130" s="34"/>
       <c r="AN130" s="7"/>
       <c r="AO130" s="7"/>
-      <c r="AP130" s="34"/>
+      <c r="AP130" s="34">
+        <v>46288</v>
+      </c>
       <c r="AQ130" s="7"/>
       <c r="AR130" s="34"/>
       <c r="AS130" s="34"/>
@@ -18773,14 +19087,24 @@
       <c r="AF131" s="34"/>
       <c r="AG131" s="7"/>
       <c r="AH131" s="34"/>
-      <c r="AI131" s="34"/>
-      <c r="AJ131" s="34"/>
-      <c r="AK131" s="34"/>
-      <c r="AL131" s="34"/>
+      <c r="AI131" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AJ131" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AK131" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AL131" s="34">
+        <v>46287</v>
+      </c>
       <c r="AM131" s="34"/>
       <c r="AN131" s="7"/>
       <c r="AO131" s="7"/>
-      <c r="AP131" s="34"/>
+      <c r="AP131" s="34">
+        <v>46288</v>
+      </c>
       <c r="AQ131" s="7"/>
       <c r="AR131" s="34"/>
       <c r="AS131" s="34"/>
@@ -18890,14 +19214,24 @@
       <c r="AF132" s="34"/>
       <c r="AG132" s="7"/>
       <c r="AH132" s="34"/>
-      <c r="AI132" s="34"/>
-      <c r="AJ132" s="34"/>
-      <c r="AK132" s="34"/>
-      <c r="AL132" s="34"/>
+      <c r="AI132" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AJ132" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AK132" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AL132" s="34">
+        <v>46287</v>
+      </c>
       <c r="AM132" s="34"/>
       <c r="AN132" s="7"/>
       <c r="AO132" s="7"/>
-      <c r="AP132" s="34"/>
+      <c r="AP132" s="34">
+        <v>46288</v>
+      </c>
       <c r="AQ132" s="7"/>
       <c r="AR132" s="34"/>
       <c r="AS132" s="34"/>
@@ -19007,14 +19341,24 @@
       <c r="AF133" s="34"/>
       <c r="AG133" s="7"/>
       <c r="AH133" s="34"/>
-      <c r="AI133" s="34"/>
-      <c r="AJ133" s="34"/>
-      <c r="AK133" s="34"/>
-      <c r="AL133" s="34"/>
+      <c r="AI133" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AJ133" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AK133" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AL133" s="34">
+        <v>46287</v>
+      </c>
       <c r="AM133" s="34"/>
       <c r="AN133" s="7"/>
       <c r="AO133" s="7"/>
-      <c r="AP133" s="34"/>
+      <c r="AP133" s="34">
+        <v>46288</v>
+      </c>
       <c r="AQ133" s="7"/>
       <c r="AR133" s="34"/>
       <c r="AS133" s="34"/>
@@ -19139,7 +19483,9 @@
       <c r="AM134" s="34"/>
       <c r="AN134" s="7"/>
       <c r="AO134" s="7"/>
-      <c r="AP134" s="34"/>
+      <c r="AP134" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ134" s="7"/>
       <c r="AR134" s="34"/>
       <c r="AS134" s="34"/>
@@ -19249,14 +19595,24 @@
       <c r="AF135" s="34"/>
       <c r="AG135" s="7"/>
       <c r="AH135" s="34"/>
-      <c r="AI135" s="34"/>
-      <c r="AJ135" s="34"/>
-      <c r="AK135" s="34"/>
-      <c r="AL135" s="34"/>
+      <c r="AI135" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AJ135" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AK135" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AL135" s="34">
+        <v>46286</v>
+      </c>
       <c r="AM135" s="34"/>
       <c r="AN135" s="7"/>
       <c r="AO135" s="7"/>
-      <c r="AP135" s="34"/>
+      <c r="AP135" s="34">
+        <v>46287</v>
+      </c>
       <c r="AQ135" s="7"/>
       <c r="AR135" s="34"/>
       <c r="AS135" s="34"/>
@@ -19366,14 +19722,24 @@
       <c r="AF136" s="34"/>
       <c r="AG136" s="7"/>
       <c r="AH136" s="34"/>
-      <c r="AI136" s="34"/>
-      <c r="AJ136" s="34"/>
-      <c r="AK136" s="34"/>
-      <c r="AL136" s="34"/>
+      <c r="AI136" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AJ136" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AK136" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AL136" s="34">
+        <v>46286</v>
+      </c>
       <c r="AM136" s="34"/>
       <c r="AN136" s="7"/>
       <c r="AO136" s="7"/>
-      <c r="AP136" s="34"/>
+      <c r="AP136" s="34">
+        <v>46287</v>
+      </c>
       <c r="AQ136" s="7"/>
       <c r="AR136" s="34"/>
       <c r="AS136" s="34"/>
@@ -19483,14 +19849,24 @@
       <c r="AF137" s="34"/>
       <c r="AG137" s="7"/>
       <c r="AH137" s="34"/>
-      <c r="AI137" s="34"/>
-      <c r="AJ137" s="34"/>
-      <c r="AK137" s="34"/>
-      <c r="AL137" s="34"/>
+      <c r="AI137" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AJ137" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AK137" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AL137" s="34">
+        <v>46286</v>
+      </c>
       <c r="AM137" s="34"/>
       <c r="AN137" s="7"/>
       <c r="AO137" s="7"/>
-      <c r="AP137" s="34"/>
+      <c r="AP137" s="34">
+        <v>46287</v>
+      </c>
       <c r="AQ137" s="7"/>
       <c r="AR137" s="34"/>
       <c r="AS137" s="34"/>
@@ -19615,7 +19991,9 @@
       <c r="AM138" s="34"/>
       <c r="AN138" s="7"/>
       <c r="AO138" s="7"/>
-      <c r="AP138" s="34"/>
+      <c r="AP138" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ138" s="7"/>
       <c r="AR138" s="34"/>
       <c r="AS138" s="34"/>
@@ -19740,7 +20118,9 @@
       <c r="AM139" s="34"/>
       <c r="AN139" s="7"/>
       <c r="AO139" s="7"/>
-      <c r="AP139" s="34"/>
+      <c r="AP139" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ139" s="7"/>
       <c r="AR139" s="34"/>
       <c r="AS139" s="34"/>
@@ -19865,7 +20245,9 @@
       <c r="AM140" s="34"/>
       <c r="AN140" s="7"/>
       <c r="AO140" s="7"/>
-      <c r="AP140" s="34"/>
+      <c r="AP140" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ140" s="7"/>
       <c r="AR140" s="34"/>
       <c r="AS140" s="34"/>
@@ -19990,7 +20372,9 @@
       <c r="AM141" s="34"/>
       <c r="AN141" s="7"/>
       <c r="AO141" s="7"/>
-      <c r="AP141" s="34"/>
+      <c r="AP141" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ141" s="7"/>
       <c r="AR141" s="34"/>
       <c r="AS141" s="34"/>
@@ -20621,9 +21005,7 @@
       <c r="AM146" s="34"/>
       <c r="AN146" s="7"/>
       <c r="AO146" s="7"/>
-      <c r="AP146" s="34">
-        <v>46252</v>
-      </c>
+      <c r="AP146" s="34"/>
       <c r="AQ146" s="7"/>
       <c r="AR146" s="34"/>
       <c r="AS146" s="34"/>
@@ -20865,7 +21247,9 @@
       <c r="AM148" s="34"/>
       <c r="AN148" s="7"/>
       <c r="AO148" s="7"/>
-      <c r="AP148" s="34"/>
+      <c r="AP148" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ148" s="7"/>
       <c r="AR148" s="34"/>
       <c r="AS148" s="34"/>
@@ -20990,7 +21374,9 @@
       <c r="AM149" s="34"/>
       <c r="AN149" s="7"/>
       <c r="AO149" s="7"/>
-      <c r="AP149" s="34"/>
+      <c r="AP149" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ149" s="7"/>
       <c r="AR149" s="34"/>
       <c r="AS149" s="34"/>
@@ -21115,7 +21501,9 @@
       <c r="AM150" s="34"/>
       <c r="AN150" s="7"/>
       <c r="AO150" s="7"/>
-      <c r="AP150" s="34"/>
+      <c r="AP150" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ150" s="7"/>
       <c r="AR150" s="34"/>
       <c r="AS150" s="34"/>
@@ -21240,7 +21628,9 @@
       <c r="AM151" s="34"/>
       <c r="AN151" s="7"/>
       <c r="AO151" s="7"/>
-      <c r="AP151" s="34"/>
+      <c r="AP151" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ151" s="7"/>
       <c r="AR151" s="34"/>
       <c r="AS151" s="34"/>
@@ -21365,7 +21755,9 @@
       <c r="AM152" s="34"/>
       <c r="AN152" s="7"/>
       <c r="AO152" s="7"/>
-      <c r="AP152" s="34"/>
+      <c r="AP152" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ152" s="7"/>
       <c r="AR152" s="34"/>
       <c r="AS152" s="34"/>
@@ -21490,7 +21882,9 @@
       <c r="AM153" s="34"/>
       <c r="AN153" s="7"/>
       <c r="AO153" s="7"/>
-      <c r="AP153" s="34"/>
+      <c r="AP153" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ153" s="7"/>
       <c r="AR153" s="34"/>
       <c r="AS153" s="34"/>
@@ -21615,7 +22009,9 @@
       <c r="AM154" s="34"/>
       <c r="AN154" s="7"/>
       <c r="AO154" s="7"/>
-      <c r="AP154" s="34"/>
+      <c r="AP154" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ154" s="7"/>
       <c r="AR154" s="34"/>
       <c r="AS154" s="34"/>
@@ -21857,7 +22253,9 @@
       <c r="AM156" s="34"/>
       <c r="AN156" s="7"/>
       <c r="AO156" s="7"/>
-      <c r="AP156" s="34"/>
+      <c r="AP156" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ156" s="7"/>
       <c r="AR156" s="34"/>
       <c r="AS156" s="34"/>
@@ -21982,7 +22380,9 @@
       <c r="AM157" s="34"/>
       <c r="AN157" s="7"/>
       <c r="AO157" s="7"/>
-      <c r="AP157" s="34"/>
+      <c r="AP157" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ157" s="7"/>
       <c r="AR157" s="34"/>
       <c r="AS157" s="34"/>
@@ -22107,7 +22507,9 @@
       <c r="AM158" s="34"/>
       <c r="AN158" s="7"/>
       <c r="AO158" s="7"/>
-      <c r="AP158" s="34"/>
+      <c r="AP158" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ158" s="7"/>
       <c r="AR158" s="34"/>
       <c r="AS158" s="34"/>
@@ -22232,7 +22634,9 @@
       <c r="AM159" s="34"/>
       <c r="AN159" s="7"/>
       <c r="AO159" s="7"/>
-      <c r="AP159" s="34"/>
+      <c r="AP159" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ159" s="7"/>
       <c r="AR159" s="34"/>
       <c r="AS159" s="34"/>
@@ -22357,7 +22761,9 @@
       <c r="AM160" s="34"/>
       <c r="AN160" s="7"/>
       <c r="AO160" s="7"/>
-      <c r="AP160" s="34"/>
+      <c r="AP160" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ160" s="7"/>
       <c r="AR160" s="34"/>
       <c r="AS160" s="34"/>
@@ -22482,7 +22888,9 @@
       <c r="AM161" s="34"/>
       <c r="AN161" s="7"/>
       <c r="AO161" s="7"/>
-      <c r="AP161" s="34"/>
+      <c r="AP161" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ161" s="7"/>
       <c r="AR161" s="34"/>
       <c r="AS161" s="34"/>
@@ -22724,7 +23132,9 @@
       <c r="AM163" s="34"/>
       <c r="AN163" s="7"/>
       <c r="AO163" s="7"/>
-      <c r="AP163" s="34"/>
+      <c r="AP163" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ163" s="7"/>
       <c r="AR163" s="34"/>
       <c r="AS163" s="34"/>
@@ -22849,9 +23259,7 @@
       <c r="AM164" s="34"/>
       <c r="AN164" s="7"/>
       <c r="AO164" s="7"/>
-      <c r="AP164" s="34">
-        <v>46252</v>
-      </c>
+      <c r="AP164" s="34"/>
       <c r="AQ164" s="7"/>
       <c r="AR164" s="34"/>
       <c r="AS164" s="34"/>
@@ -22976,9 +23384,7 @@
       <c r="AM165" s="34"/>
       <c r="AN165" s="7"/>
       <c r="AO165" s="7"/>
-      <c r="AP165" s="34">
-        <v>46258</v>
-      </c>
+      <c r="AP165" s="34"/>
       <c r="AQ165" s="7"/>
       <c r="AR165" s="34"/>
       <c r="AS165" s="34"/>
@@ -23103,9 +23509,7 @@
       <c r="AM166" s="34"/>
       <c r="AN166" s="7"/>
       <c r="AO166" s="7"/>
-      <c r="AP166" s="34">
-        <v>46258</v>
-      </c>
+      <c r="AP166" s="34"/>
       <c r="AQ166" s="7"/>
       <c r="AR166" s="34"/>
       <c r="AS166" s="34"/>
@@ -23230,9 +23634,7 @@
       <c r="AM167" s="34"/>
       <c r="AN167" s="7"/>
       <c r="AO167" s="7"/>
-      <c r="AP167" s="34">
-        <v>46258</v>
-      </c>
+      <c r="AP167" s="34"/>
       <c r="AQ167" s="7"/>
       <c r="AR167" s="34"/>
       <c r="AS167" s="34"/>
@@ -23357,9 +23759,7 @@
       <c r="AM168" s="34"/>
       <c r="AN168" s="7"/>
       <c r="AO168" s="7"/>
-      <c r="AP168" s="34">
-        <v>46258</v>
-      </c>
+      <c r="AP168" s="34"/>
       <c r="AQ168" s="7"/>
       <c r="AR168" s="34"/>
       <c r="AS168" s="34"/>
@@ -23484,9 +23884,7 @@
       <c r="AM169" s="34"/>
       <c r="AN169" s="7"/>
       <c r="AO169" s="7"/>
-      <c r="AP169" s="34">
-        <v>46258</v>
-      </c>
+      <c r="AP169" s="34"/>
       <c r="AQ169" s="7"/>
       <c r="AR169" s="34"/>
       <c r="AS169" s="34"/>
@@ -23611,9 +24009,7 @@
       <c r="AM170" s="34"/>
       <c r="AN170" s="7"/>
       <c r="AO170" s="7"/>
-      <c r="AP170" s="34">
-        <v>46258</v>
-      </c>
+      <c r="AP170" s="34"/>
       <c r="AQ170" s="7"/>
       <c r="AR170" s="34"/>
       <c r="AS170" s="34"/>
@@ -23850,10 +24246,18 @@
       <c r="AF172" s="34"/>
       <c r="AG172" s="7"/>
       <c r="AH172" s="34"/>
-      <c r="AI172" s="34"/>
-      <c r="AJ172" s="34"/>
-      <c r="AK172" s="34"/>
-      <c r="AL172" s="34"/>
+      <c r="AI172" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AJ172" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AK172" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AL172" s="34">
+        <v>46287</v>
+      </c>
       <c r="AM172" s="34"/>
       <c r="AN172" s="7"/>
       <c r="AO172" s="7"/>
@@ -24201,10 +24605,18 @@
       <c r="AF175" s="34"/>
       <c r="AG175" s="7"/>
       <c r="AH175" s="34"/>
-      <c r="AI175" s="34"/>
-      <c r="AJ175" s="34"/>
-      <c r="AK175" s="34"/>
-      <c r="AL175" s="34"/>
+      <c r="AI175" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AJ175" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AK175" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AL175" s="34">
+        <v>46286</v>
+      </c>
       <c r="AM175" s="34"/>
       <c r="AN175" s="7"/>
       <c r="AO175" s="7"/>
@@ -24318,10 +24730,18 @@
       <c r="AF176" s="34"/>
       <c r="AG176" s="7"/>
       <c r="AH176" s="34"/>
-      <c r="AI176" s="34"/>
-      <c r="AJ176" s="34"/>
-      <c r="AK176" s="34"/>
-      <c r="AL176" s="34"/>
+      <c r="AI176" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AJ176" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AK176" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AL176" s="34">
+        <v>46286</v>
+      </c>
       <c r="AM176" s="34"/>
       <c r="AN176" s="7"/>
       <c r="AO176" s="7"/>
@@ -24435,10 +24855,18 @@
       <c r="AF177" s="34"/>
       <c r="AG177" s="7"/>
       <c r="AH177" s="34"/>
-      <c r="AI177" s="34"/>
-      <c r="AJ177" s="34"/>
-      <c r="AK177" s="34"/>
-      <c r="AL177" s="34"/>
+      <c r="AI177" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AJ177" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AK177" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AL177" s="34">
+        <v>46286</v>
+      </c>
       <c r="AM177" s="34"/>
       <c r="AN177" s="7"/>
       <c r="AO177" s="7"/>
@@ -24669,10 +25097,18 @@
       <c r="AF179" s="34"/>
       <c r="AG179" s="7"/>
       <c r="AH179" s="34"/>
-      <c r="AI179" s="34"/>
-      <c r="AJ179" s="34"/>
-      <c r="AK179" s="34"/>
-      <c r="AL179" s="34"/>
+      <c r="AI179" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AJ179" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AK179" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AL179" s="34">
+        <v>46285</v>
+      </c>
       <c r="AM179" s="34"/>
       <c r="AN179" s="7"/>
       <c r="AO179" s="7"/>
@@ -24786,10 +25222,18 @@
       <c r="AF180" s="34"/>
       <c r="AG180" s="7"/>
       <c r="AH180" s="34"/>
-      <c r="AI180" s="34"/>
-      <c r="AJ180" s="34"/>
-      <c r="AK180" s="34"/>
-      <c r="AL180" s="34"/>
+      <c r="AI180" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AJ180" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AK180" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AL180" s="34">
+        <v>46285</v>
+      </c>
       <c r="AM180" s="34"/>
       <c r="AN180" s="7"/>
       <c r="AO180" s="7"/>
@@ -24918,7 +25362,9 @@
       <c r="AM181" s="34"/>
       <c r="AN181" s="7"/>
       <c r="AO181" s="7"/>
-      <c r="AP181" s="34"/>
+      <c r="AP181" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ181" s="7"/>
       <c r="AR181" s="34"/>
       <c r="AS181" s="34"/>
@@ -25043,7 +25489,9 @@
       <c r="AM182" s="34"/>
       <c r="AN182" s="7"/>
       <c r="AO182" s="7"/>
-      <c r="AP182" s="34"/>
+      <c r="AP182" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ182" s="7"/>
       <c r="AR182" s="34"/>
       <c r="AS182" s="34"/>
@@ -25168,7 +25616,9 @@
       <c r="AM183" s="34"/>
       <c r="AN183" s="7"/>
       <c r="AO183" s="7"/>
-      <c r="AP183" s="34"/>
+      <c r="AP183" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ183" s="7"/>
       <c r="AR183" s="34"/>
       <c r="AS183" s="34"/>
@@ -25293,7 +25743,9 @@
       <c r="AM184" s="34"/>
       <c r="AN184" s="7"/>
       <c r="AO184" s="7"/>
-      <c r="AP184" s="34"/>
+      <c r="AP184" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ184" s="7"/>
       <c r="AR184" s="34"/>
       <c r="AS184" s="34"/>
@@ -25418,7 +25870,9 @@
       <c r="AM185" s="34"/>
       <c r="AN185" s="7"/>
       <c r="AO185" s="7"/>
-      <c r="AP185" s="34"/>
+      <c r="AP185" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ185" s="7"/>
       <c r="AR185" s="34"/>
       <c r="AS185" s="34"/>
@@ -25543,7 +25997,9 @@
       <c r="AM186" s="34"/>
       <c r="AN186" s="7"/>
       <c r="AO186" s="7"/>
-      <c r="AP186" s="34"/>
+      <c r="AP186" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ186" s="7"/>
       <c r="AR186" s="34"/>
       <c r="AS186" s="34"/>
@@ -25668,7 +26124,9 @@
       <c r="AM187" s="34"/>
       <c r="AN187" s="7"/>
       <c r="AO187" s="7"/>
-      <c r="AP187" s="34"/>
+      <c r="AP187" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ187" s="7"/>
       <c r="AR187" s="34"/>
       <c r="AS187" s="34"/>
@@ -25793,7 +26251,9 @@
       <c r="AM188" s="34"/>
       <c r="AN188" s="7"/>
       <c r="AO188" s="7"/>
-      <c r="AP188" s="34"/>
+      <c r="AP188" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ188" s="7"/>
       <c r="AR188" s="34"/>
       <c r="AS188" s="34"/>
@@ -25918,7 +26378,9 @@
       <c r="AM189" s="34"/>
       <c r="AN189" s="7"/>
       <c r="AO189" s="7"/>
-      <c r="AP189" s="34"/>
+      <c r="AP189" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ189" s="7"/>
       <c r="AR189" s="34"/>
       <c r="AS189" s="34"/>
@@ -26043,7 +26505,9 @@
       <c r="AM190" s="34"/>
       <c r="AN190" s="7"/>
       <c r="AO190" s="7"/>
-      <c r="AP190" s="34"/>
+      <c r="AP190" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ190" s="7"/>
       <c r="AR190" s="34"/>
       <c r="AS190" s="34"/>
@@ -26168,7 +26632,9 @@
       <c r="AM191" s="34"/>
       <c r="AN191" s="7"/>
       <c r="AO191" s="7"/>
-      <c r="AP191" s="34"/>
+      <c r="AP191" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ191" s="7"/>
       <c r="AR191" s="34"/>
       <c r="AS191" s="34"/>
@@ -27180,7 +27646,9 @@
       <c r="AM199" s="34"/>
       <c r="AN199" s="7"/>
       <c r="AO199" s="7"/>
-      <c r="AP199" s="34"/>
+      <c r="AP199" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ199" s="7"/>
       <c r="AR199" s="34"/>
       <c r="AS199" s="34"/>
@@ -27305,7 +27773,9 @@
       <c r="AM200" s="34"/>
       <c r="AN200" s="7"/>
       <c r="AO200" s="7"/>
-      <c r="AP200" s="34"/>
+      <c r="AP200" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ200" s="7"/>
       <c r="AR200" s="34"/>
       <c r="AS200" s="34"/>
@@ -27430,7 +27900,9 @@
       <c r="AM201" s="34"/>
       <c r="AN201" s="7"/>
       <c r="AO201" s="7"/>
-      <c r="AP201" s="34"/>
+      <c r="AP201" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ201" s="7"/>
       <c r="AR201" s="34"/>
       <c r="AS201" s="34"/>
@@ -27555,7 +28027,9 @@
       <c r="AM202" s="34"/>
       <c r="AN202" s="7"/>
       <c r="AO202" s="7"/>
-      <c r="AP202" s="34"/>
+      <c r="AP202" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ202" s="7"/>
       <c r="AR202" s="34"/>
       <c r="AS202" s="34"/>
@@ -27680,7 +28154,9 @@
       <c r="AM203" s="34"/>
       <c r="AN203" s="7"/>
       <c r="AO203" s="7"/>
-      <c r="AP203" s="34"/>
+      <c r="AP203" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ203" s="7"/>
       <c r="AR203" s="34"/>
       <c r="AS203" s="34"/>
@@ -27805,7 +28281,9 @@
       <c r="AM204" s="34"/>
       <c r="AN204" s="7"/>
       <c r="AO204" s="7"/>
-      <c r="AP204" s="34"/>
+      <c r="AP204" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ204" s="7"/>
       <c r="AR204" s="34"/>
       <c r="AS204" s="34"/>
@@ -27930,7 +28408,9 @@
       <c r="AM205" s="34"/>
       <c r="AN205" s="7"/>
       <c r="AO205" s="7"/>
-      <c r="AP205" s="34"/>
+      <c r="AP205" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ205" s="7"/>
       <c r="AR205" s="34"/>
       <c r="AS205" s="34"/>
@@ -28680,9 +29160,7 @@
       <c r="AM211" s="34"/>
       <c r="AN211" s="7"/>
       <c r="AO211" s="7"/>
-      <c r="AP211" s="34">
-        <v>46266</v>
-      </c>
+      <c r="AP211" s="34"/>
       <c r="AQ211" s="7"/>
       <c r="AR211" s="34"/>
       <c r="AS211" s="34"/>
@@ -29061,9 +29539,7 @@
       <c r="AM214" s="34"/>
       <c r="AN214" s="7"/>
       <c r="AO214" s="7"/>
-      <c r="AP214" s="34">
-        <v>46258</v>
-      </c>
+      <c r="AP214" s="34"/>
       <c r="AQ214" s="7"/>
       <c r="AR214" s="34"/>
       <c r="AS214" s="34"/>
@@ -29188,7 +29664,9 @@
       <c r="AM215" s="34"/>
       <c r="AN215" s="7"/>
       <c r="AO215" s="7"/>
-      <c r="AP215" s="34"/>
+      <c r="AP215" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ215" s="7"/>
       <c r="AR215" s="34"/>
       <c r="AS215" s="34"/>
@@ -29557,7 +30035,9 @@
       <c r="AM218" s="34"/>
       <c r="AN218" s="7"/>
       <c r="AO218" s="7"/>
-      <c r="AP218" s="34"/>
+      <c r="AP218" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ218" s="7"/>
       <c r="AR218" s="34"/>
       <c r="AS218" s="34"/>
@@ -29682,7 +30162,9 @@
       <c r="AM219" s="34"/>
       <c r="AN219" s="7"/>
       <c r="AO219" s="7"/>
-      <c r="AP219" s="34"/>
+      <c r="AP219" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ219" s="7"/>
       <c r="AR219" s="34"/>
       <c r="AS219" s="34"/>
@@ -29807,7 +30289,9 @@
       <c r="AM220" s="34"/>
       <c r="AN220" s="7"/>
       <c r="AO220" s="7"/>
-      <c r="AP220" s="34"/>
+      <c r="AP220" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ220" s="7"/>
       <c r="AR220" s="34"/>
       <c r="AS220" s="34"/>
@@ -29932,7 +30416,9 @@
       <c r="AM221" s="34"/>
       <c r="AN221" s="7"/>
       <c r="AO221" s="7"/>
-      <c r="AP221" s="34"/>
+      <c r="AP221" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ221" s="7"/>
       <c r="AR221" s="34"/>
       <c r="AS221" s="34"/>
@@ -30174,7 +30660,9 @@
       <c r="AM223" s="34"/>
       <c r="AN223" s="7"/>
       <c r="AO223" s="7"/>
-      <c r="AP223" s="34"/>
+      <c r="AP223" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ223" s="7"/>
       <c r="AR223" s="34"/>
       <c r="AS223" s="34"/>
@@ -30299,7 +30787,9 @@
       <c r="AM224" s="34"/>
       <c r="AN224" s="7"/>
       <c r="AO224" s="7"/>
-      <c r="AP224" s="34"/>
+      <c r="AP224" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ224" s="7"/>
       <c r="AR224" s="34"/>
       <c r="AS224" s="34"/>
@@ -30424,7 +30914,9 @@
       <c r="AM225" s="34"/>
       <c r="AN225" s="7"/>
       <c r="AO225" s="7"/>
-      <c r="AP225" s="34"/>
+      <c r="AP225" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ225" s="7"/>
       <c r="AR225" s="34"/>
       <c r="AS225" s="34"/>
@@ -30549,7 +31041,9 @@
       <c r="AM226" s="34"/>
       <c r="AN226" s="7"/>
       <c r="AO226" s="7"/>
-      <c r="AP226" s="34"/>
+      <c r="AP226" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ226" s="7"/>
       <c r="AR226" s="34"/>
       <c r="AS226" s="34"/>
@@ -30791,7 +31285,9 @@
       <c r="AM228" s="34"/>
       <c r="AN228" s="7"/>
       <c r="AO228" s="7"/>
-      <c r="AP228" s="34"/>
+      <c r="AP228" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ228" s="7"/>
       <c r="AR228" s="34"/>
       <c r="AS228" s="34"/>
@@ -31150,7 +31646,9 @@
       <c r="AM231" s="34"/>
       <c r="AN231" s="7"/>
       <c r="AO231" s="7"/>
-      <c r="AP231" s="34"/>
+      <c r="AP231" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ231" s="7"/>
       <c r="AR231" s="34"/>
       <c r="AS231" s="34"/>
@@ -31275,7 +31773,9 @@
       <c r="AM232" s="34"/>
       <c r="AN232" s="7"/>
       <c r="AO232" s="7"/>
-      <c r="AP232" s="34"/>
+      <c r="AP232" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ232" s="7"/>
       <c r="AR232" s="34"/>
       <c r="AS232" s="34"/>
@@ -31400,7 +31900,9 @@
       <c r="AM233" s="34"/>
       <c r="AN233" s="7"/>
       <c r="AO233" s="7"/>
-      <c r="AP233" s="34"/>
+      <c r="AP233" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ233" s="7"/>
       <c r="AR233" s="34"/>
       <c r="AS233" s="34"/>
@@ -31510,10 +32012,18 @@
       <c r="AF234" s="34"/>
       <c r="AG234" s="7"/>
       <c r="AH234" s="34"/>
-      <c r="AI234" s="34"/>
-      <c r="AJ234" s="34"/>
-      <c r="AK234" s="34"/>
-      <c r="AL234" s="34"/>
+      <c r="AI234" s="34">
+        <v>46258</v>
+      </c>
+      <c r="AJ234" s="34">
+        <v>46258</v>
+      </c>
+      <c r="AK234" s="34">
+        <v>46258</v>
+      </c>
+      <c r="AL234" s="34">
+        <v>46258</v>
+      </c>
       <c r="AM234" s="34"/>
       <c r="AN234" s="7"/>
       <c r="AO234" s="7"/>
@@ -31642,9 +32152,7 @@
       <c r="AM235" s="34"/>
       <c r="AN235" s="7"/>
       <c r="AO235" s="7"/>
-      <c r="AP235" s="34">
-        <v>46258</v>
-      </c>
+      <c r="AP235" s="34"/>
       <c r="AQ235" s="7"/>
       <c r="AR235" s="34"/>
       <c r="AS235" s="34"/>
@@ -32394,7 +32902,9 @@
       <c r="AM241" s="34"/>
       <c r="AN241" s="7"/>
       <c r="AO241" s="7"/>
-      <c r="AP241" s="34"/>
+      <c r="AP241" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ241" s="7"/>
       <c r="AR241" s="34"/>
       <c r="AS241" s="34"/>
@@ -32636,9 +33146,7 @@
       <c r="AM243" s="34"/>
       <c r="AN243" s="7"/>
       <c r="AO243" s="7"/>
-      <c r="AP243" s="34">
-        <v>46258</v>
-      </c>
+      <c r="AP243" s="34"/>
       <c r="AQ243" s="7"/>
       <c r="AR243" s="34"/>
       <c r="AS243" s="34"/>
@@ -32865,14 +33373,24 @@
       <c r="AF245" s="34"/>
       <c r="AG245" s="7"/>
       <c r="AH245" s="34"/>
-      <c r="AI245" s="34"/>
-      <c r="AJ245" s="34"/>
-      <c r="AK245" s="34"/>
-      <c r="AL245" s="34"/>
+      <c r="AI245" s="34">
+        <v>46254</v>
+      </c>
+      <c r="AJ245" s="34">
+        <v>46254</v>
+      </c>
+      <c r="AK245" s="34">
+        <v>46254</v>
+      </c>
+      <c r="AL245" s="34">
+        <v>46254</v>
+      </c>
       <c r="AM245" s="34"/>
       <c r="AN245" s="7"/>
       <c r="AO245" s="7"/>
-      <c r="AP245" s="34"/>
+      <c r="AP245" s="34">
+        <v>46255</v>
+      </c>
       <c r="AQ245" s="7"/>
       <c r="AR245" s="34"/>
       <c r="AS245" s="34"/>
@@ -34887,10 +35405,18 @@
       <c r="AF261" s="34"/>
       <c r="AG261" s="7"/>
       <c r="AH261" s="34"/>
-      <c r="AI261" s="34"/>
-      <c r="AJ261" s="34"/>
-      <c r="AK261" s="34"/>
-      <c r="AL261" s="34"/>
+      <c r="AI261" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AJ261" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AK261" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AL261" s="34">
+        <v>46285</v>
+      </c>
       <c r="AM261" s="34"/>
       <c r="AN261" s="7"/>
       <c r="AO261" s="7"/>
@@ -35004,10 +35530,18 @@
       <c r="AF262" s="34"/>
       <c r="AG262" s="7"/>
       <c r="AH262" s="34"/>
-      <c r="AI262" s="34"/>
-      <c r="AJ262" s="34"/>
-      <c r="AK262" s="34"/>
-      <c r="AL262" s="34"/>
+      <c r="AI262" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AJ262" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AK262" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AL262" s="34">
+        <v>46285</v>
+      </c>
       <c r="AM262" s="34"/>
       <c r="AN262" s="7"/>
       <c r="AO262" s="7"/>
@@ -35121,10 +35655,18 @@
       <c r="AF263" s="34"/>
       <c r="AG263" s="7"/>
       <c r="AH263" s="34"/>
-      <c r="AI263" s="34"/>
-      <c r="AJ263" s="34"/>
-      <c r="AK263" s="34"/>
-      <c r="AL263" s="34"/>
+      <c r="AI263" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AJ263" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AK263" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AL263" s="34">
+        <v>46285</v>
+      </c>
       <c r="AM263" s="34"/>
       <c r="AN263" s="7"/>
       <c r="AO263" s="7"/>
@@ -35253,7 +35795,9 @@
       <c r="AM264" s="34"/>
       <c r="AN264" s="7"/>
       <c r="AO264" s="7"/>
-      <c r="AP264" s="34"/>
+      <c r="AP264" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ264" s="7"/>
       <c r="AR264" s="34"/>
       <c r="AS264" s="34"/>
@@ -35378,7 +35922,9 @@
       <c r="AM265" s="34"/>
       <c r="AN265" s="7"/>
       <c r="AO265" s="7"/>
-      <c r="AP265" s="34"/>
+      <c r="AP265" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ265" s="7"/>
       <c r="AR265" s="34"/>
       <c r="AS265" s="34"/>
@@ -35503,7 +36049,9 @@
       <c r="AM266" s="34"/>
       <c r="AN266" s="7"/>
       <c r="AO266" s="7"/>
-      <c r="AP266" s="34"/>
+      <c r="AP266" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ266" s="7"/>
       <c r="AR266" s="34"/>
       <c r="AS266" s="34"/>
@@ -35882,7 +36430,9 @@
       <c r="AM269" s="34"/>
       <c r="AN269" s="7"/>
       <c r="AO269" s="7"/>
-      <c r="AP269" s="34"/>
+      <c r="AP269" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ269" s="7"/>
       <c r="AR269" s="34"/>
       <c r="AS269" s="34"/>
@@ -36007,7 +36557,9 @@
       <c r="AM270" s="34"/>
       <c r="AN270" s="7"/>
       <c r="AO270" s="7"/>
-      <c r="AP270" s="34"/>
+      <c r="AP270" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ270" s="7"/>
       <c r="AR270" s="34"/>
       <c r="AS270" s="34"/>
@@ -36132,7 +36684,9 @@
       <c r="AM271" s="34"/>
       <c r="AN271" s="7"/>
       <c r="AO271" s="7"/>
-      <c r="AP271" s="34"/>
+      <c r="AP271" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ271" s="7"/>
       <c r="AR271" s="34"/>
       <c r="AS271" s="34"/>

</xml_diff>

<commit_message>
Preenche espessura do spool com a maior espessura da linha
A coluna Espessura do Mapa de Spools recebe a maior espessura entre
todas as juntas da mesma linha no Mapa de Juntas (Pipe e Campo).
Espessuras em texto com vírgula (' 4,55') são convertidas para número.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jhm2rrJCBVkJYZMmi4pDeT
</commit_message>
<xml_diff>
--- a/saida/Situacao_Geral_de_Spools_ATUALIZADO.xlsx
+++ b/saida/Situacao_Geral_de_Spools_ATUALIZADO.xlsx
@@ -3687,7 +3687,9 @@
       <c r="Q9" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="R9" s="7"/>
+      <c r="R9" s="7">
+        <v>6.02</v>
+      </c>
       <c r="S9" s="7" t="s">
         <v>455</v>
       </c>
@@ -3821,7 +3823,9 @@
       <c r="Q10" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="R10" s="7"/>
+      <c r="R10" s="7">
+        <v>6.02</v>
+      </c>
       <c r="S10" s="7" t="s">
         <v>455</v>
       </c>
@@ -3940,7 +3944,9 @@
       <c r="Q11" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="R11" s="7"/>
+      <c r="R11" s="7">
+        <v>6.02</v>
+      </c>
       <c r="S11" s="7" t="s">
         <v>455</v>
       </c>
@@ -4069,7 +4075,9 @@
       <c r="Q12" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="R12" s="7"/>
+      <c r="R12" s="7">
+        <v>6.02</v>
+      </c>
       <c r="S12" s="7" t="s">
         <v>455</v>
       </c>
@@ -4198,7 +4206,9 @@
       <c r="Q13" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="R13" s="7"/>
+      <c r="R13" s="7">
+        <v>6.02</v>
+      </c>
       <c r="S13" s="7" t="s">
         <v>455</v>
       </c>
@@ -4327,7 +4337,9 @@
       <c r="Q14" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="R14" s="7"/>
+      <c r="R14" s="7">
+        <v>6.02</v>
+      </c>
       <c r="S14" s="7" t="s">
         <v>455</v>
       </c>
@@ -4456,7 +4468,9 @@
       <c r="Q15" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R15" s="7"/>
+      <c r="R15" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S15" s="7" t="s">
         <v>456</v>
       </c>
@@ -4585,7 +4599,9 @@
       <c r="Q16" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R16" s="7"/>
+      <c r="R16" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S16" s="7" t="s">
         <v>456</v>
       </c>
@@ -4714,7 +4730,9 @@
       <c r="Q17" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R17" s="7"/>
+      <c r="R17" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S17" s="7" t="s">
         <v>456</v>
       </c>
@@ -4843,7 +4861,9 @@
       <c r="Q18" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R18" s="7"/>
+      <c r="R18" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S18" s="7" t="s">
         <v>456</v>
       </c>
@@ -4972,7 +4992,9 @@
       <c r="Q19" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R19" s="7"/>
+      <c r="R19" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S19" s="7" t="s">
         <v>456</v>
       </c>
@@ -5101,7 +5123,9 @@
       <c r="Q20" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R20" s="7"/>
+      <c r="R20" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S20" s="7" t="s">
         <v>456</v>
       </c>
@@ -5220,7 +5244,9 @@
       <c r="Q21" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R21" s="7"/>
+      <c r="R21" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S21" s="7" t="s">
         <v>456</v>
       </c>
@@ -5349,7 +5375,9 @@
       <c r="Q22" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R22" s="7"/>
+      <c r="R22" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S22" s="7" t="s">
         <v>457</v>
       </c>
@@ -5478,7 +5506,9 @@
       <c r="Q23" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R23" s="7"/>
+      <c r="R23" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S23" s="7" t="s">
         <v>457</v>
       </c>
@@ -5607,7 +5637,9 @@
       <c r="Q24" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R24" s="7"/>
+      <c r="R24" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S24" s="7" t="s">
         <v>457</v>
       </c>
@@ -5736,7 +5768,9 @@
       <c r="Q25" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R25" s="7"/>
+      <c r="R25" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S25" s="7" t="s">
         <v>457</v>
       </c>
@@ -5865,7 +5899,9 @@
       <c r="Q26" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R26" s="7"/>
+      <c r="R26" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S26" s="7" t="s">
         <v>457</v>
       </c>
@@ -5994,7 +6030,9 @@
       <c r="Q27" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R27" s="7"/>
+      <c r="R27" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S27" s="7" t="s">
         <v>457</v>
       </c>
@@ -6113,7 +6151,9 @@
       <c r="Q28" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R28" s="7"/>
+      <c r="R28" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S28" s="7" t="s">
         <v>457</v>
       </c>
@@ -6232,7 +6272,9 @@
       <c r="Q29" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R29" s="7"/>
+      <c r="R29" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S29" s="7" t="s">
         <v>457</v>
       </c>
@@ -6351,7 +6393,9 @@
       <c r="Q30" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R30" s="7"/>
+      <c r="R30" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S30" s="7" t="s">
         <v>457</v>
       </c>
@@ -6480,7 +6524,9 @@
       <c r="Q31" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R31" s="7"/>
+      <c r="R31" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S31" s="7" t="s">
         <v>457</v>
       </c>
@@ -6599,7 +6645,9 @@
       <c r="Q32" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R32" s="7"/>
+      <c r="R32" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S32" s="7" t="s">
         <v>457</v>
       </c>
@@ -6728,7 +6776,9 @@
       <c r="Q33" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R33" s="7"/>
+      <c r="R33" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S33" s="7" t="s">
         <v>457</v>
       </c>
@@ -6857,7 +6907,9 @@
       <c r="Q34" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R34" s="7"/>
+      <c r="R34" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S34" s="7" t="s">
         <v>457</v>
       </c>
@@ -6986,7 +7038,9 @@
       <c r="Q35" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R35" s="7"/>
+      <c r="R35" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S35" s="7" t="s">
         <v>457</v>
       </c>
@@ -7115,7 +7169,9 @@
       <c r="Q36" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R36" s="7"/>
+      <c r="R36" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S36" s="7" t="s">
         <v>457</v>
       </c>
@@ -7244,7 +7300,9 @@
       <c r="Q37" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R37" s="7"/>
+      <c r="R37" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S37" s="7" t="s">
         <v>457</v>
       </c>
@@ -7371,7 +7429,9 @@
       <c r="Q38" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R38" s="7"/>
+      <c r="R38" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S38" s="7" t="s">
         <v>457</v>
       </c>
@@ -7498,7 +7558,9 @@
       <c r="Q39" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R39" s="7"/>
+      <c r="R39" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S39" s="7" t="s">
         <v>457</v>
       </c>
@@ -7625,7 +7687,9 @@
       <c r="Q40" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R40" s="7"/>
+      <c r="R40" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S40" s="7" t="s">
         <v>458</v>
       </c>
@@ -7754,7 +7818,9 @@
       <c r="Q41" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R41" s="7"/>
+      <c r="R41" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S41" s="7" t="s">
         <v>458</v>
       </c>
@@ -7883,7 +7949,9 @@
       <c r="Q42" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R42" s="7"/>
+      <c r="R42" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S42" s="7" t="s">
         <v>458</v>
       </c>
@@ -8012,7 +8080,9 @@
       <c r="Q43" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R43" s="7"/>
+      <c r="R43" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S43" s="7" t="s">
         <v>458</v>
       </c>
@@ -8141,7 +8211,9 @@
       <c r="Q44" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R44" s="7"/>
+      <c r="R44" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S44" s="7" t="s">
         <v>458</v>
       </c>
@@ -8270,7 +8342,9 @@
       <c r="Q45" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R45" s="7"/>
+      <c r="R45" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S45" s="7" t="s">
         <v>455</v>
       </c>
@@ -8397,7 +8471,9 @@
       <c r="Q46" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R46" s="7"/>
+      <c r="R46" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S46" s="7" t="s">
         <v>455</v>
       </c>
@@ -8526,7 +8602,9 @@
       <c r="Q47" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R47" s="7"/>
+      <c r="R47" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S47" s="7" t="s">
         <v>455</v>
       </c>
@@ -8655,7 +8733,9 @@
       <c r="Q48" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R48" s="7"/>
+      <c r="R48" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S48" s="7" t="s">
         <v>455</v>
       </c>
@@ -8784,7 +8864,9 @@
       <c r="Q49" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R49" s="7"/>
+      <c r="R49" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S49" s="7" t="s">
         <v>455</v>
       </c>
@@ -8913,7 +8995,9 @@
       <c r="Q50" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R50" s="7"/>
+      <c r="R50" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S50" s="7" t="s">
         <v>455</v>
       </c>
@@ -9042,7 +9126,9 @@
       <c r="Q51" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R51" s="7"/>
+      <c r="R51" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S51" s="7" t="s">
         <v>455</v>
       </c>
@@ -9171,7 +9257,9 @@
       <c r="Q52" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R52" s="7"/>
+      <c r="R52" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S52" s="7" t="s">
         <v>455</v>
       </c>
@@ -9300,7 +9388,9 @@
       <c r="Q53" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R53" s="7"/>
+      <c r="R53" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S53" s="7" t="s">
         <v>455</v>
       </c>
@@ -9429,7 +9519,9 @@
       <c r="Q54" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R54" s="7"/>
+      <c r="R54" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S54" s="7" t="s">
         <v>459</v>
       </c>
@@ -9558,7 +9650,9 @@
       <c r="Q55" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R55" s="7"/>
+      <c r="R55" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S55" s="7" t="s">
         <v>459</v>
       </c>
@@ -9687,7 +9781,9 @@
       <c r="Q56" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R56" s="7"/>
+      <c r="R56" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S56" s="7" t="s">
         <v>459</v>
       </c>
@@ -9816,7 +9912,9 @@
       <c r="Q57" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R57" s="7"/>
+      <c r="R57" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S57" s="7" t="s">
         <v>459</v>
       </c>
@@ -9945,7 +10043,9 @@
       <c r="Q58" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R58" s="7"/>
+      <c r="R58" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S58" s="7" t="s">
         <v>460</v>
       </c>
@@ -10064,7 +10164,9 @@
       <c r="Q59" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="R59" s="7"/>
+      <c r="R59" s="7">
+        <v>3.68</v>
+      </c>
       <c r="S59" s="7" t="s">
         <v>456</v>
       </c>
@@ -10191,7 +10293,9 @@
       <c r="Q60" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="R60" s="7"/>
+      <c r="R60" s="7">
+        <v>3.68</v>
+      </c>
       <c r="S60" s="7" t="s">
         <v>456</v>
       </c>
@@ -10320,7 +10424,9 @@
       <c r="Q61" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="R61" s="7"/>
+      <c r="R61" s="7">
+        <v>3.68</v>
+      </c>
       <c r="S61" s="7" t="s">
         <v>456</v>
       </c>
@@ -10449,7 +10555,9 @@
       <c r="Q62" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="R62" s="7"/>
+      <c r="R62" s="7">
+        <v>5.08</v>
+      </c>
       <c r="S62" s="7" t="s">
         <v>457</v>
       </c>
@@ -10578,7 +10686,9 @@
       <c r="Q63" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="R63" s="7"/>
+      <c r="R63" s="7">
+        <v>5.08</v>
+      </c>
       <c r="S63" s="7" t="s">
         <v>457</v>
       </c>
@@ -10707,7 +10817,9 @@
       <c r="Q64" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="R64" s="7"/>
+      <c r="R64" s="7">
+        <v>5.08</v>
+      </c>
       <c r="S64" s="7" t="s">
         <v>457</v>
       </c>
@@ -10836,7 +10948,9 @@
       <c r="Q65" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="R65" s="7"/>
+      <c r="R65" s="7">
+        <v>5.08</v>
+      </c>
       <c r="S65" s="7" t="s">
         <v>457</v>
       </c>
@@ -10965,7 +11079,9 @@
       <c r="Q66" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="R66" s="7"/>
+      <c r="R66" s="7">
+        <v>3.73</v>
+      </c>
       <c r="S66" s="7" t="s">
         <v>457</v>
       </c>
@@ -11094,7 +11210,9 @@
       <c r="Q67" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="R67" s="7"/>
+      <c r="R67" s="7">
+        <v>3.73</v>
+      </c>
       <c r="S67" s="7" t="s">
         <v>457</v>
       </c>
@@ -11223,7 +11341,9 @@
       <c r="Q68" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R68" s="7"/>
+      <c r="R68" s="7">
+        <v>9.27</v>
+      </c>
       <c r="S68" s="7" t="s">
         <v>457</v>
       </c>
@@ -11352,7 +11472,9 @@
       <c r="Q69" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R69" s="7"/>
+      <c r="R69" s="7">
+        <v>8.18</v>
+      </c>
       <c r="S69" s="7" t="s">
         <v>457</v>
       </c>
@@ -11481,7 +11603,9 @@
       <c r="Q70" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R70" s="7"/>
+      <c r="R70" s="7">
+        <v>9.27</v>
+      </c>
       <c r="S70" s="7" t="s">
         <v>457</v>
       </c>
@@ -11608,7 +11732,9 @@
       <c r="Q71" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R71" s="7"/>
+      <c r="R71" s="7">
+        <v>9.27</v>
+      </c>
       <c r="S71" s="7" t="s">
         <v>457</v>
       </c>
@@ -11737,7 +11863,9 @@
       <c r="Q72" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R72" s="7"/>
+      <c r="R72" s="7">
+        <v>9.27</v>
+      </c>
       <c r="S72" s="7" t="s">
         <v>455</v>
       </c>
@@ -11866,7 +11994,9 @@
       <c r="Q73" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R73" s="7"/>
+      <c r="R73" s="7">
+        <v>9.27</v>
+      </c>
       <c r="S73" s="7" t="s">
         <v>455</v>
       </c>
@@ -11995,7 +12125,9 @@
       <c r="Q74" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R74" s="7"/>
+      <c r="R74" s="7">
+        <v>9.27</v>
+      </c>
       <c r="S74" s="7" t="s">
         <v>455</v>
       </c>
@@ -12124,7 +12256,9 @@
       <c r="Q75" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R75" s="7"/>
+      <c r="R75" s="7">
+        <v>9.27</v>
+      </c>
       <c r="S75" s="7" t="s">
         <v>455</v>
       </c>
@@ -12243,7 +12377,9 @@
       <c r="Q76" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R76" s="7"/>
+      <c r="R76" s="7">
+        <v>9.27</v>
+      </c>
       <c r="S76" s="7" t="s">
         <v>455</v>
       </c>
@@ -12372,7 +12508,9 @@
       <c r="Q77" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R77" s="7"/>
+      <c r="R77" s="7">
+        <v>9.27</v>
+      </c>
       <c r="S77" s="7" t="s">
         <v>455</v>
       </c>
@@ -12501,7 +12639,9 @@
       <c r="Q78" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R78" s="7"/>
+      <c r="R78" s="7">
+        <v>9.27</v>
+      </c>
       <c r="S78" s="7" t="s">
         <v>455</v>
       </c>
@@ -12630,7 +12770,9 @@
       <c r="Q79" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R79" s="7"/>
+      <c r="R79" s="7">
+        <v>9.27</v>
+      </c>
       <c r="S79" s="7" t="s">
         <v>455</v>
       </c>
@@ -12759,7 +12901,9 @@
       <c r="Q80" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R80" s="7"/>
+      <c r="R80" s="7">
+        <v>9.27</v>
+      </c>
       <c r="S80" s="7" t="s">
         <v>455</v>
       </c>
@@ -12888,7 +13032,9 @@
       <c r="Q81" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R81" s="7"/>
+      <c r="R81" s="7">
+        <v>9.27</v>
+      </c>
       <c r="S81" s="7" t="s">
         <v>455</v>
       </c>
@@ -13007,7 +13153,9 @@
       <c r="Q82" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R82" s="7"/>
+      <c r="R82" s="7">
+        <v>9.27</v>
+      </c>
       <c r="S82" s="7" t="s">
         <v>455</v>
       </c>
@@ -13126,7 +13274,9 @@
       <c r="Q83" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R83" s="7"/>
+      <c r="R83" s="7">
+        <v>9.27</v>
+      </c>
       <c r="S83" s="7" t="s">
         <v>455</v>
       </c>
@@ -13245,7 +13395,9 @@
       <c r="Q84" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R84" s="7"/>
+      <c r="R84" s="7">
+        <v>9.27</v>
+      </c>
       <c r="S84" s="7" t="s">
         <v>455</v>
       </c>
@@ -13364,7 +13516,9 @@
       <c r="Q85" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R85" s="7"/>
+      <c r="R85" s="7">
+        <v>9.27</v>
+      </c>
       <c r="S85" s="7" t="s">
         <v>455</v>
       </c>
@@ -13483,7 +13637,9 @@
       <c r="Q86" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R86" s="7"/>
+      <c r="R86" s="7">
+        <v>9.27</v>
+      </c>
       <c r="S86" s="7" t="s">
         <v>455</v>
       </c>
@@ -13602,7 +13758,9 @@
       <c r="Q87" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="R87" s="7"/>
+      <c r="R87" s="7">
+        <v>6.35</v>
+      </c>
       <c r="S87" s="7" t="s">
         <v>455</v>
       </c>
@@ -13729,7 +13887,9 @@
       <c r="Q88" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="R88" s="7"/>
+      <c r="R88" s="7">
+        <v>6.35</v>
+      </c>
       <c r="S88" s="7" t="s">
         <v>455</v>
       </c>
@@ -13856,7 +14016,9 @@
       <c r="Q89" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R89" s="7"/>
+      <c r="R89" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S89" s="7"/>
       <c r="T89" s="7" t="s">
         <v>448</v>
@@ -13983,7 +14145,9 @@
       <c r="Q90" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R90" s="7"/>
+      <c r="R90" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S90" s="7"/>
       <c r="T90" s="7" t="s">
         <v>103</v>
@@ -14108,7 +14272,9 @@
       <c r="Q91" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R91" s="7"/>
+      <c r="R91" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S91" s="7"/>
       <c r="T91" s="7" t="s">
         <v>103</v>
@@ -14233,7 +14399,9 @@
       <c r="Q92" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R92" s="7"/>
+      <c r="R92" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S92" s="7"/>
       <c r="T92" s="7" t="s">
         <v>103</v>
@@ -14358,7 +14526,9 @@
       <c r="Q93" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R93" s="7"/>
+      <c r="R93" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S93" s="7"/>
       <c r="T93" s="7" t="s">
         <v>103</v>
@@ -14483,7 +14653,9 @@
       <c r="Q94" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R94" s="7"/>
+      <c r="R94" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S94" s="7"/>
       <c r="T94" s="7" t="s">
         <v>103</v>
@@ -14608,7 +14780,9 @@
       <c r="Q95" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R95" s="7"/>
+      <c r="R95" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S95" s="7"/>
       <c r="T95" s="7" t="s">
         <v>103</v>
@@ -14733,7 +14907,9 @@
       <c r="Q96" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R96" s="7"/>
+      <c r="R96" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S96" s="7"/>
       <c r="T96" s="7" t="s">
         <v>103</v>
@@ -14858,7 +15034,9 @@
       <c r="Q97" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R97" s="7"/>
+      <c r="R97" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S97" s="7"/>
       <c r="T97" s="7" t="s">
         <v>103</v>
@@ -14983,7 +15161,9 @@
       <c r="Q98" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R98" s="7"/>
+      <c r="R98" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S98" s="7"/>
       <c r="T98" s="7" t="s">
         <v>103</v>
@@ -15108,7 +15288,9 @@
       <c r="Q99" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R99" s="7"/>
+      <c r="R99" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S99" s="7"/>
       <c r="T99" s="7" t="s">
         <v>103</v>
@@ -15233,7 +15415,9 @@
       <c r="Q100" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R100" s="7"/>
+      <c r="R100" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S100" s="7"/>
       <c r="T100" s="7" t="s">
         <v>103</v>
@@ -15358,7 +15542,9 @@
       <c r="Q101" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R101" s="7"/>
+      <c r="R101" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S101" s="7"/>
       <c r="T101" s="7" t="s">
         <v>103</v>
@@ -15483,7 +15669,9 @@
       <c r="Q102" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R102" s="7"/>
+      <c r="R102" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S102" s="7"/>
       <c r="T102" s="7" t="s">
         <v>103</v>
@@ -15608,7 +15796,9 @@
       <c r="Q103" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R103" s="7"/>
+      <c r="R103" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S103" s="7"/>
       <c r="T103" s="7" t="s">
         <v>103</v>
@@ -15733,7 +15923,9 @@
       <c r="Q104" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R104" s="7"/>
+      <c r="R104" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S104" s="7"/>
       <c r="T104" s="7" t="s">
         <v>103</v>
@@ -15850,7 +16042,9 @@
       <c r="Q105" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R105" s="7"/>
+      <c r="R105" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S105" s="7"/>
       <c r="T105" s="7" t="s">
         <v>103</v>
@@ -15975,7 +16169,9 @@
       <c r="Q106" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R106" s="7"/>
+      <c r="R106" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S106" s="7"/>
       <c r="T106" s="7" t="s">
         <v>103</v>
@@ -16100,7 +16296,9 @@
       <c r="Q107" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R107" s="7"/>
+      <c r="R107" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S107" s="7"/>
       <c r="T107" s="7" t="s">
         <v>103</v>
@@ -16225,7 +16423,9 @@
       <c r="Q108" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R108" s="7"/>
+      <c r="R108" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S108" s="7"/>
       <c r="T108" s="7" t="s">
         <v>103</v>
@@ -16342,7 +16542,9 @@
       <c r="Q109" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R109" s="7"/>
+      <c r="R109" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S109" s="7"/>
       <c r="T109" s="7" t="s">
         <v>103</v>
@@ -16467,7 +16669,9 @@
       <c r="Q110" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R110" s="7"/>
+      <c r="R110" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S110" s="7"/>
       <c r="T110" s="7" t="s">
         <v>103</v>
@@ -16592,7 +16796,9 @@
       <c r="Q111" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R111" s="7"/>
+      <c r="R111" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S111" s="7"/>
       <c r="T111" s="7" t="s">
         <v>103</v>
@@ -16717,7 +16923,9 @@
       <c r="Q112" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R112" s="7"/>
+      <c r="R112" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S112" s="7"/>
       <c r="T112" s="7" t="s">
         <v>103</v>
@@ -16834,7 +17042,9 @@
       <c r="Q113" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R113" s="7"/>
+      <c r="R113" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S113" s="7"/>
       <c r="T113" s="7" t="s">
         <v>103</v>
@@ -16959,7 +17169,9 @@
       <c r="Q114" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R114" s="7"/>
+      <c r="R114" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S114" s="7"/>
       <c r="T114" s="7" t="s">
         <v>103</v>
@@ -17076,7 +17288,9 @@
       <c r="Q115" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R115" s="7"/>
+      <c r="R115" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S115" s="7"/>
       <c r="T115" s="7" t="s">
         <v>103</v>
@@ -17201,7 +17415,9 @@
       <c r="Q116" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R116" s="7"/>
+      <c r="R116" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S116" s="7"/>
       <c r="T116" s="7" t="s">
         <v>103</v>
@@ -17318,7 +17534,9 @@
       <c r="Q117" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R117" s="7"/>
+      <c r="R117" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S117" s="7"/>
       <c r="T117" s="7" t="s">
         <v>103</v>
@@ -17435,7 +17653,9 @@
       <c r="Q118" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R118" s="7"/>
+      <c r="R118" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S118" s="7"/>
       <c r="T118" s="7" t="s">
         <v>103</v>
@@ -17560,7 +17780,9 @@
       <c r="Q119" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R119" s="7"/>
+      <c r="R119" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S119" s="7"/>
       <c r="T119" s="7" t="s">
         <v>103</v>
@@ -17685,7 +17907,9 @@
       <c r="Q120" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R120" s="7"/>
+      <c r="R120" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S120" s="7"/>
       <c r="T120" s="7" t="s">
         <v>103</v>
@@ -17812,7 +18036,9 @@
       <c r="Q121" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R121" s="7"/>
+      <c r="R121" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S121" s="7"/>
       <c r="T121" s="7" t="s">
         <v>103</v>
@@ -17929,7 +18155,9 @@
       <c r="Q122" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R122" s="7"/>
+      <c r="R122" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S122" s="7"/>
       <c r="T122" s="7" t="s">
         <v>103</v>
@@ -18046,7 +18274,9 @@
       <c r="Q123" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R123" s="7"/>
+      <c r="R123" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S123" s="7"/>
       <c r="T123" s="7" t="s">
         <v>103</v>
@@ -18173,7 +18403,9 @@
       <c r="Q124" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R124" s="7"/>
+      <c r="R124" s="7">
+        <v>3.38</v>
+      </c>
       <c r="S124" s="7"/>
       <c r="T124" s="7" t="s">
         <v>103</v>
@@ -18300,7 +18532,9 @@
       <c r="Q125" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R125" s="7"/>
+      <c r="R125" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S125" s="7"/>
       <c r="T125" s="7" t="s">
         <v>103</v>
@@ -18425,7 +18659,9 @@
       <c r="Q126" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R126" s="7"/>
+      <c r="R126" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S126" s="7"/>
       <c r="T126" s="7" t="s">
         <v>103</v>
@@ -18550,7 +18786,9 @@
       <c r="Q127" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R127" s="7"/>
+      <c r="R127" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S127" s="7"/>
       <c r="T127" s="7" t="s">
         <v>103</v>
@@ -18675,7 +18913,9 @@
       <c r="Q128" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R128" s="7"/>
+      <c r="R128" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S128" s="7"/>
       <c r="T128" s="7" t="s">
         <v>103</v>
@@ -18802,7 +19042,9 @@
       <c r="Q129" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R129" s="7"/>
+      <c r="R129" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S129" s="7"/>
       <c r="T129" s="7" t="s">
         <v>103</v>
@@ -18929,7 +19171,9 @@
       <c r="Q130" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R130" s="7"/>
+      <c r="R130" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S130" s="7"/>
       <c r="T130" s="7" t="s">
         <v>103</v>
@@ -19056,7 +19300,9 @@
       <c r="Q131" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R131" s="7"/>
+      <c r="R131" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S131" s="7"/>
       <c r="T131" s="7" t="s">
         <v>103</v>
@@ -19183,7 +19429,9 @@
       <c r="Q132" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R132" s="7"/>
+      <c r="R132" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S132" s="7"/>
       <c r="T132" s="7" t="s">
         <v>103</v>
@@ -19310,7 +19558,9 @@
       <c r="Q133" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R133" s="7"/>
+      <c r="R133" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S133" s="7"/>
       <c r="T133" s="7" t="s">
         <v>103</v>
@@ -19437,7 +19687,9 @@
       <c r="Q134" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R134" s="7"/>
+      <c r="R134" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S134" s="7"/>
       <c r="T134" s="7" t="s">
         <v>448</v>
@@ -19564,7 +19816,9 @@
       <c r="Q135" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R135" s="7"/>
+      <c r="R135" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S135" s="7"/>
       <c r="T135" s="7" t="s">
         <v>448</v>
@@ -19691,7 +19945,9 @@
       <c r="Q136" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R136" s="7"/>
+      <c r="R136" s="7">
+        <v>2.77</v>
+      </c>
       <c r="S136" s="7"/>
       <c r="T136" s="7" t="s">
         <v>448</v>
@@ -19818,7 +20074,9 @@
       <c r="Q137" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R137" s="7"/>
+      <c r="R137" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S137" s="7"/>
       <c r="T137" s="7" t="s">
         <v>448</v>
@@ -19945,7 +20203,9 @@
       <c r="Q138" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R138" s="7"/>
+      <c r="R138" s="7">
+        <v>5.08</v>
+      </c>
       <c r="S138" s="7"/>
       <c r="T138" s="7" t="s">
         <v>448</v>
@@ -20072,7 +20332,9 @@
       <c r="Q139" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R139" s="7"/>
+      <c r="R139" s="7">
+        <v>5.08</v>
+      </c>
       <c r="S139" s="7"/>
       <c r="T139" s="7" t="s">
         <v>448</v>
@@ -20199,7 +20461,9 @@
       <c r="Q140" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R140" s="7"/>
+      <c r="R140" s="7">
+        <v>5.08</v>
+      </c>
       <c r="S140" s="7"/>
       <c r="T140" s="7" t="s">
         <v>448</v>
@@ -20326,7 +20590,9 @@
       <c r="Q141" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R141" s="7"/>
+      <c r="R141" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S141" s="7"/>
       <c r="T141" s="7" t="s">
         <v>448</v>
@@ -20453,7 +20719,9 @@
       <c r="Q142" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R142" s="7"/>
+      <c r="R142" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S142" s="7"/>
       <c r="T142" s="7" t="s">
         <v>448</v>
@@ -20578,7 +20846,9 @@
       <c r="Q143" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R143" s="7"/>
+      <c r="R143" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S143" s="7"/>
       <c r="T143" s="7" t="s">
         <v>448</v>
@@ -20705,7 +20975,9 @@
       <c r="Q144" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R144" s="7"/>
+      <c r="R144" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S144" s="7"/>
       <c r="T144" s="7" t="s">
         <v>448</v>
@@ -20832,7 +21104,9 @@
       <c r="Q145" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R145" s="7"/>
+      <c r="R145" s="7">
+        <v>4.55</v>
+      </c>
       <c r="S145" s="7"/>
       <c r="T145" s="7" t="s">
         <v>448</v>
@@ -20959,7 +21233,9 @@
       <c r="Q146" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R146" s="7"/>
+      <c r="R146" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S146" s="7"/>
       <c r="T146" s="7" t="s">
         <v>103</v>
@@ -21084,7 +21360,9 @@
       <c r="Q147" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R147" s="7"/>
+      <c r="R147" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S147" s="7"/>
       <c r="T147" s="7" t="s">
         <v>448</v>
@@ -21201,7 +21479,9 @@
       <c r="Q148" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R148" s="7"/>
+      <c r="R148" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S148" s="7"/>
       <c r="T148" s="7" t="s">
         <v>448</v>
@@ -21328,7 +21608,9 @@
       <c r="Q149" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R149" s="7"/>
+      <c r="R149" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S149" s="7"/>
       <c r="T149" s="7" t="s">
         <v>448</v>
@@ -21455,7 +21737,9 @@
       <c r="Q150" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R150" s="7"/>
+      <c r="R150" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S150" s="7"/>
       <c r="T150" s="7" t="s">
         <v>448</v>
@@ -21582,7 +21866,9 @@
       <c r="Q151" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R151" s="7"/>
+      <c r="R151" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S151" s="7"/>
       <c r="T151" s="7" t="s">
         <v>448</v>
@@ -21709,7 +21995,9 @@
       <c r="Q152" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R152" s="7"/>
+      <c r="R152" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S152" s="7"/>
       <c r="T152" s="7" t="s">
         <v>448</v>
@@ -21836,7 +22124,9 @@
       <c r="Q153" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R153" s="7"/>
+      <c r="R153" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S153" s="7"/>
       <c r="T153" s="7" t="s">
         <v>448</v>
@@ -21963,7 +22253,9 @@
       <c r="Q154" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R154" s="7"/>
+      <c r="R154" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S154" s="7"/>
       <c r="T154" s="7" t="s">
         <v>448</v>
@@ -22090,7 +22382,9 @@
       <c r="Q155" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R155" s="7"/>
+      <c r="R155" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S155" s="7"/>
       <c r="T155" s="7" t="s">
         <v>448</v>
@@ -22207,7 +22501,9 @@
       <c r="Q156" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R156" s="7"/>
+      <c r="R156" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S156" s="7"/>
       <c r="T156" s="7" t="s">
         <v>448</v>
@@ -22334,7 +22630,9 @@
       <c r="Q157" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R157" s="7"/>
+      <c r="R157" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S157" s="7"/>
       <c r="T157" s="7" t="s">
         <v>448</v>
@@ -22461,7 +22759,9 @@
       <c r="Q158" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R158" s="7"/>
+      <c r="R158" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S158" s="7"/>
       <c r="T158" s="7" t="s">
         <v>448</v>
@@ -22588,7 +22888,9 @@
       <c r="Q159" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R159" s="7"/>
+      <c r="R159" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S159" s="7"/>
       <c r="T159" s="7" t="s">
         <v>448</v>
@@ -22715,7 +23017,9 @@
       <c r="Q160" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R160" s="7"/>
+      <c r="R160" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S160" s="7"/>
       <c r="T160" s="7" t="s">
         <v>448</v>
@@ -22842,7 +23146,9 @@
       <c r="Q161" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R161" s="7"/>
+      <c r="R161" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S161" s="7"/>
       <c r="T161" s="7" t="s">
         <v>448</v>
@@ -22969,7 +23275,9 @@
       <c r="Q162" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R162" s="7"/>
+      <c r="R162" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S162" s="7"/>
       <c r="T162" s="7" t="s">
         <v>448</v>
@@ -23086,7 +23394,9 @@
       <c r="Q163" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R163" s="7"/>
+      <c r="R163" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S163" s="7"/>
       <c r="T163" s="7" t="s">
         <v>448</v>
@@ -23213,7 +23523,9 @@
       <c r="Q164" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R164" s="7"/>
+      <c r="R164" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S164" s="7"/>
       <c r="T164" s="7" t="s">
         <v>103</v>
@@ -23338,7 +23650,9 @@
       <c r="Q165" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="R165" s="7"/>
+      <c r="R165" s="7">
+        <v>9.53</v>
+      </c>
       <c r="S165" s="7"/>
       <c r="T165" s="7" t="s">
         <v>103</v>
@@ -23463,7 +23777,9 @@
       <c r="Q166" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="R166" s="7"/>
+      <c r="R166" s="7">
+        <v>9.53</v>
+      </c>
       <c r="S166" s="7"/>
       <c r="T166" s="7" t="s">
         <v>103</v>
@@ -23588,7 +23904,9 @@
       <c r="Q167" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="R167" s="7"/>
+      <c r="R167" s="7">
+        <v>9.53</v>
+      </c>
       <c r="S167" s="7"/>
       <c r="T167" s="7" t="s">
         <v>103</v>
@@ -23713,7 +24031,9 @@
       <c r="Q168" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="R168" s="7"/>
+      <c r="R168" s="7">
+        <v>9.53</v>
+      </c>
       <c r="S168" s="7"/>
       <c r="T168" s="7" t="s">
         <v>103</v>
@@ -23838,7 +24158,9 @@
       <c r="Q169" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="R169" s="7"/>
+      <c r="R169" s="7">
+        <v>9.53</v>
+      </c>
       <c r="S169" s="7"/>
       <c r="T169" s="7" t="s">
         <v>103</v>
@@ -23963,7 +24285,9 @@
       <c r="Q170" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="R170" s="7"/>
+      <c r="R170" s="7">
+        <v>9.53</v>
+      </c>
       <c r="S170" s="7"/>
       <c r="T170" s="7" t="s">
         <v>103</v>
@@ -24088,7 +24412,9 @@
       <c r="Q171" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R171" s="7"/>
+      <c r="R171" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S171" s="7"/>
       <c r="T171" s="7" t="s">
         <v>448</v>
@@ -24215,7 +24541,9 @@
       <c r="Q172" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R172" s="7"/>
+      <c r="R172" s="7">
+        <v>3.05</v>
+      </c>
       <c r="S172" s="7"/>
       <c r="T172" s="7" t="s">
         <v>103</v>
@@ -24340,7 +24668,9 @@
       <c r="Q173" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R173" s="7"/>
+      <c r="R173" s="7">
+        <v>3.05</v>
+      </c>
       <c r="S173" s="7"/>
       <c r="T173" s="7" t="s">
         <v>103</v>
@@ -24457,7 +24787,9 @@
       <c r="Q174" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R174" s="7"/>
+      <c r="R174" s="7">
+        <v>3.05</v>
+      </c>
       <c r="S174" s="7"/>
       <c r="T174" s="7" t="s">
         <v>103</v>
@@ -24574,7 +24906,9 @@
       <c r="Q175" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R175" s="7"/>
+      <c r="R175" s="7">
+        <v>3.05</v>
+      </c>
       <c r="S175" s="7"/>
       <c r="T175" s="7" t="s">
         <v>103</v>
@@ -24699,7 +25033,9 @@
       <c r="Q176" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R176" s="7"/>
+      <c r="R176" s="7">
+        <v>3.05</v>
+      </c>
       <c r="S176" s="7"/>
       <c r="T176" s="7" t="s">
         <v>103</v>
@@ -24824,7 +25160,9 @@
       <c r="Q177" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R177" s="7"/>
+      <c r="R177" s="7">
+        <v>3.05</v>
+      </c>
       <c r="S177" s="7"/>
       <c r="T177" s="7" t="s">
         <v>103</v>
@@ -24949,7 +25287,9 @@
       <c r="Q178" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R178" s="7"/>
+      <c r="R178" s="7">
+        <v>3.05</v>
+      </c>
       <c r="S178" s="7"/>
       <c r="T178" s="7" t="s">
         <v>103</v>
@@ -25066,7 +25406,9 @@
       <c r="Q179" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R179" s="7"/>
+      <c r="R179" s="7">
+        <v>3.05</v>
+      </c>
       <c r="S179" s="7"/>
       <c r="T179" s="7" t="s">
         <v>103</v>
@@ -25191,7 +25533,9 @@
       <c r="Q180" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R180" s="7"/>
+      <c r="R180" s="7">
+        <v>3.05</v>
+      </c>
       <c r="S180" s="7"/>
       <c r="T180" s="7" t="s">
         <v>103</v>
@@ -25316,7 +25660,9 @@
       <c r="Q181" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R181" s="7"/>
+      <c r="R181" s="7">
+        <v>5.49</v>
+      </c>
       <c r="S181" s="7"/>
       <c r="T181" s="7" t="s">
         <v>448</v>
@@ -25443,7 +25789,9 @@
       <c r="Q182" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R182" s="7"/>
+      <c r="R182" s="7">
+        <v>5.49</v>
+      </c>
       <c r="S182" s="7"/>
       <c r="T182" s="7" t="s">
         <v>448</v>
@@ -25570,7 +25918,9 @@
       <c r="Q183" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R183" s="7"/>
+      <c r="R183" s="7">
+        <v>5.49</v>
+      </c>
       <c r="S183" s="7"/>
       <c r="T183" s="7" t="s">
         <v>448</v>
@@ -25697,7 +26047,9 @@
       <c r="Q184" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R184" s="7"/>
+      <c r="R184" s="7">
+        <v>5.49</v>
+      </c>
       <c r="S184" s="7"/>
       <c r="T184" s="7" t="s">
         <v>448</v>
@@ -25824,7 +26176,9 @@
       <c r="Q185" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R185" s="7"/>
+      <c r="R185" s="7">
+        <v>5.49</v>
+      </c>
       <c r="S185" s="7"/>
       <c r="T185" s="7" t="s">
         <v>448</v>
@@ -25951,7 +26305,9 @@
       <c r="Q186" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R186" s="7"/>
+      <c r="R186" s="7">
+        <v>5.49</v>
+      </c>
       <c r="S186" s="7"/>
       <c r="T186" s="7" t="s">
         <v>448</v>
@@ -26078,7 +26434,9 @@
       <c r="Q187" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R187" s="7"/>
+      <c r="R187" s="7">
+        <v>5.49</v>
+      </c>
       <c r="S187" s="7"/>
       <c r="T187" s="7" t="s">
         <v>448</v>
@@ -26205,7 +26563,9 @@
       <c r="Q188" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R188" s="7"/>
+      <c r="R188" s="7">
+        <v>5.49</v>
+      </c>
       <c r="S188" s="7"/>
       <c r="T188" s="7" t="s">
         <v>448</v>
@@ -26332,7 +26692,9 @@
       <c r="Q189" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R189" s="7"/>
+      <c r="R189" s="7">
+        <v>5.49</v>
+      </c>
       <c r="S189" s="7"/>
       <c r="T189" s="7" t="s">
         <v>448</v>
@@ -26459,7 +26821,9 @@
       <c r="Q190" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R190" s="7"/>
+      <c r="R190" s="7">
+        <v>5.49</v>
+      </c>
       <c r="S190" s="7"/>
       <c r="T190" s="7" t="s">
         <v>448</v>
@@ -26586,7 +26950,9 @@
       <c r="Q191" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R191" s="7"/>
+      <c r="R191" s="7">
+        <v>5.49</v>
+      </c>
       <c r="S191" s="7"/>
       <c r="T191" s="7" t="s">
         <v>448</v>
@@ -26713,7 +27079,9 @@
       <c r="Q192" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R192" s="7"/>
+      <c r="R192" s="7">
+        <v>5.49</v>
+      </c>
       <c r="S192" s="7"/>
       <c r="T192" s="7" t="s">
         <v>448</v>
@@ -26840,7 +27208,9 @@
       <c r="Q193" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R193" s="7"/>
+      <c r="R193" s="7">
+        <v>5.49</v>
+      </c>
       <c r="S193" s="7"/>
       <c r="T193" s="7" t="s">
         <v>448</v>
@@ -26967,7 +27337,9 @@
       <c r="Q194" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R194" s="7"/>
+      <c r="R194" s="7">
+        <v>5.49</v>
+      </c>
       <c r="S194" s="7"/>
       <c r="T194" s="7" t="s">
         <v>448</v>
@@ -27094,7 +27466,9 @@
       <c r="Q195" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R195" s="7"/>
+      <c r="R195" s="7">
+        <v>5.49</v>
+      </c>
       <c r="S195" s="7"/>
       <c r="T195" s="7" t="s">
         <v>448</v>
@@ -27221,7 +27595,9 @@
       <c r="Q196" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R196" s="7"/>
+      <c r="R196" s="7">
+        <v>5.49</v>
+      </c>
       <c r="S196" s="7"/>
       <c r="T196" s="7" t="s">
         <v>448</v>
@@ -27348,7 +27724,9 @@
       <c r="Q197" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="R197" s="7"/>
+      <c r="R197" s="7">
+        <v>5.49</v>
+      </c>
       <c r="S197" s="7"/>
       <c r="T197" s="7" t="s">
         <v>448</v>
@@ -27475,7 +27853,9 @@
       <c r="Q198" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="R198" s="7"/>
+      <c r="R198" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S198" s="7"/>
       <c r="T198" s="7" t="s">
         <v>448</v>
@@ -27600,7 +27980,9 @@
       <c r="Q199" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="R199" s="7"/>
+      <c r="R199" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S199" s="7"/>
       <c r="T199" s="7" t="s">
         <v>448</v>
@@ -27727,7 +28109,9 @@
       <c r="Q200" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="R200" s="7"/>
+      <c r="R200" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S200" s="7"/>
       <c r="T200" s="7" t="s">
         <v>448</v>
@@ -27854,7 +28238,9 @@
       <c r="Q201" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="R201" s="7"/>
+      <c r="R201" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S201" s="7"/>
       <c r="T201" s="7" t="s">
         <v>448</v>
@@ -27981,7 +28367,9 @@
       <c r="Q202" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="R202" s="7"/>
+      <c r="R202" s="7">
+        <v>3.91</v>
+      </c>
       <c r="S202" s="7"/>
       <c r="T202" s="7" t="s">
         <v>448</v>
@@ -28108,7 +28496,9 @@
       <c r="Q203" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="R203" s="7"/>
+      <c r="R203" s="7">
+        <v>6.02</v>
+      </c>
       <c r="S203" s="7"/>
       <c r="T203" s="7" t="s">
         <v>448</v>
@@ -28235,7 +28625,9 @@
       <c r="Q204" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="R204" s="7"/>
+      <c r="R204" s="7">
+        <v>6.02</v>
+      </c>
       <c r="S204" s="7"/>
       <c r="T204" s="7" t="s">
         <v>448</v>
@@ -28362,7 +28754,9 @@
       <c r="Q205" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="R205" s="7"/>
+      <c r="R205" s="7">
+        <v>6.02</v>
+      </c>
       <c r="S205" s="7"/>
       <c r="T205" s="7" t="s">
         <v>448</v>
@@ -28489,7 +28883,9 @@
       <c r="Q206" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="R206" s="7"/>
+      <c r="R206" s="7">
+        <v>6.02</v>
+      </c>
       <c r="S206" s="7"/>
       <c r="T206" s="7" t="s">
         <v>448</v>
@@ -28616,7 +29012,9 @@
       <c r="Q207" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="R207" s="7"/>
+      <c r="R207" s="7">
+        <v>6.02</v>
+      </c>
       <c r="S207" s="7"/>
       <c r="T207" s="7" t="s">
         <v>448</v>
@@ -28733,7 +29131,9 @@
       <c r="Q208" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="R208" s="7"/>
+      <c r="R208" s="7">
+        <v>6.02</v>
+      </c>
       <c r="S208" s="7"/>
       <c r="T208" s="7" t="s">
         <v>448</v>
@@ -28860,7 +29260,9 @@
       <c r="Q209" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="R209" s="7"/>
+      <c r="R209" s="7">
+        <v>6.02</v>
+      </c>
       <c r="S209" s="7"/>
       <c r="T209" s="7" t="s">
         <v>448</v>
@@ -28987,7 +29389,9 @@
       <c r="Q210" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="R210" s="7"/>
+      <c r="R210" s="7">
+        <v>6.02</v>
+      </c>
       <c r="S210" s="7"/>
       <c r="T210" s="7" t="s">
         <v>448</v>
@@ -29114,7 +29518,9 @@
       <c r="Q211" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="R211" s="7"/>
+      <c r="R211" s="7">
+        <v>6.02</v>
+      </c>
       <c r="S211" s="7"/>
       <c r="T211" s="7" t="s">
         <v>448</v>
@@ -29239,7 +29645,9 @@
       <c r="Q212" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="R212" s="7"/>
+      <c r="R212" s="7">
+        <v>6.02</v>
+      </c>
       <c r="S212" s="7"/>
       <c r="T212" s="7" t="s">
         <v>448</v>
@@ -29366,7 +29774,9 @@
       <c r="Q213" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="R213" s="7"/>
+      <c r="R213" s="7">
+        <v>6.02</v>
+      </c>
       <c r="S213" s="7"/>
       <c r="T213" s="7" t="s">
         <v>448</v>
@@ -29493,7 +29903,9 @@
       <c r="Q214" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R214" s="7"/>
+      <c r="R214" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S214" s="7"/>
       <c r="T214" s="7" t="s">
         <v>103</v>
@@ -29618,7 +30030,9 @@
       <c r="Q215" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R215" s="7"/>
+      <c r="R215" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S215" s="7"/>
       <c r="T215" s="7" t="s">
         <v>448</v>
@@ -29745,7 +30159,9 @@
       <c r="Q216" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R216" s="7"/>
+      <c r="R216" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S216" s="7"/>
       <c r="T216" s="7" t="s">
         <v>448</v>
@@ -29862,7 +30278,9 @@
       <c r="Q217" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R217" s="7"/>
+      <c r="R217" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S217" s="7"/>
       <c r="T217" s="7" t="s">
         <v>448</v>
@@ -29989,7 +30407,9 @@
       <c r="Q218" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R218" s="7"/>
+      <c r="R218" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S218" s="7"/>
       <c r="T218" s="7" t="s">
         <v>448</v>
@@ -30116,7 +30536,9 @@
       <c r="Q219" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R219" s="7"/>
+      <c r="R219" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S219" s="7"/>
       <c r="T219" s="7" t="s">
         <v>448</v>
@@ -30243,7 +30665,9 @@
       <c r="Q220" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R220" s="7"/>
+      <c r="R220" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S220" s="7"/>
       <c r="T220" s="7" t="s">
         <v>448</v>
@@ -30370,7 +30794,9 @@
       <c r="Q221" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R221" s="7"/>
+      <c r="R221" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S221" s="7"/>
       <c r="T221" s="7" t="s">
         <v>448</v>
@@ -30497,7 +30923,9 @@
       <c r="Q222" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R222" s="7"/>
+      <c r="R222" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S222" s="7"/>
       <c r="T222" s="7" t="s">
         <v>448</v>
@@ -30614,7 +31042,9 @@
       <c r="Q223" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R223" s="7"/>
+      <c r="R223" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S223" s="7"/>
       <c r="T223" s="7" t="s">
         <v>448</v>
@@ -30741,7 +31171,9 @@
       <c r="Q224" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R224" s="7"/>
+      <c r="R224" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S224" s="7"/>
       <c r="T224" s="7" t="s">
         <v>448</v>
@@ -30868,7 +31300,9 @@
       <c r="Q225" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R225" s="7"/>
+      <c r="R225" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S225" s="7"/>
       <c r="T225" s="7" t="s">
         <v>448</v>
@@ -30995,7 +31429,9 @@
       <c r="Q226" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R226" s="7"/>
+      <c r="R226" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S226" s="7"/>
       <c r="T226" s="7" t="s">
         <v>448</v>
@@ -31122,7 +31558,9 @@
       <c r="Q227" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R227" s="7"/>
+      <c r="R227" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S227" s="7"/>
       <c r="T227" s="7" t="s">
         <v>448</v>
@@ -31239,7 +31677,9 @@
       <c r="Q228" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R228" s="7"/>
+      <c r="R228" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S228" s="7"/>
       <c r="T228" s="7" t="s">
         <v>448</v>
@@ -31366,7 +31806,9 @@
       <c r="Q229" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R229" s="7"/>
+      <c r="R229" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S229" s="7"/>
       <c r="T229" s="7" t="s">
         <v>448</v>
@@ -31483,7 +31925,9 @@
       <c r="Q230" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R230" s="7"/>
+      <c r="R230" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S230" s="7"/>
       <c r="T230" s="7" t="s">
         <v>448</v>
@@ -31600,7 +32044,9 @@
       <c r="Q231" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R231" s="7"/>
+      <c r="R231" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S231" s="7"/>
       <c r="T231" s="7" t="s">
         <v>448</v>
@@ -31727,7 +32173,9 @@
       <c r="Q232" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R232" s="7"/>
+      <c r="R232" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S232" s="7"/>
       <c r="T232" s="7" t="s">
         <v>448</v>
@@ -31854,7 +32302,9 @@
       <c r="Q233" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R233" s="7"/>
+      <c r="R233" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S233" s="7"/>
       <c r="T233" s="7" t="s">
         <v>448</v>
@@ -31981,7 +32431,9 @@
       <c r="Q234" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R234" s="7"/>
+      <c r="R234" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S234" s="7"/>
       <c r="T234" s="7" t="s">
         <v>103</v>
@@ -32106,7 +32558,9 @@
       <c r="Q235" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R235" s="7"/>
+      <c r="R235" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S235" s="7"/>
       <c r="T235" s="7" t="s">
         <v>103</v>
@@ -32231,7 +32685,9 @@
       <c r="Q236" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R236" s="7"/>
+      <c r="R236" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S236" s="7"/>
       <c r="T236" s="7" t="s">
         <v>448</v>
@@ -32358,7 +32814,9 @@
       <c r="Q237" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R237" s="7"/>
+      <c r="R237" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S237" s="7"/>
       <c r="T237" s="7" t="s">
         <v>448</v>
@@ -32485,7 +32943,9 @@
       <c r="Q238" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R238" s="7"/>
+      <c r="R238" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S238" s="7"/>
       <c r="T238" s="7" t="s">
         <v>448</v>
@@ -32612,7 +33072,9 @@
       <c r="Q239" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R239" s="7"/>
+      <c r="R239" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S239" s="7"/>
       <c r="T239" s="7" t="s">
         <v>448</v>
@@ -32729,7 +33191,9 @@
       <c r="Q240" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R240" s="7"/>
+      <c r="R240" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S240" s="7"/>
       <c r="T240" s="7" t="s">
         <v>448</v>
@@ -32856,7 +33320,9 @@
       <c r="Q241" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R241" s="7"/>
+      <c r="R241" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S241" s="7"/>
       <c r="T241" s="7" t="s">
         <v>448</v>
@@ -32983,7 +33449,9 @@
       <c r="Q242" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R242" s="7"/>
+      <c r="R242" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S242" s="7"/>
       <c r="T242" s="7" t="s">
         <v>448</v>
@@ -33100,7 +33568,9 @@
       <c r="Q243" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R243" s="7"/>
+      <c r="R243" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S243" s="7"/>
       <c r="T243" s="7" t="s">
         <v>103</v>
@@ -33225,7 +33695,9 @@
       <c r="Q244" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R244" s="7"/>
+      <c r="R244" s="7">
+        <v>10.97</v>
+      </c>
       <c r="S244" s="7"/>
       <c r="T244" s="7" t="s">
         <v>448</v>
@@ -33342,7 +33814,9 @@
       <c r="Q245" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R245" s="7"/>
+      <c r="R245" s="7">
+        <v>10.97</v>
+      </c>
       <c r="S245" s="7"/>
       <c r="T245" s="7" t="s">
         <v>448</v>
@@ -33469,7 +33943,9 @@
       <c r="Q246" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R246" s="7"/>
+      <c r="R246" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S246" s="7"/>
       <c r="T246" s="7" t="s">
         <v>448</v>
@@ -33596,7 +34072,9 @@
       <c r="Q247" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R247" s="7"/>
+      <c r="R247" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S247" s="7"/>
       <c r="T247" s="7" t="s">
         <v>448</v>
@@ -33723,7 +34201,9 @@
       <c r="Q248" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R248" s="7"/>
+      <c r="R248" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S248" s="7"/>
       <c r="T248" s="7" t="s">
         <v>448</v>
@@ -33850,7 +34330,9 @@
       <c r="Q249" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R249" s="7"/>
+      <c r="R249" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S249" s="7"/>
       <c r="T249" s="7" t="s">
         <v>448</v>
@@ -33977,7 +34459,9 @@
       <c r="Q250" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R250" s="7"/>
+      <c r="R250" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S250" s="7"/>
       <c r="T250" s="7" t="s">
         <v>448</v>
@@ -34104,7 +34588,9 @@
       <c r="Q251" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R251" s="7"/>
+      <c r="R251" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S251" s="7"/>
       <c r="T251" s="7" t="s">
         <v>448</v>
@@ -34231,7 +34717,9 @@
       <c r="Q252" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R252" s="7"/>
+      <c r="R252" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S252" s="7"/>
       <c r="T252" s="7" t="s">
         <v>448</v>
@@ -34358,7 +34846,9 @@
       <c r="Q253" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R253" s="7"/>
+      <c r="R253" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S253" s="7"/>
       <c r="T253" s="7" t="s">
         <v>448</v>
@@ -34485,7 +34975,9 @@
       <c r="Q254" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R254" s="7"/>
+      <c r="R254" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S254" s="7"/>
       <c r="T254" s="7" t="s">
         <v>448</v>
@@ -34612,7 +35104,9 @@
       <c r="Q255" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R255" s="7"/>
+      <c r="R255" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S255" s="7"/>
       <c r="T255" s="7" t="s">
         <v>448</v>
@@ -34739,7 +35233,9 @@
       <c r="Q256" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R256" s="7"/>
+      <c r="R256" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S256" s="7"/>
       <c r="T256" s="7" t="s">
         <v>448</v>
@@ -34866,7 +35362,9 @@
       <c r="Q257" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R257" s="7"/>
+      <c r="R257" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S257" s="7"/>
       <c r="T257" s="7" t="s">
         <v>448</v>
@@ -34993,7 +35491,9 @@
       <c r="Q258" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R258" s="7"/>
+      <c r="R258" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S258" s="7"/>
       <c r="T258" s="7" t="s">
         <v>448</v>
@@ -35120,7 +35620,9 @@
       <c r="Q259" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R259" s="7"/>
+      <c r="R259" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S259" s="7"/>
       <c r="T259" s="7" t="s">
         <v>448</v>
@@ -35247,7 +35749,9 @@
       <c r="Q260" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="R260" s="7"/>
+      <c r="R260" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S260" s="7"/>
       <c r="T260" s="7" t="s">
         <v>448</v>
@@ -35374,7 +35878,9 @@
       <c r="Q261" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="R261" s="7"/>
+      <c r="R261" s="7">
+        <v>3.76</v>
+      </c>
       <c r="S261" s="7"/>
       <c r="T261" s="7" t="s">
         <v>103</v>
@@ -35499,7 +36005,9 @@
       <c r="Q262" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="R262" s="7"/>
+      <c r="R262" s="7">
+        <v>3.76</v>
+      </c>
       <c r="S262" s="7"/>
       <c r="T262" s="7" t="s">
         <v>103</v>
@@ -35624,7 +36132,9 @@
       <c r="Q263" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="R263" s="7"/>
+      <c r="R263" s="7">
+        <v>3.76</v>
+      </c>
       <c r="S263" s="7"/>
       <c r="T263" s="7" t="s">
         <v>103</v>
@@ -35749,7 +36259,9 @@
       <c r="Q264" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="R264" s="7"/>
+      <c r="R264" s="7">
+        <v>8.18</v>
+      </c>
       <c r="S264" s="7"/>
       <c r="T264" s="7" t="s">
         <v>448</v>
@@ -35876,7 +36388,9 @@
       <c r="Q265" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="R265" s="7"/>
+      <c r="R265" s="7">
+        <v>8.18</v>
+      </c>
       <c r="S265" s="7"/>
       <c r="T265" s="7" t="s">
         <v>448</v>
@@ -36003,7 +36517,9 @@
       <c r="Q266" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="R266" s="7"/>
+      <c r="R266" s="7">
+        <v>8.18</v>
+      </c>
       <c r="S266" s="7"/>
       <c r="T266" s="7" t="s">
         <v>448</v>
@@ -36130,7 +36646,9 @@
       <c r="Q267" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="R267" s="7"/>
+      <c r="R267" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S267" s="7"/>
       <c r="T267" s="7" t="s">
         <v>448</v>
@@ -36257,7 +36775,9 @@
       <c r="Q268" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="R268" s="7"/>
+      <c r="R268" s="7">
+        <v>7.11</v>
+      </c>
       <c r="S268" s="7"/>
       <c r="T268" s="7" t="s">
         <v>448</v>
@@ -36384,7 +36904,9 @@
       <c r="Q269" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="R269" s="7"/>
+      <c r="R269" s="7">
+        <v>8.18</v>
+      </c>
       <c r="S269" s="7"/>
       <c r="T269" s="7" t="s">
         <v>448</v>
@@ -36511,7 +37033,9 @@
       <c r="Q270" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="R270" s="7"/>
+      <c r="R270" s="7">
+        <v>3.73</v>
+      </c>
       <c r="S270" s="7"/>
       <c r="T270" s="7" t="s">
         <v>448</v>
@@ -36638,7 +37162,9 @@
       <c r="Q271" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="R271" s="7"/>
+      <c r="R271" s="7">
+        <v>3.73</v>
+      </c>
       <c r="S271" s="7"/>
       <c r="T271" s="7" t="s">
         <v>448</v>

</xml_diff>

<commit_message>
Corrige Total_Juntas e Total_Juntas_Pipe pelo Mapa de Juntas
- Total_Juntas recebe o total de juntas do spool e Total_Juntas_Pipe as
  juntas Pipe Shop, contados no Mapa de Juntas (repetidas contam uma vez).
- Documento passa a manter a folha (FL1/FL2): eram tratados como o mesmo
  documento e o spool 002 da FL2 herdava juntas/datas da FL1.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jhm2rrJCBVkJYZMmi4pDeT
</commit_message>
<xml_diff>
--- a/saida/Situacao_Geral_de_Spools_ATUALIZADO.xlsx
+++ b/saida/Situacao_Geral_de_Spools_ATUALIZADO.xlsx
@@ -3853,7 +3853,7 @@
         <v>2</v>
       </c>
       <c r="AE10" s="36">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AF10" s="34"/>
       <c r="AG10" s="7"/>
@@ -5153,7 +5153,7 @@
         <v>6</v>
       </c>
       <c r="AE20" s="36">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AF20" s="34"/>
       <c r="AG20" s="7"/>
@@ -5798,7 +5798,7 @@
         <v>6</v>
       </c>
       <c r="AE25" s="36">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AF25" s="34"/>
       <c r="AG25" s="7"/>
@@ -5929,7 +5929,7 @@
         <v>6</v>
       </c>
       <c r="AE26" s="36">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AF26" s="34"/>
       <c r="AG26" s="7"/>
@@ -6423,7 +6423,7 @@
         <v>8</v>
       </c>
       <c r="AE30" s="36">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AF30" s="34"/>
       <c r="AG30" s="7"/>
@@ -6675,7 +6675,7 @@
         <v>5</v>
       </c>
       <c r="AE32" s="36">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AF32" s="34"/>
       <c r="AG32" s="7"/>
@@ -6806,7 +6806,7 @@
         <v>10</v>
       </c>
       <c r="AE33" s="36">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AF33" s="34"/>
       <c r="AG33" s="7"/>
@@ -7068,7 +7068,7 @@
         <v>2</v>
       </c>
       <c r="AE35" s="36">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AF35" s="34"/>
       <c r="AG35" s="7"/>
@@ -8501,7 +8501,7 @@
         <v>3</v>
       </c>
       <c r="AE46" s="36">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AF46" s="34"/>
       <c r="AG46" s="7"/>
@@ -8894,7 +8894,7 @@
         <v>3</v>
       </c>
       <c r="AE49" s="36">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AF49" s="34"/>
       <c r="AG49" s="7"/>
@@ -9942,7 +9942,7 @@
         <v>10</v>
       </c>
       <c r="AE57" s="36">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="AF57" s="34"/>
       <c r="AG57" s="7"/>
@@ -10716,7 +10716,7 @@
         <v>9</v>
       </c>
       <c r="AE63" s="36">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="AF63" s="34"/>
       <c r="AG63" s="7"/>
@@ -10978,7 +10978,7 @@
         <v>7</v>
       </c>
       <c r="AE65" s="36">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AF65" s="34"/>
       <c r="AG65" s="7"/>
@@ -12024,7 +12024,7 @@
         <v>1</v>
       </c>
       <c r="AE73" s="36">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AF73" s="34"/>
       <c r="AG73" s="7"/>
@@ -12286,7 +12286,7 @@
         <v>1</v>
       </c>
       <c r="AE75" s="36">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AF75" s="34"/>
       <c r="AG75" s="7"/>
@@ -12538,7 +12538,7 @@
         <v>1</v>
       </c>
       <c r="AE77" s="36">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AF77" s="34"/>
       <c r="AG77" s="7"/>
@@ -12931,7 +12931,7 @@
         <v>15</v>
       </c>
       <c r="AE80" s="36">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="AF80" s="34"/>
       <c r="AG80" s="7"/>
@@ -13183,7 +13183,7 @@
         <v>4</v>
       </c>
       <c r="AE82" s="36">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AF82" s="34"/>
       <c r="AG82" s="7"/>
@@ -13304,7 +13304,7 @@
         <v>12</v>
       </c>
       <c r="AE83" s="36">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AF83" s="34"/>
       <c r="AG83" s="7"/>
@@ -13546,7 +13546,7 @@
         <v>4</v>
       </c>
       <c r="AE85" s="36">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="AF85" s="34"/>
       <c r="AG85" s="7"/>
@@ -13667,7 +13667,7 @@
         <v>4</v>
       </c>
       <c r="AE86" s="36">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="AF86" s="34"/>
       <c r="AG86" s="7"/>
@@ -14170,7 +14170,7 @@
       <c r="AB90" s="7"/>
       <c r="AC90" s="7"/>
       <c r="AD90" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AE90" s="36">
         <v>3</v>
@@ -14297,10 +14297,10 @@
       <c r="AB91" s="7"/>
       <c r="AC91" s="7"/>
       <c r="AD91" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AE91" s="36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AF91" s="34"/>
       <c r="AG91" s="7"/>
@@ -14424,7 +14424,7 @@
       <c r="AB92" s="7"/>
       <c r="AC92" s="7"/>
       <c r="AD92" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AE92" s="36">
         <v>3</v>
@@ -14551,10 +14551,10 @@
       <c r="AB93" s="7"/>
       <c r="AC93" s="7"/>
       <c r="AD93" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AE93" s="36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AF93" s="34"/>
       <c r="AG93" s="7"/>
@@ -14678,7 +14678,7 @@
       <c r="AB94" s="7"/>
       <c r="AC94" s="7"/>
       <c r="AD94" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AE94" s="36">
         <v>3</v>
@@ -14805,10 +14805,10 @@
       <c r="AB95" s="7"/>
       <c r="AC95" s="7"/>
       <c r="AD95" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AE95" s="36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AF95" s="34"/>
       <c r="AG95" s="7"/>
@@ -14932,7 +14932,7 @@
       <c r="AB96" s="7"/>
       <c r="AC96" s="7"/>
       <c r="AD96" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AE96" s="36">
         <v>3</v>
@@ -15059,10 +15059,10 @@
       <c r="AB97" s="7"/>
       <c r="AC97" s="7"/>
       <c r="AD97" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AE97" s="36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AF97" s="34"/>
       <c r="AG97" s="7"/>
@@ -15186,7 +15186,7 @@
       <c r="AB98" s="7"/>
       <c r="AC98" s="7"/>
       <c r="AD98" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AE98" s="36">
         <v>3</v>
@@ -15313,10 +15313,10 @@
       <c r="AB99" s="7"/>
       <c r="AC99" s="7"/>
       <c r="AD99" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AE99" s="36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AF99" s="34"/>
       <c r="AG99" s="7"/>
@@ -15440,7 +15440,7 @@
       <c r="AB100" s="7"/>
       <c r="AC100" s="7"/>
       <c r="AD100" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AE100" s="36">
         <v>2</v>
@@ -15567,10 +15567,10 @@
       <c r="AB101" s="7"/>
       <c r="AC101" s="7"/>
       <c r="AD101" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AE101" s="36">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AF101" s="34"/>
       <c r="AG101" s="7"/>
@@ -15694,7 +15694,7 @@
       <c r="AB102" s="7"/>
       <c r="AC102" s="7"/>
       <c r="AD102" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AE102" s="36">
         <v>3</v>
@@ -15821,10 +15821,10 @@
       <c r="AB103" s="7"/>
       <c r="AC103" s="7"/>
       <c r="AD103" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AE103" s="36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AF103" s="34"/>
       <c r="AG103" s="7"/>
@@ -15948,7 +15948,7 @@
       <c r="AB104" s="7"/>
       <c r="AC104" s="7"/>
       <c r="AD104" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AE104" s="36">
         <v>2</v>
@@ -16067,10 +16067,10 @@
       <c r="AB105" s="7"/>
       <c r="AC105" s="7"/>
       <c r="AD105" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AE105" s="36">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AF105" s="34"/>
       <c r="AG105" s="7"/>
@@ -16194,7 +16194,7 @@
       <c r="AB106" s="7"/>
       <c r="AC106" s="7"/>
       <c r="AD106" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AE106" s="36">
         <v>2</v>
@@ -16321,10 +16321,10 @@
       <c r="AB107" s="7"/>
       <c r="AC107" s="7"/>
       <c r="AD107" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AE107" s="36">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AF107" s="34"/>
       <c r="AG107" s="7"/>
@@ -16448,7 +16448,7 @@
       <c r="AB108" s="7"/>
       <c r="AC108" s="7"/>
       <c r="AD108" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AE108" s="36">
         <v>2</v>
@@ -16567,10 +16567,10 @@
       <c r="AB109" s="7"/>
       <c r="AC109" s="7"/>
       <c r="AD109" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AE109" s="36">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AF109" s="34"/>
       <c r="AG109" s="7"/>
@@ -16694,7 +16694,7 @@
       <c r="AB110" s="7"/>
       <c r="AC110" s="7"/>
       <c r="AD110" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AE110" s="36">
         <v>2</v>
@@ -16821,10 +16821,10 @@
       <c r="AB111" s="7"/>
       <c r="AC111" s="7"/>
       <c r="AD111" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AE111" s="36">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AF111" s="34"/>
       <c r="AG111" s="7"/>
@@ -16948,7 +16948,7 @@
       <c r="AB112" s="7"/>
       <c r="AC112" s="7"/>
       <c r="AD112" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AE112" s="36">
         <v>2</v>
@@ -17067,10 +17067,10 @@
       <c r="AB113" s="7"/>
       <c r="AC113" s="7"/>
       <c r="AD113" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AE113" s="36">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AF113" s="34"/>
       <c r="AG113" s="7"/>
@@ -17194,7 +17194,7 @@
       <c r="AB114" s="7"/>
       <c r="AC114" s="7"/>
       <c r="AD114" s="7">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AE114" s="36">
         <v>6</v>
@@ -17313,7 +17313,7 @@
       <c r="AB115" s="7"/>
       <c r="AC115" s="7"/>
       <c r="AD115" s="7">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AE115" s="36">
         <v>4</v>
@@ -17443,7 +17443,7 @@
         <v>4</v>
       </c>
       <c r="AE116" s="36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF116" s="34"/>
       <c r="AG116" s="7"/>
@@ -17559,7 +17559,7 @@
       <c r="AB117" s="7"/>
       <c r="AC117" s="7"/>
       <c r="AD117" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AE117" s="36">
         <v>0</v>
@@ -17678,7 +17678,7 @@
       <c r="AB118" s="7"/>
       <c r="AC118" s="7"/>
       <c r="AD118" s="7">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AE118" s="36">
         <v>5</v>
@@ -17805,7 +17805,7 @@
       <c r="AB119" s="7"/>
       <c r="AC119" s="7"/>
       <c r="AD119" s="7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AE119" s="36">
         <v>6</v>
@@ -17932,7 +17932,7 @@
       <c r="AB120" s="7"/>
       <c r="AC120" s="7"/>
       <c r="AD120" s="7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AE120" s="36">
         <v>7</v>
@@ -18061,10 +18061,10 @@
       <c r="AB121" s="7"/>
       <c r="AC121" s="7"/>
       <c r="AD121" s="7">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AE121" s="36">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AF121" s="34"/>
       <c r="AG121" s="7"/>
@@ -18180,10 +18180,10 @@
       <c r="AB122" s="7"/>
       <c r="AC122" s="7"/>
       <c r="AD122" s="7">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AE122" s="36">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AF122" s="34"/>
       <c r="AG122" s="7"/>
@@ -18299,10 +18299,10 @@
       <c r="AB123" s="7"/>
       <c r="AC123" s="7"/>
       <c r="AD123" s="7">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="AE123" s="36">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="AF123" s="34"/>
       <c r="AG123" s="7"/>
@@ -18428,10 +18428,10 @@
       <c r="AB124" s="7"/>
       <c r="AC124" s="7"/>
       <c r="AD124" s="7">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AE124" s="36">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AF124" s="34"/>
       <c r="AG124" s="7"/>
@@ -18557,7 +18557,7 @@
       <c r="AB125" s="7"/>
       <c r="AC125" s="7"/>
       <c r="AD125" s="7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AE125" s="36">
         <v>4</v>
@@ -18811,7 +18811,7 @@
       <c r="AB127" s="7"/>
       <c r="AC127" s="7"/>
       <c r="AD127" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AE127" s="36">
         <v>1</v>
@@ -18938,7 +18938,7 @@
       <c r="AB128" s="7"/>
       <c r="AC128" s="7"/>
       <c r="AD128" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE128" s="36">
         <v>1</v>
@@ -19712,7 +19712,7 @@
       <c r="AB134" s="7"/>
       <c r="AC134" s="7"/>
       <c r="AD134" s="7">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AE134" s="36">
         <v>4</v>
@@ -19841,7 +19841,7 @@
       <c r="AB135" s="7"/>
       <c r="AC135" s="7"/>
       <c r="AD135" s="7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AE135" s="36">
         <v>4</v>
@@ -20099,7 +20099,7 @@
       <c r="AB137" s="7"/>
       <c r="AC137" s="7"/>
       <c r="AD137" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AE137" s="36">
         <v>1</v>
@@ -20228,7 +20228,7 @@
       <c r="AB138" s="7"/>
       <c r="AC138" s="7"/>
       <c r="AD138" s="7">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AE138" s="36">
         <v>6</v>
@@ -20360,7 +20360,7 @@
         <v>6</v>
       </c>
       <c r="AE139" s="36">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AF139" s="34"/>
       <c r="AG139" s="7"/>
@@ -20486,10 +20486,10 @@
       <c r="AB140" s="7"/>
       <c r="AC140" s="7"/>
       <c r="AD140" s="7">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AE140" s="36">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AF140" s="34"/>
       <c r="AG140" s="7"/>
@@ -20615,7 +20615,7 @@
       <c r="AB141" s="7"/>
       <c r="AC141" s="7"/>
       <c r="AD141" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AE141" s="36">
         <v>3</v>
@@ -20744,10 +20744,10 @@
       <c r="AB142" s="7"/>
       <c r="AC142" s="7"/>
       <c r="AD142" s="7">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AE142" s="36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AF142" s="34"/>
       <c r="AG142" s="7"/>
@@ -20871,7 +20871,7 @@
       <c r="AB143" s="7"/>
       <c r="AC143" s="7"/>
       <c r="AD143" s="7">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AE143" s="36">
         <v>2</v>
@@ -21000,10 +21000,10 @@
       <c r="AB144" s="7"/>
       <c r="AC144" s="7"/>
       <c r="AD144" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AE144" s="36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AF144" s="34"/>
       <c r="AG144" s="7"/>
@@ -21129,10 +21129,10 @@
       <c r="AB145" s="7"/>
       <c r="AC145" s="7"/>
       <c r="AD145" s="7">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="AE145" s="36">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="AF145" s="34"/>
       <c r="AG145" s="7"/>
@@ -21258,7 +21258,7 @@
       <c r="AB146" s="7"/>
       <c r="AC146" s="7"/>
       <c r="AD146" s="7">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="AE146" s="36">
         <v>12</v>
@@ -21385,7 +21385,7 @@
       <c r="AB147" s="7"/>
       <c r="AC147" s="7"/>
       <c r="AD147" s="7">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AE147" s="36">
         <v>0</v>
@@ -21504,10 +21504,10 @@
       <c r="AB148" s="7"/>
       <c r="AC148" s="7"/>
       <c r="AD148" s="7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AE148" s="36">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AF148" s="34"/>
       <c r="AG148" s="7"/>
@@ -21633,10 +21633,10 @@
       <c r="AB149" s="7"/>
       <c r="AC149" s="7"/>
       <c r="AD149" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AE149" s="36">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AF149" s="34"/>
       <c r="AG149" s="7"/>
@@ -21765,7 +21765,7 @@
         <v>4</v>
       </c>
       <c r="AE150" s="36">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AF150" s="34"/>
       <c r="AG150" s="7"/>
@@ -22020,10 +22020,10 @@
       <c r="AB152" s="7"/>
       <c r="AC152" s="7"/>
       <c r="AD152" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AE152" s="36">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AF152" s="34"/>
       <c r="AG152" s="7"/>
@@ -22149,10 +22149,10 @@
       <c r="AB153" s="7"/>
       <c r="AC153" s="7"/>
       <c r="AD153" s="7">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AE153" s="36">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AF153" s="34"/>
       <c r="AG153" s="7"/>
@@ -22278,10 +22278,10 @@
       <c r="AB154" s="7"/>
       <c r="AC154" s="7"/>
       <c r="AD154" s="7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AE154" s="36">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AF154" s="34"/>
       <c r="AG154" s="7"/>
@@ -22407,10 +22407,10 @@
       <c r="AB155" s="7"/>
       <c r="AC155" s="7"/>
       <c r="AD155" s="7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AE155" s="36">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AF155" s="34"/>
       <c r="AG155" s="7"/>
@@ -22526,7 +22526,7 @@
       <c r="AB156" s="7"/>
       <c r="AC156" s="7"/>
       <c r="AD156" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE156" s="36">
         <v>2</v>
@@ -22655,7 +22655,7 @@
       <c r="AB157" s="7"/>
       <c r="AC157" s="7"/>
       <c r="AD157" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AE157" s="36">
         <v>4</v>
@@ -22913,10 +22913,10 @@
       <c r="AB159" s="7"/>
       <c r="AC159" s="7"/>
       <c r="AD159" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AE159" s="36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AF159" s="34"/>
       <c r="AG159" s="7"/>
@@ -23042,7 +23042,7 @@
       <c r="AB160" s="7"/>
       <c r="AC160" s="7"/>
       <c r="AD160" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE160" s="36">
         <v>3</v>
@@ -23171,10 +23171,10 @@
       <c r="AB161" s="7"/>
       <c r="AC161" s="7"/>
       <c r="AD161" s="7">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AE161" s="36">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AF161" s="34"/>
       <c r="AG161" s="7"/>
@@ -23300,10 +23300,10 @@
       <c r="AB162" s="7"/>
       <c r="AC162" s="7"/>
       <c r="AD162" s="7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AE162" s="36">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AF162" s="34"/>
       <c r="AG162" s="7"/>
@@ -23419,7 +23419,7 @@
       <c r="AB163" s="7"/>
       <c r="AC163" s="7"/>
       <c r="AD163" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AE163" s="36">
         <v>4</v>
@@ -23548,7 +23548,7 @@
       <c r="AB164" s="7"/>
       <c r="AC164" s="7"/>
       <c r="AD164" s="7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AE164" s="36">
         <v>3</v>
@@ -23675,7 +23675,7 @@
       <c r="AB165" s="7"/>
       <c r="AC165" s="7"/>
       <c r="AD165" s="7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AE165" s="36">
         <v>3</v>
@@ -23802,10 +23802,10 @@
       <c r="AB166" s="7"/>
       <c r="AC166" s="7"/>
       <c r="AD166" s="7">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="AE166" s="36">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AF166" s="34"/>
       <c r="AG166" s="7"/>
@@ -23929,7 +23929,7 @@
       <c r="AB167" s="7"/>
       <c r="AC167" s="7"/>
       <c r="AD167" s="7">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AE167" s="36">
         <v>3</v>
@@ -24056,10 +24056,10 @@
       <c r="AB168" s="7"/>
       <c r="AC168" s="7"/>
       <c r="AD168" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AE168" s="36">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AF168" s="34"/>
       <c r="AG168" s="7"/>
@@ -24186,7 +24186,7 @@
         <v>2</v>
       </c>
       <c r="AE169" s="36">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AF169" s="34"/>
       <c r="AG169" s="7"/>
@@ -24310,10 +24310,10 @@
       <c r="AB170" s="7"/>
       <c r="AC170" s="7"/>
       <c r="AD170" s="7">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AE170" s="36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AF170" s="34"/>
       <c r="AG170" s="7"/>
@@ -24437,7 +24437,7 @@
       <c r="AB171" s="7"/>
       <c r="AC171" s="7"/>
       <c r="AD171" s="7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AE171" s="36">
         <v>3</v>
@@ -24566,7 +24566,7 @@
       <c r="AB172" s="7"/>
       <c r="AC172" s="7"/>
       <c r="AD172" s="7">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AE172" s="36">
         <v>6</v>
@@ -24693,7 +24693,7 @@
       <c r="AB173" s="7"/>
       <c r="AC173" s="7"/>
       <c r="AD173" s="7">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AE173" s="36">
         <v>3</v>
@@ -24812,7 +24812,7 @@
       <c r="AB174" s="7"/>
       <c r="AC174" s="7"/>
       <c r="AD174" s="7">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AE174" s="36">
         <v>5</v>
@@ -24931,7 +24931,7 @@
       <c r="AB175" s="7"/>
       <c r="AC175" s="7"/>
       <c r="AD175" s="7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AE175" s="36">
         <v>1</v>
@@ -25058,7 +25058,7 @@
       <c r="AB176" s="7"/>
       <c r="AC176" s="7"/>
       <c r="AD176" s="7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AE176" s="36">
         <v>4</v>
@@ -25185,7 +25185,7 @@
       <c r="AB177" s="7"/>
       <c r="AC177" s="7"/>
       <c r="AD177" s="7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AE177" s="36">
         <v>5</v>
@@ -25312,7 +25312,7 @@
       <c r="AB178" s="7"/>
       <c r="AC178" s="7"/>
       <c r="AD178" s="7">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AE178" s="36">
         <v>0</v>
@@ -25431,7 +25431,7 @@
       <c r="AB179" s="7"/>
       <c r="AC179" s="7"/>
       <c r="AD179" s="7">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="AE179" s="36">
         <v>13</v>
@@ -25558,7 +25558,7 @@
       <c r="AB180" s="7"/>
       <c r="AC180" s="7"/>
       <c r="AD180" s="7">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AE180" s="36">
         <v>14</v>
@@ -25685,7 +25685,7 @@
       <c r="AB181" s="7"/>
       <c r="AC181" s="7"/>
       <c r="AD181" s="7">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AE181" s="36">
         <v>1</v>
@@ -25814,7 +25814,7 @@
       <c r="AB182" s="7"/>
       <c r="AC182" s="7"/>
       <c r="AD182" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE182" s="36">
         <v>1</v>
@@ -25943,10 +25943,10 @@
       <c r="AB183" s="7"/>
       <c r="AC183" s="7"/>
       <c r="AD183" s="7">
+        <v>3</v>
+      </c>
+      <c r="AE183" s="36">
         <v>2</v>
-      </c>
-      <c r="AE183" s="36">
-        <v>1</v>
       </c>
       <c r="AF183" s="34"/>
       <c r="AG183" s="7"/>
@@ -26072,10 +26072,10 @@
       <c r="AB184" s="7"/>
       <c r="AC184" s="7"/>
       <c r="AD184" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AE184" s="36">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF184" s="34"/>
       <c r="AG184" s="7"/>
@@ -26201,7 +26201,7 @@
       <c r="AB185" s="7"/>
       <c r="AC185" s="7"/>
       <c r="AD185" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AE185" s="36">
         <v>4</v>
@@ -26459,10 +26459,10 @@
       <c r="AB187" s="7"/>
       <c r="AC187" s="7"/>
       <c r="AD187" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AE187" s="36">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AF187" s="34"/>
       <c r="AG187" s="7"/>
@@ -26588,7 +26588,7 @@
       <c r="AB188" s="7"/>
       <c r="AC188" s="7"/>
       <c r="AD188" s="7">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AE188" s="36">
         <v>5</v>
@@ -26717,10 +26717,10 @@
       <c r="AB189" s="7"/>
       <c r="AC189" s="7"/>
       <c r="AD189" s="7">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AE189" s="36">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AF189" s="34"/>
       <c r="AG189" s="7"/>
@@ -26846,7 +26846,7 @@
       <c r="AB190" s="7"/>
       <c r="AC190" s="7"/>
       <c r="AD190" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AE190" s="36">
         <v>4</v>
@@ -27107,7 +27107,7 @@
         <v>4</v>
       </c>
       <c r="AE192" s="36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AF192" s="34"/>
       <c r="AG192" s="7"/>
@@ -27233,10 +27233,10 @@
       <c r="AB193" s="7"/>
       <c r="AC193" s="7"/>
       <c r="AD193" s="7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AE193" s="36">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AF193" s="34"/>
       <c r="AG193" s="7"/>
@@ -27362,10 +27362,10 @@
       <c r="AB194" s="7"/>
       <c r="AC194" s="7"/>
       <c r="AD194" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AE194" s="36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AF194" s="34"/>
       <c r="AG194" s="7"/>
@@ -27494,7 +27494,7 @@
         <v>4</v>
       </c>
       <c r="AE195" s="36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AF195" s="34"/>
       <c r="AG195" s="7"/>
@@ -27620,10 +27620,10 @@
       <c r="AB196" s="7"/>
       <c r="AC196" s="7"/>
       <c r="AD196" s="7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AE196" s="36">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AF196" s="34"/>
       <c r="AG196" s="7"/>
@@ -27749,10 +27749,10 @@
       <c r="AB197" s="7"/>
       <c r="AC197" s="7"/>
       <c r="AD197" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AE197" s="36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AF197" s="34"/>
       <c r="AG197" s="7"/>
@@ -27878,7 +27878,7 @@
       <c r="AB198" s="7"/>
       <c r="AC198" s="7"/>
       <c r="AD198" s="7">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="AE198" s="36">
         <v>6</v>
@@ -28005,7 +28005,7 @@
       <c r="AB199" s="7"/>
       <c r="AC199" s="7"/>
       <c r="AD199" s="7">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AE199" s="36">
         <v>8</v>
@@ -28134,7 +28134,7 @@
       <c r="AB200" s="7"/>
       <c r="AC200" s="7"/>
       <c r="AD200" s="7">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AE200" s="36">
         <v>9</v>
@@ -28263,10 +28263,10 @@
       <c r="AB201" s="7"/>
       <c r="AC201" s="7"/>
       <c r="AD201" s="7">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AE201" s="36">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AF201" s="34"/>
       <c r="AG201" s="7"/>
@@ -28392,10 +28392,10 @@
       <c r="AB202" s="7"/>
       <c r="AC202" s="7"/>
       <c r="AD202" s="7">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="AE202" s="36">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AF202" s="34"/>
       <c r="AG202" s="7"/>
@@ -28521,7 +28521,7 @@
       <c r="AB203" s="7"/>
       <c r="AC203" s="7"/>
       <c r="AD203" s="7">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="AE203" s="36">
         <v>2</v>
@@ -28650,7 +28650,7 @@
       <c r="AB204" s="7"/>
       <c r="AC204" s="7"/>
       <c r="AD204" s="7">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AE204" s="36">
         <v>5</v>
@@ -28779,10 +28779,10 @@
       <c r="AB205" s="7"/>
       <c r="AC205" s="7"/>
       <c r="AD205" s="7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AE205" s="36">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AF205" s="34"/>
       <c r="AG205" s="7"/>
@@ -28908,7 +28908,7 @@
       <c r="AB206" s="7"/>
       <c r="AC206" s="7"/>
       <c r="AD206" s="7">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AE206" s="36">
         <v>6</v>
@@ -29037,7 +29037,7 @@
       <c r="AB207" s="7"/>
       <c r="AC207" s="7"/>
       <c r="AD207" s="7">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AE207" s="36">
         <v>4</v>
@@ -29285,7 +29285,7 @@
       <c r="AB209" s="7"/>
       <c r="AC209" s="7"/>
       <c r="AD209" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AE209" s="36">
         <v>3</v>
@@ -29543,7 +29543,7 @@
       <c r="AB211" s="7"/>
       <c r="AC211" s="7"/>
       <c r="AD211" s="7">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AE211" s="36">
         <v>9</v>
@@ -29670,10 +29670,10 @@
       <c r="AB212" s="7"/>
       <c r="AC212" s="7"/>
       <c r="AD212" s="7">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="AE212" s="36">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AF212" s="34"/>
       <c r="AG212" s="7"/>
@@ -29799,7 +29799,7 @@
       <c r="AB213" s="7"/>
       <c r="AC213" s="7"/>
       <c r="AD213" s="7">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="AE213" s="36">
         <v>22</v>
@@ -29928,7 +29928,7 @@
       <c r="AB214" s="7"/>
       <c r="AC214" s="7"/>
       <c r="AD214" s="7">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="AE214" s="36">
         <v>4</v>
@@ -30055,7 +30055,7 @@
       <c r="AB215" s="7"/>
       <c r="AC215" s="7"/>
       <c r="AD215" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AE215" s="36">
         <v>1</v>
@@ -30303,7 +30303,7 @@
       <c r="AB217" s="7"/>
       <c r="AC217" s="7"/>
       <c r="AD217" s="7">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AE217" s="36">
         <v>6</v>
@@ -30432,7 +30432,7 @@
       <c r="AB218" s="7"/>
       <c r="AC218" s="7"/>
       <c r="AD218" s="7">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AE218" s="36">
         <v>2</v>
@@ -30561,10 +30561,10 @@
       <c r="AB219" s="7"/>
       <c r="AC219" s="7"/>
       <c r="AD219" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE219" s="36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF219" s="34"/>
       <c r="AG219" s="7"/>
@@ -30690,10 +30690,10 @@
       <c r="AB220" s="7"/>
       <c r="AC220" s="7"/>
       <c r="AD220" s="7">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AE220" s="36">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AF220" s="34"/>
       <c r="AG220" s="7"/>
@@ -30819,10 +30819,10 @@
       <c r="AB221" s="7"/>
       <c r="AC221" s="7"/>
       <c r="AD221" s="7">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AE221" s="36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AF221" s="34"/>
       <c r="AG221" s="7"/>
@@ -30948,10 +30948,10 @@
       <c r="AB222" s="7"/>
       <c r="AC222" s="7"/>
       <c r="AD222" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AE222" s="36">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AF222" s="34"/>
       <c r="AG222" s="7"/>
@@ -31067,7 +31067,7 @@
       <c r="AB223" s="7"/>
       <c r="AC223" s="7"/>
       <c r="AD223" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE223" s="36">
         <v>2</v>
@@ -31196,10 +31196,10 @@
       <c r="AB224" s="7"/>
       <c r="AC224" s="7"/>
       <c r="AD224" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE224" s="36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF224" s="34"/>
       <c r="AG224" s="7"/>
@@ -31325,7 +31325,7 @@
       <c r="AB225" s="7"/>
       <c r="AC225" s="7"/>
       <c r="AD225" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AE225" s="36">
         <v>1</v>
@@ -31454,7 +31454,7 @@
       <c r="AB226" s="7"/>
       <c r="AC226" s="7"/>
       <c r="AD226" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AE226" s="36">
         <v>3</v>
@@ -31583,10 +31583,10 @@
       <c r="AB227" s="7"/>
       <c r="AC227" s="7"/>
       <c r="AD227" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AE227" s="36">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AF227" s="34"/>
       <c r="AG227" s="7"/>
@@ -31702,7 +31702,7 @@
       <c r="AB228" s="7"/>
       <c r="AC228" s="7"/>
       <c r="AD228" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AE228" s="36">
         <v>3</v>
@@ -31831,10 +31831,10 @@
       <c r="AB229" s="7"/>
       <c r="AC229" s="7"/>
       <c r="AD229" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AE229" s="36">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AF229" s="34"/>
       <c r="AG229" s="7"/>
@@ -32072,7 +32072,7 @@
         <v>1</v>
       </c>
       <c r="AE231" s="36">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF231" s="34"/>
       <c r="AG231" s="7"/>
@@ -32198,7 +32198,7 @@
       <c r="AB232" s="7"/>
       <c r="AC232" s="7"/>
       <c r="AD232" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE232" s="36">
         <v>2</v>
@@ -32327,7 +32327,7 @@
       <c r="AB233" s="7"/>
       <c r="AC233" s="7"/>
       <c r="AD233" s="7">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AE233" s="36">
         <v>5</v>
@@ -32456,7 +32456,7 @@
       <c r="AB234" s="7"/>
       <c r="AC234" s="7"/>
       <c r="AD234" s="7">
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="AE234" s="36">
         <v>28</v>
@@ -32583,7 +32583,7 @@
       <c r="AB235" s="7"/>
       <c r="AC235" s="7"/>
       <c r="AD235" s="7">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="AE235" s="36">
         <v>20</v>
@@ -32710,7 +32710,7 @@
       <c r="AB236" s="7"/>
       <c r="AC236" s="7"/>
       <c r="AD236" s="7">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="AE236" s="36">
         <v>2</v>
@@ -32842,7 +32842,7 @@
         <v>2</v>
       </c>
       <c r="AE237" s="36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AF237" s="34"/>
       <c r="AG237" s="7"/>
@@ -32968,10 +32968,10 @@
       <c r="AB238" s="7"/>
       <c r="AC238" s="7"/>
       <c r="AD238" s="7">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AE238" s="36">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AF238" s="34"/>
       <c r="AG238" s="7"/>
@@ -33097,7 +33097,7 @@
       <c r="AB239" s="7"/>
       <c r="AC239" s="7"/>
       <c r="AD239" s="7">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AE239" s="36">
         <v>4</v>
@@ -33474,7 +33474,7 @@
       <c r="AB242" s="7"/>
       <c r="AC242" s="7"/>
       <c r="AD242" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AE242" s="36">
         <v>2</v>
@@ -33593,7 +33593,7 @@
       <c r="AB243" s="7"/>
       <c r="AC243" s="7"/>
       <c r="AD243" s="7">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="AE243" s="36">
         <v>8</v>
@@ -33720,7 +33720,7 @@
       <c r="AB244" s="7"/>
       <c r="AC244" s="7"/>
       <c r="AD244" s="7">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="AE244" s="36">
         <v>5</v>
@@ -33839,7 +33839,7 @@
       <c r="AB245" s="7"/>
       <c r="AC245" s="7"/>
       <c r="AD245" s="7">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AE245" s="36">
         <v>3</v>
@@ -33968,7 +33968,7 @@
       <c r="AB246" s="7"/>
       <c r="AC246" s="7"/>
       <c r="AD246" s="7">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AE246" s="36">
         <v>6</v>
@@ -34097,10 +34097,10 @@
       <c r="AB247" s="7"/>
       <c r="AC247" s="7"/>
       <c r="AD247" s="7">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="AE247" s="36">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="AF247" s="34"/>
       <c r="AG247" s="7"/>
@@ -34229,7 +34229,7 @@
         <v>13</v>
       </c>
       <c r="AE248" s="36">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="AF248" s="34"/>
       <c r="AG248" s="7"/>
@@ -34355,7 +34355,7 @@
       <c r="AB249" s="7"/>
       <c r="AC249" s="7"/>
       <c r="AD249" s="7">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="AE249" s="36">
         <v>2</v>
@@ -34484,10 +34484,10 @@
       <c r="AB250" s="7"/>
       <c r="AC250" s="7"/>
       <c r="AD250" s="7">
+        <v>4</v>
+      </c>
+      <c r="AE250" s="36">
         <v>3</v>
-      </c>
-      <c r="AE250" s="36">
-        <v>2</v>
       </c>
       <c r="AF250" s="34"/>
       <c r="AG250" s="7"/>
@@ -34613,10 +34613,10 @@
       <c r="AB251" s="7"/>
       <c r="AC251" s="7"/>
       <c r="AD251" s="7">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="AE251" s="36">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AF251" s="34"/>
       <c r="AG251" s="7"/>
@@ -34745,7 +34745,7 @@
         <v>8</v>
       </c>
       <c r="AE252" s="36">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AF252" s="34"/>
       <c r="AG252" s="7"/>
@@ -34871,10 +34871,10 @@
       <c r="AB253" s="7"/>
       <c r="AC253" s="7"/>
       <c r="AD253" s="7">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="AE253" s="36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF253" s="34"/>
       <c r="AG253" s="7"/>
@@ -35000,10 +35000,10 @@
       <c r="AB254" s="7"/>
       <c r="AC254" s="7"/>
       <c r="AD254" s="7">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="AE254" s="36">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AF254" s="34"/>
       <c r="AG254" s="7"/>
@@ -35129,7 +35129,7 @@
       <c r="AB255" s="7"/>
       <c r="AC255" s="7"/>
       <c r="AD255" s="7">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AE255" s="36">
         <v>10</v>
@@ -35258,10 +35258,10 @@
       <c r="AB256" s="7"/>
       <c r="AC256" s="7"/>
       <c r="AD256" s="7">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="AE256" s="36">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AF256" s="34"/>
       <c r="AG256" s="7"/>
@@ -35387,32 +35387,22 @@
       <c r="AB257" s="7"/>
       <c r="AC257" s="7"/>
       <c r="AD257" s="7">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AE257" s="36">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AF257" s="34"/>
       <c r="AG257" s="7"/>
       <c r="AH257" s="34"/>
-      <c r="AI257" s="34">
-        <v>46262</v>
-      </c>
-      <c r="AJ257" s="34">
-        <v>46262</v>
-      </c>
-      <c r="AK257" s="34">
-        <v>46262</v>
-      </c>
-      <c r="AL257" s="34">
-        <v>46262</v>
-      </c>
+      <c r="AI257" s="34"/>
+      <c r="AJ257" s="34"/>
+      <c r="AK257" s="34"/>
+      <c r="AL257" s="34"/>
       <c r="AM257" s="34"/>
       <c r="AN257" s="7"/>
       <c r="AO257" s="7"/>
-      <c r="AP257" s="34">
-        <v>46266</v>
-      </c>
+      <c r="AP257" s="34"/>
       <c r="AQ257" s="7"/>
       <c r="AR257" s="34"/>
       <c r="AS257" s="34"/>
@@ -35516,10 +35506,10 @@
       <c r="AB258" s="7"/>
       <c r="AC258" s="7"/>
       <c r="AD258" s="7">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="AE258" s="36">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="AF258" s="34"/>
       <c r="AG258" s="7"/>
@@ -35645,7 +35635,7 @@
       <c r="AB259" s="7"/>
       <c r="AC259" s="7"/>
       <c r="AD259" s="7">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="AE259" s="36">
         <v>8</v>
@@ -35774,10 +35764,10 @@
       <c r="AB260" s="7"/>
       <c r="AC260" s="7"/>
       <c r="AD260" s="7">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="AE260" s="36">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="AF260" s="34"/>
       <c r="AG260" s="7"/>
@@ -35903,7 +35893,7 @@
       <c r="AB261" s="7"/>
       <c r="AC261" s="7"/>
       <c r="AD261" s="7">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="AE261" s="36">
         <v>3</v>
@@ -36030,7 +36020,7 @@
       <c r="AB262" s="7"/>
       <c r="AC262" s="7"/>
       <c r="AD262" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AE262" s="36">
         <v>4</v>
@@ -36416,7 +36406,7 @@
         <v>4</v>
       </c>
       <c r="AE265" s="36">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AF265" s="34"/>
       <c r="AG265" s="7"/>
@@ -36542,10 +36532,10 @@
       <c r="AB266" s="7"/>
       <c r="AC266" s="7"/>
       <c r="AD266" s="7">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="AE266" s="36">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AF266" s="34"/>
       <c r="AG266" s="7"/>
@@ -36800,10 +36790,10 @@
       <c r="AB268" s="7"/>
       <c r="AC268" s="7"/>
       <c r="AD268" s="7">
+        <v>5</v>
+      </c>
+      <c r="AE268" s="36">
         <v>4</v>
-      </c>
-      <c r="AE268" s="36">
-        <v>3</v>
       </c>
       <c r="AF268" s="34"/>
       <c r="AG268" s="7"/>
@@ -36929,7 +36919,7 @@
       <c r="AB269" s="7"/>
       <c r="AC269" s="7"/>
       <c r="AD269" s="7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AE269" s="36">
         <v>4</v>
@@ -37058,7 +37048,7 @@
       <c r="AB270" s="7"/>
       <c r="AC270" s="7"/>
       <c r="AD270" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AE270" s="36">
         <v>2</v>
@@ -37187,10 +37177,10 @@
       <c r="AB271" s="7"/>
       <c r="AC271" s="7"/>
       <c r="AD271" s="7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="AE271" s="36">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="AF271" s="34"/>
       <c r="AG271" s="7"/>

</xml_diff>

<commit_message>
Preenche Relatório DF do spool com o relatório dimensional das juntas
Relatório DF do Mapa de Spools recebe o nº do relatório do grupo
"Rastreabilidade - dimensional" das juntas Pipe Shop do spool (spool
sem juntas Pipe usa as de Campo). Relatório múltiplo, juntas sem
relatório e relatório vindo de junta de Campo são listados no CSV.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jhm2rrJCBVkJYZMmi4pDeT
</commit_message>
<xml_diff>
--- a/saida/Situacao_Geral_de_Spools_ATUALIZADO.xlsx
+++ b/saida/Situacao_Geral_de_Spools_ATUALIZADO.xlsx
@@ -3735,7 +3735,11 @@
         <v>46262</v>
       </c>
       <c r="AM9" s="34"/>
-      <c r="AN9" s="7"/>
+      <c r="AN9" s="7" t="inlineStr">
+        <is>
+          <t>049/26</t>
+        </is>
+      </c>
       <c r="AO9" s="7"/>
       <c r="AP9" s="34">
         <v>46266</v>
@@ -3863,7 +3867,11 @@
       <c r="AK10" s="34"/>
       <c r="AL10" s="34"/>
       <c r="AM10" s="34"/>
-      <c r="AN10" s="7"/>
+      <c r="AN10" s="7" t="inlineStr">
+        <is>
+          <t>049/26</t>
+        </is>
+      </c>
       <c r="AO10" s="7"/>
       <c r="AP10" s="34"/>
       <c r="AQ10" s="7"/>
@@ -3992,7 +4000,11 @@
         <v>46263</v>
       </c>
       <c r="AM11" s="34"/>
-      <c r="AN11" s="7"/>
+      <c r="AN11" s="7" t="inlineStr">
+        <is>
+          <t>051/26</t>
+        </is>
+      </c>
       <c r="AO11" s="7"/>
       <c r="AP11" s="34">
         <v>46266</v>
@@ -4123,7 +4135,11 @@
         <v>46262</v>
       </c>
       <c r="AM12" s="34"/>
-      <c r="AN12" s="7"/>
+      <c r="AN12" s="7" t="inlineStr">
+        <is>
+          <t>052/26</t>
+        </is>
+      </c>
       <c r="AO12" s="7"/>
       <c r="AP12" s="34">
         <v>46266</v>
@@ -4254,7 +4270,11 @@
         <v>46265</v>
       </c>
       <c r="AM13" s="34"/>
-      <c r="AN13" s="7"/>
+      <c r="AN13" s="7" t="inlineStr">
+        <is>
+          <t>053/26</t>
+        </is>
+      </c>
       <c r="AO13" s="7"/>
       <c r="AP13" s="34">
         <v>46266</v>
@@ -4385,7 +4405,11 @@
         <v>46265</v>
       </c>
       <c r="AM14" s="34"/>
-      <c r="AN14" s="7"/>
+      <c r="AN14" s="7" t="inlineStr">
+        <is>
+          <t>054/26</t>
+        </is>
+      </c>
       <c r="AO14" s="7"/>
       <c r="AP14" s="34">
         <v>46266</v>
@@ -4647,7 +4671,11 @@
         <v>46266</v>
       </c>
       <c r="AM16" s="34"/>
-      <c r="AN16" s="7"/>
+      <c r="AN16" s="7" t="inlineStr">
+        <is>
+          <t>036/26</t>
+        </is>
+      </c>
       <c r="AO16" s="7"/>
       <c r="AP16" s="34">
         <v>46267</v>
@@ -4778,7 +4806,11 @@
         <v>47363</v>
       </c>
       <c r="AM17" s="34"/>
-      <c r="AN17" s="7"/>
+      <c r="AN17" s="7" t="inlineStr">
+        <is>
+          <t>037/26</t>
+        </is>
+      </c>
       <c r="AO17" s="7"/>
       <c r="AP17" s="34">
         <v>46267</v>
@@ -4909,7 +4941,11 @@
         <v>46266</v>
       </c>
       <c r="AM18" s="34"/>
-      <c r="AN18" s="7"/>
+      <c r="AN18" s="7" t="inlineStr">
+        <is>
+          <t>038/26</t>
+        </is>
+      </c>
       <c r="AO18" s="7"/>
       <c r="AP18" s="34">
         <v>46267</v>
@@ -5040,7 +5076,11 @@
         <v>47363</v>
       </c>
       <c r="AM19" s="34"/>
-      <c r="AN19" s="7"/>
+      <c r="AN19" s="7" t="inlineStr">
+        <is>
+          <t>039/26</t>
+        </is>
+      </c>
       <c r="AO19" s="7"/>
       <c r="AP19" s="34">
         <v>46267</v>
@@ -6070,7 +6110,11 @@
       <c r="AK27" s="34"/>
       <c r="AL27" s="34"/>
       <c r="AM27" s="34"/>
-      <c r="AN27" s="7"/>
+      <c r="AN27" s="7" t="inlineStr">
+        <is>
+          <t>080/26</t>
+        </is>
+      </c>
       <c r="AO27" s="7"/>
       <c r="AP27" s="34"/>
       <c r="AQ27" s="7"/>
@@ -8390,7 +8434,11 @@
         <v>46267</v>
       </c>
       <c r="AM45" s="34"/>
-      <c r="AN45" s="7"/>
+      <c r="AN45" s="7" t="inlineStr">
+        <is>
+          <t>040/26</t>
+        </is>
+      </c>
       <c r="AO45" s="7"/>
       <c r="AP45" s="34"/>
       <c r="AQ45" s="7"/>
@@ -8519,7 +8567,11 @@
         <v>46267</v>
       </c>
       <c r="AM46" s="34"/>
-      <c r="AN46" s="7"/>
+      <c r="AN46" s="7" t="inlineStr">
+        <is>
+          <t>040/26</t>
+        </is>
+      </c>
       <c r="AO46" s="7"/>
       <c r="AP46" s="34">
         <v>46267</v>
@@ -8781,7 +8833,11 @@
         <v>46266</v>
       </c>
       <c r="AM48" s="34"/>
-      <c r="AN48" s="7"/>
+      <c r="AN48" s="7" t="inlineStr">
+        <is>
+          <t>041/26</t>
+        </is>
+      </c>
       <c r="AO48" s="7"/>
       <c r="AP48" s="34">
         <v>46267</v>
@@ -8912,7 +8968,11 @@
         <v>46266</v>
       </c>
       <c r="AM49" s="34"/>
-      <c r="AN49" s="7"/>
+      <c r="AN49" s="7" t="inlineStr">
+        <is>
+          <t>041/26</t>
+        </is>
+      </c>
       <c r="AO49" s="7"/>
       <c r="AP49" s="34">
         <v>46267</v>
@@ -9043,7 +9103,11 @@
         <v>46267</v>
       </c>
       <c r="AM50" s="34"/>
-      <c r="AN50" s="7"/>
+      <c r="AN50" s="7" t="inlineStr">
+        <is>
+          <t>042/26</t>
+        </is>
+      </c>
       <c r="AO50" s="7"/>
       <c r="AP50" s="34">
         <v>46267</v>
@@ -9174,7 +9238,11 @@
         <v>46267</v>
       </c>
       <c r="AM51" s="34"/>
-      <c r="AN51" s="7"/>
+      <c r="AN51" s="7" t="inlineStr">
+        <is>
+          <t>043/26</t>
+        </is>
+      </c>
       <c r="AO51" s="7"/>
       <c r="AP51" s="34">
         <v>46267</v>
@@ -9305,7 +9373,11 @@
         <v>46266</v>
       </c>
       <c r="AM52" s="34"/>
-      <c r="AN52" s="7"/>
+      <c r="AN52" s="7" t="inlineStr">
+        <is>
+          <t>044/26</t>
+        </is>
+      </c>
       <c r="AO52" s="7"/>
       <c r="AP52" s="34">
         <v>46267</v>
@@ -9436,7 +9508,11 @@
         <v>46267</v>
       </c>
       <c r="AM53" s="34"/>
-      <c r="AN53" s="7"/>
+      <c r="AN53" s="7" t="inlineStr">
+        <is>
+          <t>046/26</t>
+        </is>
+      </c>
       <c r="AO53" s="7"/>
       <c r="AP53" s="34">
         <v>46267</v>
@@ -11911,7 +11987,11 @@
         <v>46261</v>
       </c>
       <c r="AM72" s="34"/>
-      <c r="AN72" s="7"/>
+      <c r="AN72" s="7" t="inlineStr">
+        <is>
+          <t>066/26</t>
+        </is>
+      </c>
       <c r="AO72" s="7"/>
       <c r="AP72" s="34">
         <v>46266</v>
@@ -12173,7 +12253,11 @@
         <v>46261</v>
       </c>
       <c r="AM74" s="34"/>
-      <c r="AN74" s="7"/>
+      <c r="AN74" s="7" t="inlineStr">
+        <is>
+          <t>066/26</t>
+        </is>
+      </c>
       <c r="AO74" s="7"/>
       <c r="AP74" s="34">
         <v>46266</v>
@@ -12296,7 +12380,11 @@
       <c r="AK75" s="34"/>
       <c r="AL75" s="34"/>
       <c r="AM75" s="34"/>
-      <c r="AN75" s="7"/>
+      <c r="AN75" s="7" t="inlineStr">
+        <is>
+          <t>066/26</t>
+        </is>
+      </c>
       <c r="AO75" s="7"/>
       <c r="AP75" s="34"/>
       <c r="AQ75" s="7"/>
@@ -12425,7 +12513,11 @@
         <v>46262</v>
       </c>
       <c r="AM76" s="34"/>
-      <c r="AN76" s="7"/>
+      <c r="AN76" s="7" t="inlineStr">
+        <is>
+          <t>067/26</t>
+        </is>
+      </c>
       <c r="AO76" s="7"/>
       <c r="AP76" s="34">
         <v>46266</v>
@@ -12687,7 +12779,11 @@
         <v>46262</v>
       </c>
       <c r="AM78" s="34"/>
-      <c r="AN78" s="7"/>
+      <c r="AN78" s="7" t="inlineStr">
+        <is>
+          <t>067/26</t>
+        </is>
+      </c>
       <c r="AO78" s="7"/>
       <c r="AP78" s="34">
         <v>46266</v>
@@ -12818,7 +12914,11 @@
         <v>46262</v>
       </c>
       <c r="AM79" s="34"/>
-      <c r="AN79" s="7"/>
+      <c r="AN79" s="7" t="inlineStr">
+        <is>
+          <t>065/26</t>
+        </is>
+      </c>
       <c r="AO79" s="7"/>
       <c r="AP79" s="34">
         <v>46266</v>
@@ -12949,7 +13049,11 @@
         <v>46262</v>
       </c>
       <c r="AM80" s="34"/>
-      <c r="AN80" s="7"/>
+      <c r="AN80" s="7" t="inlineStr">
+        <is>
+          <t>065/26</t>
+        </is>
+      </c>
       <c r="AO80" s="7"/>
       <c r="AP80" s="34">
         <v>46266</v>
@@ -13806,7 +13910,11 @@
         <v>46262</v>
       </c>
       <c r="AM87" s="34"/>
-      <c r="AN87" s="7"/>
+      <c r="AN87" s="7" t="inlineStr">
+        <is>
+          <t>068/26</t>
+        </is>
+      </c>
       <c r="AO87" s="7"/>
       <c r="AP87" s="34"/>
       <c r="AQ87" s="7"/>
@@ -13935,7 +14043,11 @@
         <v>46263</v>
       </c>
       <c r="AM88" s="34"/>
-      <c r="AN88" s="7"/>
+      <c r="AN88" s="7" t="inlineStr">
+        <is>
+          <t>069/26</t>
+        </is>
+      </c>
       <c r="AO88" s="7"/>
       <c r="AP88" s="34"/>
       <c r="AQ88" s="7"/>
@@ -14191,7 +14303,11 @@
         <v>46288</v>
       </c>
       <c r="AM90" s="34"/>
-      <c r="AN90" s="7"/>
+      <c r="AN90" s="7" t="inlineStr">
+        <is>
+          <t>081/26</t>
+        </is>
+      </c>
       <c r="AO90" s="7"/>
       <c r="AP90" s="34"/>
       <c r="AQ90" s="7"/>
@@ -14318,7 +14434,11 @@
         <v>46288</v>
       </c>
       <c r="AM91" s="34"/>
-      <c r="AN91" s="7"/>
+      <c r="AN91" s="7" t="inlineStr">
+        <is>
+          <t>081/26</t>
+        </is>
+      </c>
       <c r="AO91" s="7"/>
       <c r="AP91" s="34"/>
       <c r="AQ91" s="7"/>
@@ -14445,7 +14565,11 @@
         <v>46288</v>
       </c>
       <c r="AM92" s="34"/>
-      <c r="AN92" s="7"/>
+      <c r="AN92" s="7" t="inlineStr">
+        <is>
+          <t>082/26</t>
+        </is>
+      </c>
       <c r="AO92" s="7"/>
       <c r="AP92" s="34"/>
       <c r="AQ92" s="7"/>
@@ -14572,7 +14696,11 @@
         <v>46288</v>
       </c>
       <c r="AM93" s="34"/>
-      <c r="AN93" s="7"/>
+      <c r="AN93" s="7" t="inlineStr">
+        <is>
+          <t>082/26</t>
+        </is>
+      </c>
       <c r="AO93" s="7"/>
       <c r="AP93" s="34"/>
       <c r="AQ93" s="7"/>
@@ -14699,7 +14827,11 @@
         <v>46288</v>
       </c>
       <c r="AM94" s="34"/>
-      <c r="AN94" s="7"/>
+      <c r="AN94" s="7" t="inlineStr">
+        <is>
+          <t>083/26</t>
+        </is>
+      </c>
       <c r="AO94" s="7"/>
       <c r="AP94" s="34"/>
       <c r="AQ94" s="7"/>
@@ -14826,7 +14958,11 @@
         <v>46288</v>
       </c>
       <c r="AM95" s="34"/>
-      <c r="AN95" s="7"/>
+      <c r="AN95" s="7" t="inlineStr">
+        <is>
+          <t>083/26</t>
+        </is>
+      </c>
       <c r="AO95" s="7"/>
       <c r="AP95" s="34"/>
       <c r="AQ95" s="7"/>
@@ -14953,7 +15089,11 @@
         <v>46288</v>
       </c>
       <c r="AM96" s="34"/>
-      <c r="AN96" s="7"/>
+      <c r="AN96" s="7" t="inlineStr">
+        <is>
+          <t>084/26</t>
+        </is>
+      </c>
       <c r="AO96" s="7"/>
       <c r="AP96" s="34"/>
       <c r="AQ96" s="7"/>
@@ -15080,7 +15220,11 @@
         <v>46288</v>
       </c>
       <c r="AM97" s="34"/>
-      <c r="AN97" s="7"/>
+      <c r="AN97" s="7" t="inlineStr">
+        <is>
+          <t>084/26</t>
+        </is>
+      </c>
       <c r="AO97" s="7"/>
       <c r="AP97" s="34"/>
       <c r="AQ97" s="7"/>
@@ -15207,7 +15351,11 @@
         <v>46288</v>
       </c>
       <c r="AM98" s="34"/>
-      <c r="AN98" s="7"/>
+      <c r="AN98" s="7" t="inlineStr">
+        <is>
+          <t>085/26</t>
+        </is>
+      </c>
       <c r="AO98" s="7"/>
       <c r="AP98" s="34"/>
       <c r="AQ98" s="7"/>
@@ -15334,7 +15482,11 @@
         <v>46288</v>
       </c>
       <c r="AM99" s="34"/>
-      <c r="AN99" s="7"/>
+      <c r="AN99" s="7" t="inlineStr">
+        <is>
+          <t>085/26</t>
+        </is>
+      </c>
       <c r="AO99" s="7"/>
       <c r="AP99" s="34"/>
       <c r="AQ99" s="7"/>
@@ -15461,7 +15613,11 @@
         <v>46286</v>
       </c>
       <c r="AM100" s="34"/>
-      <c r="AN100" s="7"/>
+      <c r="AN100" s="7" t="inlineStr">
+        <is>
+          <t>087/26</t>
+        </is>
+      </c>
       <c r="AO100" s="7"/>
       <c r="AP100" s="34"/>
       <c r="AQ100" s="7"/>
@@ -15588,7 +15744,11 @@
         <v>46286</v>
       </c>
       <c r="AM101" s="34"/>
-      <c r="AN101" s="7"/>
+      <c r="AN101" s="7" t="inlineStr">
+        <is>
+          <t>087/26</t>
+        </is>
+      </c>
       <c r="AO101" s="7"/>
       <c r="AP101" s="34"/>
       <c r="AQ101" s="7"/>
@@ -15715,7 +15875,11 @@
         <v>46286</v>
       </c>
       <c r="AM102" s="34"/>
-      <c r="AN102" s="7"/>
+      <c r="AN102" s="7" t="inlineStr">
+        <is>
+          <t>086/26</t>
+        </is>
+      </c>
       <c r="AO102" s="7"/>
       <c r="AP102" s="34"/>
       <c r="AQ102" s="7"/>
@@ -15842,7 +16006,11 @@
         <v>46286</v>
       </c>
       <c r="AM103" s="34"/>
-      <c r="AN103" s="7"/>
+      <c r="AN103" s="7" t="inlineStr">
+        <is>
+          <t>086/26</t>
+        </is>
+      </c>
       <c r="AO103" s="7"/>
       <c r="AP103" s="34"/>
       <c r="AQ103" s="7"/>
@@ -15961,7 +16129,11 @@
       <c r="AK104" s="34"/>
       <c r="AL104" s="34"/>
       <c r="AM104" s="34"/>
-      <c r="AN104" s="7"/>
+      <c r="AN104" s="7" t="inlineStr">
+        <is>
+          <t>088/26</t>
+        </is>
+      </c>
       <c r="AO104" s="7"/>
       <c r="AP104" s="34"/>
       <c r="AQ104" s="7"/>
@@ -16088,7 +16260,11 @@
         <v>46286</v>
       </c>
       <c r="AM105" s="34"/>
-      <c r="AN105" s="7"/>
+      <c r="AN105" s="7" t="inlineStr">
+        <is>
+          <t>088/26</t>
+        </is>
+      </c>
       <c r="AO105" s="7"/>
       <c r="AP105" s="34"/>
       <c r="AQ105" s="7"/>
@@ -16215,7 +16391,11 @@
         <v>46286</v>
       </c>
       <c r="AM106" s="34"/>
-      <c r="AN106" s="7"/>
+      <c r="AN106" s="7" t="inlineStr">
+        <is>
+          <t>089/26</t>
+        </is>
+      </c>
       <c r="AO106" s="7"/>
       <c r="AP106" s="34"/>
       <c r="AQ106" s="7"/>
@@ -16342,7 +16522,11 @@
         <v>46286</v>
       </c>
       <c r="AM107" s="34"/>
-      <c r="AN107" s="7"/>
+      <c r="AN107" s="7" t="inlineStr">
+        <is>
+          <t>089/26</t>
+        </is>
+      </c>
       <c r="AO107" s="7"/>
       <c r="AP107" s="34"/>
       <c r="AQ107" s="7"/>
@@ -16461,7 +16645,11 @@
       <c r="AK108" s="34"/>
       <c r="AL108" s="34"/>
       <c r="AM108" s="34"/>
-      <c r="AN108" s="7"/>
+      <c r="AN108" s="7" t="inlineStr">
+        <is>
+          <t>090/26</t>
+        </is>
+      </c>
       <c r="AO108" s="7"/>
       <c r="AP108" s="34"/>
       <c r="AQ108" s="7"/>
@@ -16588,7 +16776,11 @@
         <v>46285</v>
       </c>
       <c r="AM109" s="34"/>
-      <c r="AN109" s="7"/>
+      <c r="AN109" s="7" t="inlineStr">
+        <is>
+          <t>090/26</t>
+        </is>
+      </c>
       <c r="AO109" s="7"/>
       <c r="AP109" s="34"/>
       <c r="AQ109" s="7"/>
@@ -16715,7 +16907,11 @@
         <v>46285</v>
       </c>
       <c r="AM110" s="34"/>
-      <c r="AN110" s="7"/>
+      <c r="AN110" s="7" t="inlineStr">
+        <is>
+          <t>091/26</t>
+        </is>
+      </c>
       <c r="AO110" s="7"/>
       <c r="AP110" s="34"/>
       <c r="AQ110" s="7"/>
@@ -16842,7 +17038,11 @@
         <v>46285</v>
       </c>
       <c r="AM111" s="34"/>
-      <c r="AN111" s="7"/>
+      <c r="AN111" s="7" t="inlineStr">
+        <is>
+          <t>091/26</t>
+        </is>
+      </c>
       <c r="AO111" s="7"/>
       <c r="AP111" s="34"/>
       <c r="AQ111" s="7"/>
@@ -16961,7 +17161,11 @@
       <c r="AK112" s="34"/>
       <c r="AL112" s="34"/>
       <c r="AM112" s="34"/>
-      <c r="AN112" s="7"/>
+      <c r="AN112" s="7" t="inlineStr">
+        <is>
+          <t>092/26</t>
+        </is>
+      </c>
       <c r="AO112" s="7"/>
       <c r="AP112" s="34"/>
       <c r="AQ112" s="7"/>
@@ -17088,7 +17292,11 @@
         <v>46285</v>
       </c>
       <c r="AM113" s="34"/>
-      <c r="AN113" s="7"/>
+      <c r="AN113" s="7" t="inlineStr">
+        <is>
+          <t>092/26</t>
+        </is>
+      </c>
       <c r="AO113" s="7"/>
       <c r="AP113" s="34"/>
       <c r="AQ113" s="7"/>
@@ -17207,7 +17415,11 @@
       <c r="AK114" s="34"/>
       <c r="AL114" s="34"/>
       <c r="AM114" s="34"/>
-      <c r="AN114" s="7"/>
+      <c r="AN114" s="7" t="inlineStr">
+        <is>
+          <t>098/26</t>
+        </is>
+      </c>
       <c r="AO114" s="7"/>
       <c r="AP114" s="34"/>
       <c r="AQ114" s="7"/>
@@ -17334,7 +17546,11 @@
         <v>46286</v>
       </c>
       <c r="AM115" s="34"/>
-      <c r="AN115" s="7"/>
+      <c r="AN115" s="7" t="inlineStr">
+        <is>
+          <t>099/26</t>
+        </is>
+      </c>
       <c r="AO115" s="7"/>
       <c r="AP115" s="34"/>
       <c r="AQ115" s="7"/>
@@ -17699,7 +17915,11 @@
         <v>46287</v>
       </c>
       <c r="AM118" s="34"/>
-      <c r="AN118" s="7"/>
+      <c r="AN118" s="7" t="inlineStr">
+        <is>
+          <t>076/26</t>
+        </is>
+      </c>
       <c r="AO118" s="7"/>
       <c r="AP118" s="34"/>
       <c r="AQ118" s="7"/>
@@ -17953,7 +18173,11 @@
         <v>46254</v>
       </c>
       <c r="AM120" s="34"/>
-      <c r="AN120" s="7"/>
+      <c r="AN120" s="7" t="inlineStr">
+        <is>
+          <t>016/26</t>
+        </is>
+      </c>
       <c r="AO120" s="7"/>
       <c r="AP120" s="34">
         <v>46255</v>
@@ -18074,7 +18298,11 @@
       <c r="AK121" s="34"/>
       <c r="AL121" s="34"/>
       <c r="AM121" s="34"/>
-      <c r="AN121" s="7"/>
+      <c r="AN121" s="7" t="inlineStr">
+        <is>
+          <t>016/26</t>
+        </is>
+      </c>
       <c r="AO121" s="7"/>
       <c r="AP121" s="34"/>
       <c r="AQ121" s="7"/>
@@ -18193,7 +18421,11 @@
       <c r="AK122" s="34"/>
       <c r="AL122" s="34"/>
       <c r="AM122" s="34"/>
-      <c r="AN122" s="7"/>
+      <c r="AN122" s="7" t="inlineStr">
+        <is>
+          <t>017/26</t>
+        </is>
+      </c>
       <c r="AO122" s="7"/>
       <c r="AP122" s="34"/>
       <c r="AQ122" s="7"/>
@@ -18320,7 +18552,11 @@
         <v>46258</v>
       </c>
       <c r="AM123" s="34"/>
-      <c r="AN123" s="7"/>
+      <c r="AN123" s="7" t="inlineStr">
+        <is>
+          <t>018/26</t>
+        </is>
+      </c>
       <c r="AO123" s="7"/>
       <c r="AP123" s="34">
         <v>46258</v>
@@ -18449,7 +18685,11 @@
         <v>46258</v>
       </c>
       <c r="AM124" s="34"/>
-      <c r="AN124" s="7"/>
+      <c r="AN124" s="7" t="inlineStr">
+        <is>
+          <t>019/26</t>
+        </is>
+      </c>
       <c r="AO124" s="7"/>
       <c r="AP124" s="34">
         <v>46258</v>
@@ -18578,7 +18818,11 @@
         <v>46287</v>
       </c>
       <c r="AM125" s="34"/>
-      <c r="AN125" s="7"/>
+      <c r="AN125" s="7" t="inlineStr">
+        <is>
+          <t>073/26</t>
+        </is>
+      </c>
       <c r="AO125" s="7"/>
       <c r="AP125" s="34"/>
       <c r="AQ125" s="7"/>
@@ -18705,7 +18949,11 @@
         <v>46287</v>
       </c>
       <c r="AM126" s="34"/>
-      <c r="AN126" s="7"/>
+      <c r="AN126" s="7" t="inlineStr">
+        <is>
+          <t>074/26</t>
+        </is>
+      </c>
       <c r="AO126" s="7"/>
       <c r="AP126" s="34"/>
       <c r="AQ126" s="7"/>
@@ -18832,7 +19080,11 @@
         <v>46287</v>
       </c>
       <c r="AM127" s="34"/>
-      <c r="AN127" s="7"/>
+      <c r="AN127" s="7" t="inlineStr">
+        <is>
+          <t>075/26</t>
+        </is>
+      </c>
       <c r="AO127" s="7"/>
       <c r="AP127" s="34"/>
       <c r="AQ127" s="7"/>
@@ -19862,7 +20114,11 @@
         <v>46286</v>
       </c>
       <c r="AM135" s="34"/>
-      <c r="AN135" s="7"/>
+      <c r="AN135" s="7" t="inlineStr">
+        <is>
+          <t>077/26</t>
+        </is>
+      </c>
       <c r="AO135" s="7"/>
       <c r="AP135" s="34">
         <v>46287</v>
@@ -19991,7 +20247,11 @@
         <v>46286</v>
       </c>
       <c r="AM136" s="34"/>
-      <c r="AN136" s="7"/>
+      <c r="AN136" s="7" t="inlineStr">
+        <is>
+          <t>078/26</t>
+        </is>
+      </c>
       <c r="AO136" s="7"/>
       <c r="AP136" s="34">
         <v>46287</v>
@@ -20120,7 +20380,11 @@
         <v>46286</v>
       </c>
       <c r="AM137" s="34"/>
-      <c r="AN137" s="7"/>
+      <c r="AN137" s="7" t="inlineStr">
+        <is>
+          <t>079/26</t>
+        </is>
+      </c>
       <c r="AO137" s="7"/>
       <c r="AP137" s="34">
         <v>46287</v>
@@ -24587,7 +24851,11 @@
         <v>46287</v>
       </c>
       <c r="AM172" s="34"/>
-      <c r="AN172" s="7"/>
+      <c r="AN172" s="7" t="inlineStr">
+        <is>
+          <t>072/26</t>
+        </is>
+      </c>
       <c r="AO172" s="7"/>
       <c r="AP172" s="34"/>
       <c r="AQ172" s="7"/>
@@ -24706,7 +24974,11 @@
       <c r="AK173" s="34"/>
       <c r="AL173" s="34"/>
       <c r="AM173" s="34"/>
-      <c r="AN173" s="7"/>
+      <c r="AN173" s="7" t="inlineStr">
+        <is>
+          <t>070/26</t>
+        </is>
+      </c>
       <c r="AO173" s="7"/>
       <c r="AP173" s="34"/>
       <c r="AQ173" s="7"/>
@@ -24825,7 +25097,11 @@
       <c r="AK174" s="34"/>
       <c r="AL174" s="34"/>
       <c r="AM174" s="34"/>
-      <c r="AN174" s="7"/>
+      <c r="AN174" s="7" t="inlineStr">
+        <is>
+          <t>071/26</t>
+        </is>
+      </c>
       <c r="AO174" s="7"/>
       <c r="AP174" s="34"/>
       <c r="AQ174" s="7"/>
@@ -24952,7 +25228,11 @@
         <v>46286</v>
       </c>
       <c r="AM175" s="34"/>
-      <c r="AN175" s="7"/>
+      <c r="AN175" s="7" t="inlineStr">
+        <is>
+          <t>100/26</t>
+        </is>
+      </c>
       <c r="AO175" s="7"/>
       <c r="AP175" s="34"/>
       <c r="AQ175" s="7"/>
@@ -25079,7 +25359,11 @@
         <v>46286</v>
       </c>
       <c r="AM176" s="34"/>
-      <c r="AN176" s="7"/>
+      <c r="AN176" s="7" t="inlineStr">
+        <is>
+          <t>101/26</t>
+        </is>
+      </c>
       <c r="AO176" s="7"/>
       <c r="AP176" s="34"/>
       <c r="AQ176" s="7"/>
@@ -25206,7 +25490,11 @@
         <v>46286</v>
       </c>
       <c r="AM177" s="34"/>
-      <c r="AN177" s="7"/>
+      <c r="AN177" s="7" t="inlineStr">
+        <is>
+          <t>102/26</t>
+        </is>
+      </c>
       <c r="AO177" s="7"/>
       <c r="AP177" s="34"/>
       <c r="AQ177" s="7"/>
@@ -25452,7 +25740,11 @@
         <v>46285</v>
       </c>
       <c r="AM179" s="34"/>
-      <c r="AN179" s="7"/>
+      <c r="AN179" s="7" t="inlineStr">
+        <is>
+          <t>096/26</t>
+        </is>
+      </c>
       <c r="AO179" s="7"/>
       <c r="AP179" s="34"/>
       <c r="AQ179" s="7"/>
@@ -25579,7 +25871,11 @@
         <v>46285</v>
       </c>
       <c r="AM180" s="34"/>
-      <c r="AN180" s="7"/>
+      <c r="AN180" s="7" t="inlineStr">
+        <is>
+          <t>097/26</t>
+        </is>
+      </c>
       <c r="AO180" s="7"/>
       <c r="AP180" s="34"/>
       <c r="AQ180" s="7"/>
@@ -27125,7 +27421,11 @@
         <v>46261</v>
       </c>
       <c r="AM192" s="34"/>
-      <c r="AN192" s="7"/>
+      <c r="AN192" s="7" t="inlineStr">
+        <is>
+          <t>047/26</t>
+        </is>
+      </c>
       <c r="AO192" s="7"/>
       <c r="AP192" s="34">
         <v>46266</v>
@@ -27383,7 +27683,11 @@
         <v>46261</v>
       </c>
       <c r="AM194" s="34"/>
-      <c r="AN194" s="7"/>
+      <c r="AN194" s="7" t="inlineStr">
+        <is>
+          <t>047/26</t>
+        </is>
+      </c>
       <c r="AO194" s="7"/>
       <c r="AP194" s="34">
         <v>46266</v>
@@ -27512,7 +27816,11 @@
         <v>46261</v>
       </c>
       <c r="AM195" s="34"/>
-      <c r="AN195" s="7"/>
+      <c r="AN195" s="7" t="inlineStr">
+        <is>
+          <t>048/26</t>
+        </is>
+      </c>
       <c r="AO195" s="7"/>
       <c r="AP195" s="34">
         <v>46266</v>
@@ -27770,7 +28078,11 @@
         <v>46261</v>
       </c>
       <c r="AM197" s="34"/>
-      <c r="AN197" s="7"/>
+      <c r="AN197" s="7" t="inlineStr">
+        <is>
+          <t>048/26</t>
+        </is>
+      </c>
       <c r="AO197" s="7"/>
       <c r="AP197" s="34">
         <v>46266</v>
@@ -29306,7 +29618,11 @@
         <v>46261</v>
       </c>
       <c r="AM209" s="34"/>
-      <c r="AN209" s="7"/>
+      <c r="AN209" s="7" t="inlineStr">
+        <is>
+          <t>055/26</t>
+        </is>
+      </c>
       <c r="AO209" s="7"/>
       <c r="AP209" s="34">
         <v>46266</v>
@@ -29435,7 +29751,11 @@
         <v>46261</v>
       </c>
       <c r="AM210" s="34"/>
-      <c r="AN210" s="7"/>
+      <c r="AN210" s="7" t="inlineStr">
+        <is>
+          <t>056/26</t>
+        </is>
+      </c>
       <c r="AO210" s="7"/>
       <c r="AP210" s="34">
         <v>46266</v>
@@ -29564,7 +29884,11 @@
         <v>46262</v>
       </c>
       <c r="AM211" s="34"/>
-      <c r="AN211" s="7"/>
+      <c r="AN211" s="7" t="inlineStr">
+        <is>
+          <t>050/26</t>
+        </is>
+      </c>
       <c r="AO211" s="7"/>
       <c r="AP211" s="34"/>
       <c r="AQ211" s="7"/>
@@ -29691,7 +30015,11 @@
         <v>46262</v>
       </c>
       <c r="AM212" s="34"/>
-      <c r="AN212" s="7"/>
+      <c r="AN212" s="7" t="inlineStr">
+        <is>
+          <t>050/26</t>
+        </is>
+      </c>
       <c r="AO212" s="7"/>
       <c r="AP212" s="34">
         <v>46266</v>
@@ -29820,7 +30148,11 @@
         <v>46265</v>
       </c>
       <c r="AM213" s="34"/>
-      <c r="AN213" s="7"/>
+      <c r="AN213" s="7" t="inlineStr">
+        <is>
+          <t>053/26</t>
+        </is>
+      </c>
       <c r="AO213" s="7"/>
       <c r="AP213" s="34">
         <v>46267</v>
@@ -33237,7 +33569,11 @@
         <v>46261</v>
       </c>
       <c r="AM240" s="34"/>
-      <c r="AN240" s="7"/>
+      <c r="AN240" s="7" t="inlineStr">
+        <is>
+          <t>064/26</t>
+        </is>
+      </c>
       <c r="AO240" s="7"/>
       <c r="AP240" s="34">
         <v>46266</v>
@@ -33860,7 +34196,11 @@
         <v>46254</v>
       </c>
       <c r="AM245" s="34"/>
-      <c r="AN245" s="7"/>
+      <c r="AN245" s="7" t="inlineStr">
+        <is>
+          <t>032/26</t>
+        </is>
+      </c>
       <c r="AO245" s="7"/>
       <c r="AP245" s="34">
         <v>46255</v>
@@ -33989,7 +34329,11 @@
         <v>46265</v>
       </c>
       <c r="AM246" s="34"/>
-      <c r="AN246" s="7"/>
+      <c r="AN246" s="7" t="inlineStr">
+        <is>
+          <t>057/26</t>
+        </is>
+      </c>
       <c r="AO246" s="7"/>
       <c r="AP246" s="34">
         <v>46266</v>
@@ -34118,7 +34462,11 @@
         <v>46265</v>
       </c>
       <c r="AM247" s="34"/>
-      <c r="AN247" s="7"/>
+      <c r="AN247" s="7" t="inlineStr">
+        <is>
+          <t>057/26</t>
+        </is>
+      </c>
       <c r="AO247" s="7"/>
       <c r="AP247" s="34">
         <v>46266</v>
@@ -34247,7 +34595,11 @@
         <v>46265</v>
       </c>
       <c r="AM248" s="34"/>
-      <c r="AN248" s="7"/>
+      <c r="AN248" s="7" t="inlineStr">
+        <is>
+          <t>057/26</t>
+        </is>
+      </c>
       <c r="AO248" s="7"/>
       <c r="AP248" s="34">
         <v>46266</v>
@@ -34376,7 +34728,11 @@
         <v>46262</v>
       </c>
       <c r="AM249" s="34"/>
-      <c r="AN249" s="7"/>
+      <c r="AN249" s="7" t="inlineStr">
+        <is>
+          <t>018/26</t>
+        </is>
+      </c>
       <c r="AO249" s="7"/>
       <c r="AP249" s="34">
         <v>46266</v>
@@ -34505,7 +34861,11 @@
         <v>46262</v>
       </c>
       <c r="AM250" s="34"/>
-      <c r="AN250" s="7"/>
+      <c r="AN250" s="7" t="inlineStr">
+        <is>
+          <t>018/26</t>
+        </is>
+      </c>
       <c r="AO250" s="7"/>
       <c r="AP250" s="34">
         <v>46266</v>
@@ -34634,7 +34994,11 @@
         <v>46262</v>
       </c>
       <c r="AM251" s="34"/>
-      <c r="AN251" s="7"/>
+      <c r="AN251" s="7" t="inlineStr">
+        <is>
+          <t>018/26</t>
+        </is>
+      </c>
       <c r="AO251" s="7"/>
       <c r="AP251" s="34">
         <v>46266</v>
@@ -34763,7 +35127,11 @@
         <v>46262</v>
       </c>
       <c r="AM252" s="34"/>
-      <c r="AN252" s="7"/>
+      <c r="AN252" s="7" t="inlineStr">
+        <is>
+          <t>018/26</t>
+        </is>
+      </c>
       <c r="AO252" s="7"/>
       <c r="AP252" s="34">
         <v>46266</v>
@@ -34892,7 +35260,11 @@
         <v>46265</v>
       </c>
       <c r="AM253" s="34"/>
-      <c r="AN253" s="7"/>
+      <c r="AN253" s="7" t="inlineStr">
+        <is>
+          <t>019/26</t>
+        </is>
+      </c>
       <c r="AO253" s="7"/>
       <c r="AP253" s="34">
         <v>46266</v>
@@ -35021,7 +35393,11 @@
         <v>46265</v>
       </c>
       <c r="AM254" s="34"/>
-      <c r="AN254" s="7"/>
+      <c r="AN254" s="7" t="inlineStr">
+        <is>
+          <t>019/26</t>
+        </is>
+      </c>
       <c r="AO254" s="7"/>
       <c r="AP254" s="34">
         <v>46266</v>
@@ -35150,7 +35526,11 @@
         <v>46262</v>
       </c>
       <c r="AM255" s="34"/>
-      <c r="AN255" s="7"/>
+      <c r="AN255" s="7" t="inlineStr">
+        <is>
+          <t>060/26</t>
+        </is>
+      </c>
       <c r="AO255" s="7"/>
       <c r="AP255" s="34">
         <v>46266</v>
@@ -35279,7 +35659,11 @@
         <v>46262</v>
       </c>
       <c r="AM256" s="34"/>
-      <c r="AN256" s="7"/>
+      <c r="AN256" s="7" t="inlineStr">
+        <is>
+          <t>060/26</t>
+        </is>
+      </c>
       <c r="AO256" s="7"/>
       <c r="AP256" s="34">
         <v>46266</v>
@@ -35400,7 +35784,11 @@
       <c r="AK257" s="34"/>
       <c r="AL257" s="34"/>
       <c r="AM257" s="34"/>
-      <c r="AN257" s="7"/>
+      <c r="AN257" s="7" t="inlineStr">
+        <is>
+          <t>060/26</t>
+        </is>
+      </c>
       <c r="AO257" s="7"/>
       <c r="AP257" s="34"/>
       <c r="AQ257" s="7"/>
@@ -35527,7 +35915,11 @@
         <v>46294</v>
       </c>
       <c r="AM258" s="34"/>
-      <c r="AN258" s="7"/>
+      <c r="AN258" s="7" t="inlineStr">
+        <is>
+          <t>060/26</t>
+        </is>
+      </c>
       <c r="AO258" s="7"/>
       <c r="AP258" s="34">
         <v>46266</v>
@@ -35656,7 +36048,11 @@
         <v>46263</v>
       </c>
       <c r="AM259" s="34"/>
-      <c r="AN259" s="7"/>
+      <c r="AN259" s="7" t="inlineStr">
+        <is>
+          <t>061/26</t>
+        </is>
+      </c>
       <c r="AO259" s="7"/>
       <c r="AP259" s="34">
         <v>46266</v>
@@ -35785,7 +36181,11 @@
         <v>46265</v>
       </c>
       <c r="AM260" s="34"/>
-      <c r="AN260" s="7"/>
+      <c r="AN260" s="7" t="inlineStr">
+        <is>
+          <t>062/26</t>
+        </is>
+      </c>
       <c r="AO260" s="7"/>
       <c r="AP260" s="34">
         <v>46266</v>
@@ -35914,7 +36314,11 @@
         <v>46285</v>
       </c>
       <c r="AM261" s="34"/>
-      <c r="AN261" s="7"/>
+      <c r="AN261" s="7" t="inlineStr">
+        <is>
+          <t>093/26</t>
+        </is>
+      </c>
       <c r="AO261" s="7"/>
       <c r="AP261" s="34"/>
       <c r="AQ261" s="7"/>
@@ -36041,7 +36445,11 @@
         <v>46285</v>
       </c>
       <c r="AM262" s="34"/>
-      <c r="AN262" s="7"/>
+      <c r="AN262" s="7" t="inlineStr">
+        <is>
+          <t>094/26</t>
+        </is>
+      </c>
       <c r="AO262" s="7"/>
       <c r="AP262" s="34"/>
       <c r="AQ262" s="7"/>
@@ -36168,7 +36576,11 @@
         <v>46285</v>
       </c>
       <c r="AM263" s="34"/>
-      <c r="AN263" s="7"/>
+      <c r="AN263" s="7" t="inlineStr">
+        <is>
+          <t>095/26</t>
+        </is>
+      </c>
       <c r="AO263" s="7"/>
       <c r="AP263" s="34"/>
       <c r="AQ263" s="7"/>

</xml_diff>

<commit_message>
Relatório DF pelo nº de relatório da Linha + Documento
O Relatório DF de cada spool passa a vir do relatório dimensional das
juntas Pipe Shop da mesma Linha + Documento (não mais só do spool, e sem
usar juntas de Campo). Documento com mais de um relatório usa o do
próprio spool e é avisado no relatório CSV.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jhm2rrJCBVkJYZMmi4pDeT
</commit_message>
<xml_diff>
--- a/saida/Situacao_Geral_de_Spools_ATUALIZADO.xlsx
+++ b/saida/Situacao_Geral_de_Spools_ATUALIZADO.xlsx
@@ -12122,7 +12122,11 @@
         <v>46261</v>
       </c>
       <c r="AM73" s="34"/>
-      <c r="AN73" s="7"/>
+      <c r="AN73" s="7" t="inlineStr">
+        <is>
+          <t>066/26</t>
+        </is>
+      </c>
       <c r="AO73" s="7"/>
       <c r="AP73" s="34">
         <v>46266</v>
@@ -12380,11 +12384,7 @@
       <c r="AK75" s="34"/>
       <c r="AL75" s="34"/>
       <c r="AM75" s="34"/>
-      <c r="AN75" s="7" t="inlineStr">
-        <is>
-          <t>066/26</t>
-        </is>
-      </c>
+      <c r="AN75" s="7"/>
       <c r="AO75" s="7"/>
       <c r="AP75" s="34"/>
       <c r="AQ75" s="7"/>
@@ -12648,7 +12648,11 @@
         <v>46262</v>
       </c>
       <c r="AM77" s="34"/>
-      <c r="AN77" s="7"/>
+      <c r="AN77" s="7" t="inlineStr">
+        <is>
+          <t>067/26</t>
+        </is>
+      </c>
       <c r="AO77" s="7"/>
       <c r="AP77" s="34">
         <v>46266</v>
@@ -27554,7 +27558,11 @@
         <v>46261</v>
       </c>
       <c r="AM193" s="34"/>
-      <c r="AN193" s="7"/>
+      <c r="AN193" s="7" t="inlineStr">
+        <is>
+          <t>047/26</t>
+        </is>
+      </c>
       <c r="AO193" s="7"/>
       <c r="AP193" s="34">
         <v>46266</v>
@@ -27949,7 +27957,11 @@
         <v>46261</v>
       </c>
       <c r="AM196" s="34"/>
-      <c r="AN196" s="7"/>
+      <c r="AN196" s="7" t="inlineStr">
+        <is>
+          <t>048/26</t>
+        </is>
+      </c>
       <c r="AO196" s="7"/>
       <c r="AP196" s="34">
         <v>46266</v>

</xml_diff>

<commit_message>
Diâmetro do spool pelo maior diâmetro das juntas
Di_Pol do Mapa de Spools recebe o maior diâmetro (em polegadas) entre
as juntas do spool no Mapa de Juntas e Diametro (mm) o valor da tabela
DIAMETRO (a coluna em mm do Mapa de Juntas tem erros de digitação).
Correções são listadas no relatório CSV.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jhm2rrJCBVkJYZMmi4pDeT
</commit_message>
<xml_diff>
--- a/saida/Situacao_Geral_de_Spools_ATUALIZADO.xlsx
+++ b/saida/Situacao_Geral_de_Spools_ATUALIZADO.xlsx
@@ -11543,10 +11543,12 @@
         <v>448</v>
       </c>
       <c r="P69" s="36">
-        <v>273</v>
-      </c>
-      <c r="Q69" s="7" t="s">
-        <v>105</v>
+        <v>219</v>
+      </c>
+      <c r="Q69" s="7" t="inlineStr">
+        <is>
+          <t>8"</t>
+        </is>
       </c>
       <c r="R69" s="7">
         <v>8.18</v>
@@ -17630,10 +17632,12 @@
         <v>103</v>
       </c>
       <c r="P116" s="36">
-        <v>60</v>
-      </c>
-      <c r="Q116" s="7" t="s">
-        <v>109</v>
+        <v>33</v>
+      </c>
+      <c r="Q116" s="7" t="inlineStr">
+        <is>
+          <t>1"</t>
+        </is>
       </c>
       <c r="R116" s="7">
         <v>3.38</v>
@@ -18505,10 +18509,12 @@
         <v>103</v>
       </c>
       <c r="P123" s="36">
-        <v>60</v>
-      </c>
-      <c r="Q123" s="7" t="s">
-        <v>109</v>
+        <v>33</v>
+      </c>
+      <c r="Q123" s="7" t="inlineStr">
+        <is>
+          <t>1"</t>
+        </is>
       </c>
       <c r="R123" s="7">
         <v>3.38</v>
@@ -19164,10 +19170,12 @@
         <v>103</v>
       </c>
       <c r="P128" s="36">
-        <v>60</v>
-      </c>
-      <c r="Q128" s="7" t="s">
-        <v>109</v>
+        <v>21</v>
+      </c>
+      <c r="Q128" s="7" t="inlineStr">
+        <is>
+          <t>1/2"</t>
+        </is>
       </c>
       <c r="R128" s="7">
         <v>2.77</v>
@@ -19293,10 +19301,12 @@
         <v>103</v>
       </c>
       <c r="P129" s="36">
-        <v>60</v>
-      </c>
-      <c r="Q129" s="7" t="s">
-        <v>109</v>
+        <v>21</v>
+      </c>
+      <c r="Q129" s="7" t="inlineStr">
+        <is>
+          <t>1/2"</t>
+        </is>
       </c>
       <c r="R129" s="7">
         <v>2.77</v>
@@ -19422,10 +19432,12 @@
         <v>103</v>
       </c>
       <c r="P130" s="36">
-        <v>60</v>
-      </c>
-      <c r="Q130" s="7" t="s">
-        <v>109</v>
+        <v>21</v>
+      </c>
+      <c r="Q130" s="7" t="inlineStr">
+        <is>
+          <t>1/2"</t>
+        </is>
       </c>
       <c r="R130" s="7">
         <v>2.77</v>
@@ -19551,10 +19563,12 @@
         <v>103</v>
       </c>
       <c r="P131" s="36">
-        <v>60</v>
-      </c>
-      <c r="Q131" s="7" t="s">
-        <v>109</v>
+        <v>21</v>
+      </c>
+      <c r="Q131" s="7" t="inlineStr">
+        <is>
+          <t>1/2"</t>
+        </is>
       </c>
       <c r="R131" s="7">
         <v>2.77</v>
@@ -19680,10 +19694,12 @@
         <v>103</v>
       </c>
       <c r="P132" s="36">
-        <v>60</v>
-      </c>
-      <c r="Q132" s="7" t="s">
-        <v>109</v>
+        <v>21</v>
+      </c>
+      <c r="Q132" s="7" t="inlineStr">
+        <is>
+          <t>1/2"</t>
+        </is>
       </c>
       <c r="R132" s="7">
         <v>2.77</v>
@@ -19809,10 +19825,12 @@
         <v>103</v>
       </c>
       <c r="P133" s="36">
-        <v>60</v>
-      </c>
-      <c r="Q133" s="7" t="s">
-        <v>109</v>
+        <v>21</v>
+      </c>
+      <c r="Q133" s="7" t="inlineStr">
+        <is>
+          <t>1/2"</t>
+        </is>
       </c>
       <c r="R133" s="7">
         <v>2.77</v>
@@ -20333,10 +20351,12 @@
         <v>448</v>
       </c>
       <c r="P137" s="36">
-        <v>60</v>
-      </c>
-      <c r="Q137" s="7" t="s">
-        <v>109</v>
+        <v>33</v>
+      </c>
+      <c r="Q137" s="7" t="inlineStr">
+        <is>
+          <t>1"</t>
+        </is>
       </c>
       <c r="R137" s="7">
         <v>4.55</v>
@@ -30746,10 +30766,12 @@
         <v>448</v>
       </c>
       <c r="P218" s="36">
-        <v>168</v>
-      </c>
-      <c r="Q218" s="7" t="s">
-        <v>113</v>
+        <v>89</v>
+      </c>
+      <c r="Q218" s="7" t="inlineStr">
+        <is>
+          <t>3"</t>
+        </is>
       </c>
       <c r="R218" s="7">
         <v>7.11</v>
@@ -31381,10 +31403,12 @@
         <v>448</v>
       </c>
       <c r="P223" s="36">
-        <v>168</v>
-      </c>
-      <c r="Q223" s="7" t="s">
-        <v>113</v>
+        <v>89</v>
+      </c>
+      <c r="Q223" s="7" t="inlineStr">
+        <is>
+          <t>3"</t>
+        </is>
       </c>
       <c r="R223" s="7">
         <v>7.11</v>
@@ -31510,10 +31534,12 @@
         <v>448</v>
       </c>
       <c r="P224" s="36">
-        <v>168</v>
-      </c>
-      <c r="Q224" s="7" t="s">
-        <v>113</v>
+        <v>89</v>
+      </c>
+      <c r="Q224" s="7" t="inlineStr">
+        <is>
+          <t>3"</t>
+        </is>
       </c>
       <c r="R224" s="7">
         <v>7.11</v>

</xml_diff>

<commit_message>
Relatório DF volta à regra por spool
Volta à primeira regra: Relatório DF recebe o relatório dimensional das
juntas Pipe Shop do próprio spool (sem juntas Pipe, usa as de Campo),
em vez do relatório da Linha + Documento.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jhm2rrJCBVkJYZMmi4pDeT
</commit_message>
<xml_diff>
--- a/saida/Situacao_Geral_de_Spools_ATUALIZADO.xlsx
+++ b/saida/Situacao_Geral_de_Spools_ATUALIZADO.xlsx
@@ -12124,11 +12124,7 @@
         <v>46261</v>
       </c>
       <c r="AM73" s="34"/>
-      <c r="AN73" s="7" t="inlineStr">
-        <is>
-          <t>066/26</t>
-        </is>
-      </c>
+      <c r="AN73" s="7"/>
       <c r="AO73" s="7"/>
       <c r="AP73" s="34">
         <v>46266</v>
@@ -12386,7 +12382,11 @@
       <c r="AK75" s="34"/>
       <c r="AL75" s="34"/>
       <c r="AM75" s="34"/>
-      <c r="AN75" s="7"/>
+      <c r="AN75" s="7" t="inlineStr">
+        <is>
+          <t>066/26</t>
+        </is>
+      </c>
       <c r="AO75" s="7"/>
       <c r="AP75" s="34"/>
       <c r="AQ75" s="7"/>
@@ -12650,11 +12650,7 @@
         <v>46262</v>
       </c>
       <c r="AM77" s="34"/>
-      <c r="AN77" s="7" t="inlineStr">
-        <is>
-          <t>067/26</t>
-        </is>
-      </c>
+      <c r="AN77" s="7"/>
       <c r="AO77" s="7"/>
       <c r="AP77" s="34">
         <v>46266</v>
@@ -27578,11 +27574,7 @@
         <v>46261</v>
       </c>
       <c r="AM193" s="34"/>
-      <c r="AN193" s="7" t="inlineStr">
-        <is>
-          <t>047/26</t>
-        </is>
-      </c>
+      <c r="AN193" s="7"/>
       <c r="AO193" s="7"/>
       <c r="AP193" s="34">
         <v>46266</v>
@@ -27977,11 +27969,7 @@
         <v>46261</v>
       </c>
       <c r="AM196" s="34"/>
-      <c r="AN196" s="7" t="inlineStr">
-        <is>
-          <t>048/26</t>
-        </is>
-      </c>
+      <c r="AN196" s="7"/>
       <c r="AO196" s="7"/>
       <c r="AP196" s="34">
         <v>46266</v>

</xml_diff>

<commit_message>
Atualiza Mapa de Spools com a nova base do Mapa de Juntas
- Substitui o Mapa de Juntas v2 pela versão recebida e regenera o Mapa
  de Spools atualizado e o relatório (15 spools a mais concluídos nas
  etapas de fabricação, 14 no END).
- Juntas com P/C desconhecido (ex.: PENDT) passam a ser avisadas em uma
  única linha agrupada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jhm2rrJCBVkJYZMmi4pDeT
</commit_message>
<xml_diff>
--- a/saida/Situacao_Geral_de_Spools_ATUALIZADO.xlsx
+++ b/saida/Situacao_Geral_de_Spools_ATUALIZADO.xlsx
@@ -5193,19 +5193,29 @@
         <v>6</v>
       </c>
       <c r="AE20" s="36">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AF20" s="34"/>
       <c r="AG20" s="7"/>
       <c r="AH20" s="34"/>
-      <c r="AI20" s="34"/>
-      <c r="AJ20" s="34"/>
-      <c r="AK20" s="34"/>
-      <c r="AL20" s="34"/>
+      <c r="AI20" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AJ20" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AK20" s="34">
+        <v>46288</v>
+      </c>
+      <c r="AL20" s="34">
+        <v>46288</v>
+      </c>
       <c r="AM20" s="34"/>
       <c r="AN20" s="7"/>
       <c r="AO20" s="7"/>
-      <c r="AP20" s="34"/>
+      <c r="AP20" s="34">
+        <v>46288</v>
+      </c>
       <c r="AQ20" s="7"/>
       <c r="AR20" s="34"/>
       <c r="AS20" s="34"/>
@@ -6100,15 +6110,23 @@
         <v>5</v>
       </c>
       <c r="AE27" s="36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AF27" s="34"/>
       <c r="AG27" s="7"/>
       <c r="AH27" s="34"/>
-      <c r="AI27" s="34"/>
-      <c r="AJ27" s="34"/>
-      <c r="AK27" s="34"/>
-      <c r="AL27" s="34"/>
+      <c r="AI27" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AJ27" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AK27" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AL27" s="34">
+        <v>46286</v>
+      </c>
       <c r="AM27" s="34"/>
       <c r="AN27" s="7" t="inlineStr">
         <is>
@@ -6116,7 +6134,9 @@
         </is>
       </c>
       <c r="AO27" s="7"/>
-      <c r="AP27" s="34"/>
+      <c r="AP27" s="34">
+        <v>46288</v>
+      </c>
       <c r="AQ27" s="7"/>
       <c r="AR27" s="34"/>
       <c r="AS27" s="34"/>
@@ -7394,7 +7414,9 @@
       <c r="AM37" s="34"/>
       <c r="AN37" s="7"/>
       <c r="AO37" s="7"/>
-      <c r="AP37" s="34"/>
+      <c r="AP37" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ37" s="7"/>
       <c r="AR37" s="34"/>
       <c r="AS37" s="34"/>
@@ -7523,7 +7545,9 @@
       <c r="AM38" s="34"/>
       <c r="AN38" s="7"/>
       <c r="AO38" s="7"/>
-      <c r="AP38" s="34"/>
+      <c r="AP38" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ38" s="7"/>
       <c r="AR38" s="34"/>
       <c r="AS38" s="34"/>
@@ -7632,7 +7656,7 @@
         <v>4</v>
       </c>
       <c r="AE39" s="36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AF39" s="34"/>
       <c r="AG39" s="7"/>
@@ -7652,7 +7676,9 @@
       <c r="AM39" s="34"/>
       <c r="AN39" s="7"/>
       <c r="AO39" s="7"/>
-      <c r="AP39" s="34"/>
+      <c r="AP39" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ39" s="7"/>
       <c r="AR39" s="34"/>
       <c r="AS39" s="34"/>
@@ -8440,7 +8466,9 @@
         </is>
       </c>
       <c r="AO45" s="7"/>
-      <c r="AP45" s="34"/>
+      <c r="AP45" s="34">
+        <v>46267</v>
+      </c>
       <c r="AQ45" s="7"/>
       <c r="AR45" s="34"/>
       <c r="AS45" s="34"/>
@@ -10290,7 +10318,9 @@
       <c r="AM59" s="34"/>
       <c r="AN59" s="7"/>
       <c r="AO59" s="7"/>
-      <c r="AP59" s="34"/>
+      <c r="AP59" s="34">
+        <v>46278</v>
+      </c>
       <c r="AQ59" s="7"/>
       <c r="AR59" s="34"/>
       <c r="AS59" s="34"/>
@@ -13168,7 +13198,7 @@
         <v>5</v>
       </c>
       <c r="AE81" s="36">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AF81" s="34"/>
       <c r="AG81" s="7"/>
@@ -13289,7 +13319,7 @@
         <v>4</v>
       </c>
       <c r="AE82" s="36">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AF82" s="34"/>
       <c r="AG82" s="7"/>
@@ -13410,7 +13440,7 @@
         <v>12</v>
       </c>
       <c r="AE83" s="36">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AF83" s="34"/>
       <c r="AG83" s="7"/>
@@ -13531,7 +13561,7 @@
         <v>11</v>
       </c>
       <c r="AE84" s="36">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AF84" s="34"/>
       <c r="AG84" s="7"/>
@@ -13652,7 +13682,7 @@
         <v>4</v>
       </c>
       <c r="AE85" s="36">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AF85" s="34"/>
       <c r="AG85" s="7"/>
@@ -13773,7 +13803,7 @@
         <v>4</v>
       </c>
       <c r="AE86" s="36">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AF86" s="34"/>
       <c r="AG86" s="7"/>
@@ -16121,15 +16151,23 @@
         <v>2</v>
       </c>
       <c r="AE104" s="36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AF104" s="34"/>
       <c r="AG104" s="7"/>
       <c r="AH104" s="34"/>
-      <c r="AI104" s="34"/>
-      <c r="AJ104" s="34"/>
-      <c r="AK104" s="34"/>
-      <c r="AL104" s="34"/>
+      <c r="AI104" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AJ104" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AK104" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AL104" s="34">
+        <v>46286</v>
+      </c>
       <c r="AM104" s="34"/>
       <c r="AN104" s="7" t="inlineStr">
         <is>
@@ -16637,15 +16675,23 @@
         <v>2</v>
       </c>
       <c r="AE108" s="36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AF108" s="34"/>
       <c r="AG108" s="7"/>
       <c r="AH108" s="34"/>
-      <c r="AI108" s="34"/>
-      <c r="AJ108" s="34"/>
-      <c r="AK108" s="34"/>
-      <c r="AL108" s="34"/>
+      <c r="AI108" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AJ108" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AK108" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AL108" s="34">
+        <v>46285</v>
+      </c>
       <c r="AM108" s="34"/>
       <c r="AN108" s="7" t="inlineStr">
         <is>
@@ -17153,15 +17199,23 @@
         <v>2</v>
       </c>
       <c r="AE112" s="36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AF112" s="34"/>
       <c r="AG112" s="7"/>
       <c r="AH112" s="34"/>
-      <c r="AI112" s="34"/>
-      <c r="AJ112" s="34"/>
-      <c r="AK112" s="34"/>
-      <c r="AL112" s="34"/>
+      <c r="AI112" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AJ112" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AK112" s="34">
+        <v>46285</v>
+      </c>
+      <c r="AL112" s="34">
+        <v>46285</v>
+      </c>
       <c r="AM112" s="34"/>
       <c r="AN112" s="7" t="inlineStr">
         <is>
@@ -17407,15 +17461,23 @@
         <v>6</v>
       </c>
       <c r="AE114" s="36">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AF114" s="34"/>
       <c r="AG114" s="7"/>
       <c r="AH114" s="34"/>
-      <c r="AI114" s="34"/>
-      <c r="AJ114" s="34"/>
-      <c r="AK114" s="34"/>
-      <c r="AL114" s="34"/>
+      <c r="AI114" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AJ114" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AK114" s="34">
+        <v>46286</v>
+      </c>
+      <c r="AL114" s="34">
+        <v>46286</v>
+      </c>
       <c r="AM114" s="34"/>
       <c r="AN114" s="7" t="inlineStr">
         <is>
@@ -17663,19 +17725,29 @@
         <v>4</v>
       </c>
       <c r="AE116" s="36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AF116" s="34"/>
       <c r="AG116" s="7"/>
       <c r="AH116" s="34"/>
-      <c r="AI116" s="34"/>
-      <c r="AJ116" s="34"/>
-      <c r="AK116" s="34"/>
-      <c r="AL116" s="34"/>
+      <c r="AI116" s="34">
+        <v>46252</v>
+      </c>
+      <c r="AJ116" s="34">
+        <v>46252</v>
+      </c>
+      <c r="AK116" s="34">
+        <v>46252</v>
+      </c>
+      <c r="AL116" s="34">
+        <v>46252</v>
+      </c>
       <c r="AM116" s="34"/>
       <c r="AN116" s="7"/>
       <c r="AO116" s="7"/>
-      <c r="AP116" s="34"/>
+      <c r="AP116" s="34">
+        <v>46252</v>
+      </c>
       <c r="AQ116" s="7"/>
       <c r="AR116" s="34"/>
       <c r="AS116" s="34"/>
@@ -18292,15 +18364,23 @@
         <v>5</v>
       </c>
       <c r="AE121" s="36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AF121" s="34"/>
       <c r="AG121" s="7"/>
       <c r="AH121" s="34"/>
-      <c r="AI121" s="34"/>
-      <c r="AJ121" s="34"/>
-      <c r="AK121" s="34"/>
-      <c r="AL121" s="34"/>
+      <c r="AI121" s="34">
+        <v>46254</v>
+      </c>
+      <c r="AJ121" s="34">
+        <v>46254</v>
+      </c>
+      <c r="AK121" s="34">
+        <v>46254</v>
+      </c>
+      <c r="AL121" s="34">
+        <v>46254</v>
+      </c>
       <c r="AM121" s="34"/>
       <c r="AN121" s="7" t="inlineStr">
         <is>
@@ -18308,7 +18388,9 @@
         </is>
       </c>
       <c r="AO121" s="7"/>
-      <c r="AP121" s="34"/>
+      <c r="AP121" s="34">
+        <v>46255</v>
+      </c>
       <c r="AQ121" s="7"/>
       <c r="AR121" s="34"/>
       <c r="AS121" s="34"/>
@@ -18415,15 +18497,23 @@
         <v>9</v>
       </c>
       <c r="AE122" s="36">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AF122" s="34"/>
       <c r="AG122" s="7"/>
       <c r="AH122" s="34"/>
-      <c r="AI122" s="34"/>
-      <c r="AJ122" s="34"/>
-      <c r="AK122" s="34"/>
-      <c r="AL122" s="34"/>
+      <c r="AI122" s="34">
+        <v>46255</v>
+      </c>
+      <c r="AJ122" s="34">
+        <v>46255</v>
+      </c>
+      <c r="AK122" s="34">
+        <v>46255</v>
+      </c>
+      <c r="AL122" s="34">
+        <v>46255</v>
+      </c>
       <c r="AM122" s="34"/>
       <c r="AN122" s="7" t="inlineStr">
         <is>
@@ -18431,7 +18521,9 @@
         </is>
       </c>
       <c r="AO122" s="7"/>
-      <c r="AP122" s="34"/>
+      <c r="AP122" s="34">
+        <v>46258</v>
+      </c>
       <c r="AQ122" s="7"/>
       <c r="AR122" s="34"/>
       <c r="AS122" s="34"/>
@@ -21416,7 +21508,7 @@
         <v>9</v>
       </c>
       <c r="AE145" s="36">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AF145" s="34"/>
       <c r="AG145" s="7"/>
@@ -24984,15 +25076,23 @@
         <v>3</v>
       </c>
       <c r="AE173" s="36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AF173" s="34"/>
       <c r="AG173" s="7"/>
       <c r="AH173" s="34"/>
-      <c r="AI173" s="34"/>
-      <c r="AJ173" s="34"/>
-      <c r="AK173" s="34"/>
-      <c r="AL173" s="34"/>
+      <c r="AI173" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AJ173" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AK173" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AL173" s="34">
+        <v>46287</v>
+      </c>
       <c r="AM173" s="34"/>
       <c r="AN173" s="7" t="inlineStr">
         <is>
@@ -25107,15 +25207,23 @@
         <v>5</v>
       </c>
       <c r="AE174" s="36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AF174" s="34"/>
       <c r="AG174" s="7"/>
       <c r="AH174" s="34"/>
-      <c r="AI174" s="34"/>
-      <c r="AJ174" s="34"/>
-      <c r="AK174" s="34"/>
-      <c r="AL174" s="34"/>
+      <c r="AI174" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AJ174" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AK174" s="34">
+        <v>46287</v>
+      </c>
+      <c r="AL174" s="34">
+        <v>46287</v>
+      </c>
       <c r="AM174" s="34"/>
       <c r="AN174" s="7" t="inlineStr">
         <is>
@@ -28233,7 +28341,9 @@
       <c r="AM198" s="34"/>
       <c r="AN198" s="7"/>
       <c r="AO198" s="7"/>
-      <c r="AP198" s="34"/>
+      <c r="AP198" s="34">
+        <v>46279</v>
+      </c>
       <c r="AQ198" s="7"/>
       <c r="AR198" s="34"/>
       <c r="AS198" s="34"/>
@@ -29372,19 +29482,29 @@
         <v>4</v>
       </c>
       <c r="AE207" s="36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AF207" s="34"/>
       <c r="AG207" s="7"/>
       <c r="AH207" s="34"/>
-      <c r="AI207" s="34"/>
-      <c r="AJ207" s="34"/>
-      <c r="AK207" s="34"/>
-      <c r="AL207" s="34"/>
+      <c r="AI207" s="34">
+        <v>46255</v>
+      </c>
+      <c r="AJ207" s="34">
+        <v>46255</v>
+      </c>
+      <c r="AK207" s="34">
+        <v>46255</v>
+      </c>
+      <c r="AL207" s="34">
+        <v>46255</v>
+      </c>
       <c r="AM207" s="34"/>
       <c r="AN207" s="7"/>
       <c r="AO207" s="7"/>
-      <c r="AP207" s="34"/>
+      <c r="AP207" s="34">
+        <v>46256</v>
+      </c>
       <c r="AQ207" s="7"/>
       <c r="AR207" s="34"/>
       <c r="AS207" s="34"/>
@@ -33463,14 +33583,24 @@
       <c r="AF239" s="34"/>
       <c r="AG239" s="7"/>
       <c r="AH239" s="34"/>
-      <c r="AI239" s="34"/>
-      <c r="AJ239" s="34"/>
-      <c r="AK239" s="34"/>
-      <c r="AL239" s="34"/>
+      <c r="AI239" s="34">
+        <v>46261</v>
+      </c>
+      <c r="AJ239" s="34">
+        <v>46261</v>
+      </c>
+      <c r="AK239" s="34">
+        <v>46261</v>
+      </c>
+      <c r="AL239" s="34">
+        <v>46261</v>
+      </c>
       <c r="AM239" s="34"/>
       <c r="AN239" s="7"/>
       <c r="AO239" s="7"/>
-      <c r="AP239" s="34"/>
+      <c r="AP239" s="34">
+        <v>46266</v>
+      </c>
       <c r="AQ239" s="7"/>
       <c r="AR239" s="34"/>
       <c r="AS239" s="34"/>
@@ -33844,10 +33974,18 @@
       <c r="AF242" s="34"/>
       <c r="AG242" s="7"/>
       <c r="AH242" s="34"/>
-      <c r="AI242" s="34"/>
-      <c r="AJ242" s="34"/>
-      <c r="AK242" s="34"/>
-      <c r="AL242" s="34"/>
+      <c r="AI242" s="34">
+        <v>46272</v>
+      </c>
+      <c r="AJ242" s="34">
+        <v>46272</v>
+      </c>
+      <c r="AK242" s="34">
+        <v>46272</v>
+      </c>
+      <c r="AL242" s="34">
+        <v>46272</v>
+      </c>
       <c r="AM242" s="34"/>
       <c r="AN242" s="7"/>
       <c r="AO242" s="7"/>
@@ -34090,14 +34228,24 @@
       <c r="AF244" s="34"/>
       <c r="AG244" s="7"/>
       <c r="AH244" s="34"/>
-      <c r="AI244" s="34"/>
-      <c r="AJ244" s="34"/>
-      <c r="AK244" s="34"/>
-      <c r="AL244" s="34"/>
+      <c r="AI244" s="34">
+        <v>46279</v>
+      </c>
+      <c r="AJ244" s="34">
+        <v>46279</v>
+      </c>
+      <c r="AK244" s="34">
+        <v>46279</v>
+      </c>
+      <c r="AL244" s="34">
+        <v>46279</v>
+      </c>
       <c r="AM244" s="34"/>
       <c r="AN244" s="7"/>
       <c r="AO244" s="7"/>
-      <c r="AP244" s="34"/>
+      <c r="AP244" s="34">
+        <v>46280</v>
+      </c>
       <c r="AQ244" s="7"/>
       <c r="AR244" s="34"/>
       <c r="AS244" s="34"/>

</xml_diff>

<commit_message>
Atualiza Mapa de Spools com a base do Mapa de Juntas de 07/10 21:29
Na nova base as 32 juntas com P/C "PENDT" passaram a "P"; os spools
dessas juntas (10"-B3B-LO-5103B-2 e 10"-B3B-MR-5201B-2) têm o
Total_Juntas_Pipe corrigido. Demais campos sem alteração.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jhm2rrJCBVkJYZMmi4pDeT
</commit_message>
<xml_diff>
--- a/saida/Situacao_Geral_de_Spools_ATUALIZADO.xlsx
+++ b/saida/Situacao_Geral_de_Spools_ATUALIZADO.xlsx
@@ -13198,7 +13198,7 @@
         <v>5</v>
       </c>
       <c r="AE81" s="36">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AF81" s="34"/>
       <c r="AG81" s="7"/>
@@ -13319,7 +13319,7 @@
         <v>4</v>
       </c>
       <c r="AE82" s="36">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AF82" s="34"/>
       <c r="AG82" s="7"/>
@@ -13440,7 +13440,7 @@
         <v>12</v>
       </c>
       <c r="AE83" s="36">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AF83" s="34"/>
       <c r="AG83" s="7"/>
@@ -13561,7 +13561,7 @@
         <v>11</v>
       </c>
       <c r="AE84" s="36">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AF84" s="34"/>
       <c r="AG84" s="7"/>
@@ -13682,7 +13682,7 @@
         <v>4</v>
       </c>
       <c r="AE85" s="36">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF85" s="34"/>
       <c r="AG85" s="7"/>
@@ -13803,7 +13803,7 @@
         <v>4</v>
       </c>
       <c r="AE86" s="36">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AF86" s="34"/>
       <c r="AG86" s="7"/>

</xml_diff>